<commit_message>
fix modificacion de scripts
</commit_message>
<xml_diff>
--- a/Guias Produccion/HU-55188.xlsx
+++ b/Guias Produccion/HU-55188.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Alliance\ScriptsEntidades\Guias Produccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78BA7D31-FE1C-4305-871D-3A9090432D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E704160-5019-4291-B3DE-FFE182156D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -564,9 +564,6 @@
     <t>18-AlterOrdenesLocales.sql</t>
   </si>
   <si>
-    <t>19-AlterTableGuias.sql</t>
-  </si>
-  <si>
     <t>20-AlterAsignacionServiciosLocales.sql</t>
   </si>
   <si>
@@ -639,13 +636,16 @@
     <t>43-InsertDictionaryParametrosLista.sql</t>
   </si>
   <si>
-    <t>45-AddIndexes_GuiasHouse_BilltoConsigneeId.sql</t>
-  </si>
-  <si>
     <t>44-AddIndexes_Entities.sql</t>
   </si>
   <si>
-    <t>46-AddIndexes_GuiasHouseDetalles_idGuiaHouseShipToId.sql</t>
+    <t>19-AlterGuias.sql</t>
+  </si>
+  <si>
+    <t>45-AddIndexes_GuiasHouse.sql</t>
+  </si>
+  <si>
+    <t>46-AddIndexes_GuiasHouseDetalles.sql</t>
   </si>
 </sst>
 </file>
@@ -1877,51 +1877,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="45" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="46" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="48" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1972,6 +1927,51 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="45" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="46" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="48" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -11681,44 +11681,44 @@
   <sheetData>
     <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:16" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="80" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
-      <c r="L3" s="96"/>
-      <c r="M3" s="96"/>
-      <c r="O3" s="91" t="s">
+      <c r="B3" s="81"/>
+      <c r="C3" s="81"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="81"/>
+      <c r="M3" s="81"/>
+      <c r="O3" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="P3" s="92"/>
+      <c r="P3" s="77"/>
     </row>
     <row r="4" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="100" t="s">
+      <c r="B4" s="85" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="101"/>
-      <c r="D4" s="101"/>
-      <c r="E4" s="101"/>
-      <c r="F4" s="101"/>
-      <c r="G4" s="101"/>
-      <c r="H4" s="101"/>
-      <c r="I4" s="101"/>
-      <c r="J4" s="102"/>
-      <c r="K4" s="102"/>
-      <c r="L4" s="102"/>
-      <c r="M4" s="102"/>
+      <c r="C4" s="86"/>
+      <c r="D4" s="86"/>
+      <c r="E4" s="86"/>
+      <c r="F4" s="86"/>
+      <c r="G4" s="86"/>
+      <c r="H4" s="86"/>
+      <c r="I4" s="86"/>
+      <c r="J4" s="87"/>
+      <c r="K4" s="87"/>
+      <c r="L4" s="87"/>
+      <c r="M4" s="87"/>
       <c r="O4" s="20" t="s">
         <v>2</v>
       </c>
@@ -11728,20 +11728,20 @@
       <c r="A5" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="103" t="s">
+      <c r="B5" s="88" t="s">
         <v>113</v>
       </c>
-      <c r="C5" s="103"/>
-      <c r="D5" s="103"/>
-      <c r="E5" s="103"/>
-      <c r="F5" s="103"/>
-      <c r="G5" s="103"/>
-      <c r="H5" s="103"/>
-      <c r="I5" s="103"/>
-      <c r="J5" s="104"/>
-      <c r="K5" s="104"/>
-      <c r="L5" s="104"/>
-      <c r="M5" s="104"/>
+      <c r="C5" s="88"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="88"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
+      <c r="K5" s="89"/>
+      <c r="L5" s="89"/>
+      <c r="M5" s="89"/>
       <c r="O5" s="14" t="s">
         <v>4</v>
       </c>
@@ -11751,20 +11751,20 @@
       <c r="A6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="93">
+      <c r="B6" s="78">
         <v>45974</v>
       </c>
-      <c r="C6" s="94"/>
-      <c r="D6" s="94"/>
-      <c r="E6" s="94"/>
-      <c r="F6" s="94"/>
-      <c r="G6" s="94"/>
-      <c r="H6" s="94"/>
-      <c r="I6" s="94"/>
-      <c r="J6" s="94"/>
-      <c r="K6" s="94"/>
-      <c r="L6" s="94"/>
-      <c r="M6" s="94"/>
+      <c r="C6" s="79"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
+      <c r="I6" s="79"/>
+      <c r="J6" s="79"/>
+      <c r="K6" s="79"/>
+      <c r="L6" s="79"/>
+      <c r="M6" s="79"/>
       <c r="O6" s="13"/>
       <c r="P6" s="13"/>
     </row>
@@ -11772,18 +11772,18 @@
       <c r="A7" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="105"/>
-      <c r="C7" s="106"/>
-      <c r="D7" s="106"/>
-      <c r="E7" s="106"/>
-      <c r="F7" s="106"/>
-      <c r="G7" s="106"/>
-      <c r="H7" s="106"/>
-      <c r="I7" s="106"/>
-      <c r="J7" s="107"/>
-      <c r="K7" s="107"/>
-      <c r="L7" s="107"/>
-      <c r="M7" s="107"/>
+      <c r="B7" s="90"/>
+      <c r="C7" s="91"/>
+      <c r="D7" s="91"/>
+      <c r="E7" s="91"/>
+      <c r="F7" s="91"/>
+      <c r="G7" s="91"/>
+      <c r="H7" s="91"/>
+      <c r="I7" s="91"/>
+      <c r="J7" s="92"/>
+      <c r="K7" s="92"/>
+      <c r="L7" s="92"/>
+      <c r="M7" s="92"/>
     </row>
     <row r="8" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11"/>
@@ -11801,21 +11801,21 @@
       <c r="M8" s="12"/>
     </row>
     <row r="9" spans="1:16" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="97" t="s">
+      <c r="A9" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="98"/>
-      <c r="C9" s="98"/>
-      <c r="D9" s="98"/>
-      <c r="E9" s="98"/>
-      <c r="F9" s="98"/>
-      <c r="G9" s="98"/>
-      <c r="H9" s="98"/>
-      <c r="I9" s="98"/>
-      <c r="J9" s="99"/>
-      <c r="K9" s="99"/>
-      <c r="L9" s="99"/>
-      <c r="M9" s="99"/>
+      <c r="B9" s="83"/>
+      <c r="C9" s="83"/>
+      <c r="D9" s="83"/>
+      <c r="E9" s="83"/>
+      <c r="F9" s="83"/>
+      <c r="G9" s="83"/>
+      <c r="H9" s="83"/>
+      <c r="I9" s="83"/>
+      <c r="J9" s="84"/>
+      <c r="K9" s="84"/>
+      <c r="L9" s="84"/>
+      <c r="M9" s="84"/>
     </row>
     <row r="10" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -11916,67 +11916,67 @@
       <c r="A14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="89"/>
-      <c r="C14" s="90"/>
-      <c r="D14" s="90"/>
-      <c r="E14" s="90"/>
-      <c r="F14" s="90"/>
-      <c r="G14" s="90"/>
-      <c r="H14" s="90"/>
-      <c r="I14" s="90"/>
-      <c r="J14" s="90"/>
-      <c r="K14" s="90"/>
-      <c r="L14" s="90"/>
-      <c r="M14" s="90"/>
+      <c r="B14" s="106"/>
+      <c r="C14" s="107"/>
+      <c r="D14" s="107"/>
+      <c r="E14" s="107"/>
+      <c r="F14" s="107"/>
+      <c r="G14" s="107"/>
+      <c r="H14" s="107"/>
+      <c r="I14" s="107"/>
+      <c r="J14" s="107"/>
+      <c r="K14" s="107"/>
+      <c r="L14" s="107"/>
+      <c r="M14" s="107"/>
     </row>
     <row r="15" spans="1:16" s="75" customFormat="1" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="89"/>
-      <c r="C15" s="90"/>
-      <c r="D15" s="90"/>
-      <c r="E15" s="90"/>
-      <c r="F15" s="90"/>
-      <c r="G15" s="90"/>
-      <c r="H15" s="90"/>
-      <c r="I15" s="90"/>
-      <c r="J15" s="90"/>
-      <c r="K15" s="90"/>
-      <c r="L15" s="90"/>
-      <c r="M15" s="90"/>
+      <c r="B15" s="106"/>
+      <c r="C15" s="107"/>
+      <c r="D15" s="107"/>
+      <c r="E15" s="107"/>
+      <c r="F15" s="107"/>
+      <c r="G15" s="107"/>
+      <c r="H15" s="107"/>
+      <c r="I15" s="107"/>
+      <c r="J15" s="107"/>
+      <c r="K15" s="107"/>
+      <c r="L15" s="107"/>
+      <c r="M15" s="107"/>
     </row>
     <row r="16" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="80"/>
-      <c r="B16" s="81"/>
-      <c r="C16" s="81"/>
-      <c r="D16" s="81"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="81"/>
-      <c r="G16" s="81"/>
-      <c r="H16" s="81"/>
-      <c r="I16" s="81"/>
-      <c r="J16" s="81"/>
-      <c r="K16" s="81"/>
-      <c r="L16" s="81"/>
-      <c r="M16" s="81"/>
+      <c r="A16" s="97"/>
+      <c r="B16" s="98"/>
+      <c r="C16" s="98"/>
+      <c r="D16" s="98"/>
+      <c r="E16" s="98"/>
+      <c r="F16" s="98"/>
+      <c r="G16" s="98"/>
+      <c r="H16" s="98"/>
+      <c r="I16" s="98"/>
+      <c r="J16" s="98"/>
+      <c r="K16" s="98"/>
+      <c r="L16" s="98"/>
+      <c r="M16" s="98"/>
     </row>
     <row r="17" spans="1:13" s="5" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="82" t="s">
+      <c r="A17" s="99" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="83"/>
-      <c r="C17" s="83"/>
-      <c r="D17" s="83"/>
-      <c r="E17" s="83"/>
-      <c r="F17" s="83"/>
-      <c r="G17" s="83"/>
-      <c r="H17" s="83"/>
-      <c r="I17" s="83"/>
-      <c r="J17" s="84"/>
-      <c r="K17" s="84"/>
-      <c r="L17" s="84"/>
-      <c r="M17" s="84"/>
+      <c r="B17" s="100"/>
+      <c r="C17" s="100"/>
+      <c r="D17" s="100"/>
+      <c r="E17" s="100"/>
+      <c r="F17" s="100"/>
+      <c r="G17" s="100"/>
+      <c r="H17" s="100"/>
+      <c r="I17" s="100"/>
+      <c r="J17" s="101"/>
+      <c r="K17" s="101"/>
+      <c r="L17" s="101"/>
+      <c r="M17" s="101"/>
     </row>
     <row r="18" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
@@ -12048,17 +12048,17 @@
       <c r="D21" s="120" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="76" t="s">
+      <c r="E21" s="93" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="77"/>
-      <c r="G21" s="77"/>
-      <c r="H21" s="77"/>
-      <c r="I21" s="77"/>
-      <c r="J21" s="77"/>
-      <c r="K21" s="77"/>
-      <c r="L21" s="77"/>
-      <c r="M21" s="77"/>
+      <c r="F21" s="94"/>
+      <c r="G21" s="94"/>
+      <c r="H21" s="94"/>
+      <c r="I21" s="94"/>
+      <c r="J21" s="94"/>
+      <c r="K21" s="94"/>
+      <c r="L21" s="94"/>
+      <c r="M21" s="94"/>
     </row>
     <row r="22" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
@@ -12069,15 +12069,15 @@
         <v>103</v>
       </c>
       <c r="D22" s="121"/>
-      <c r="E22" s="78"/>
-      <c r="F22" s="79"/>
-      <c r="G22" s="79"/>
-      <c r="H22" s="79"/>
-      <c r="I22" s="79"/>
-      <c r="J22" s="79"/>
-      <c r="K22" s="79"/>
-      <c r="L22" s="79"/>
-      <c r="M22" s="79"/>
+      <c r="E22" s="95"/>
+      <c r="F22" s="96"/>
+      <c r="G22" s="96"/>
+      <c r="H22" s="96"/>
+      <c r="I22" s="96"/>
+      <c r="J22" s="96"/>
+      <c r="K22" s="96"/>
+      <c r="L22" s="96"/>
+      <c r="M22" s="96"/>
     </row>
     <row r="23" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="115"/>
@@ -12142,18 +12142,18 @@
         <v>115</v>
       </c>
       <c r="C26" s="33"/>
-      <c r="D26" s="85" t="s">
+      <c r="D26" s="102" t="s">
         <v>111</v>
       </c>
-      <c r="E26" s="86"/>
-      <c r="F26" s="86"/>
-      <c r="G26" s="86"/>
-      <c r="H26" s="86"/>
-      <c r="I26" s="86"/>
-      <c r="J26" s="86"/>
-      <c r="K26" s="86"/>
-      <c r="L26" s="86"/>
-      <c r="M26" s="86"/>
+      <c r="E26" s="103"/>
+      <c r="F26" s="103"/>
+      <c r="G26" s="103"/>
+      <c r="H26" s="103"/>
+      <c r="I26" s="103"/>
+      <c r="J26" s="103"/>
+      <c r="K26" s="103"/>
+      <c r="L26" s="103"/>
+      <c r="M26" s="103"/>
     </row>
     <row r="27" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="32">
@@ -12163,16 +12163,16 @@
         <v>116</v>
       </c>
       <c r="C27" s="33"/>
-      <c r="D27" s="87"/>
-      <c r="E27" s="88"/>
-      <c r="F27" s="88"/>
-      <c r="G27" s="88"/>
-      <c r="H27" s="88"/>
-      <c r="I27" s="88"/>
-      <c r="J27" s="88"/>
-      <c r="K27" s="88"/>
-      <c r="L27" s="88"/>
-      <c r="M27" s="88"/>
+      <c r="D27" s="104"/>
+      <c r="E27" s="105"/>
+      <c r="F27" s="105"/>
+      <c r="G27" s="105"/>
+      <c r="H27" s="105"/>
+      <c r="I27" s="105"/>
+      <c r="J27" s="105"/>
+      <c r="K27" s="105"/>
+      <c r="L27" s="105"/>
+      <c r="M27" s="105"/>
     </row>
     <row r="28" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="32">
@@ -12182,16 +12182,16 @@
         <v>117</v>
       </c>
       <c r="C28" s="33"/>
-      <c r="D28" s="87"/>
-      <c r="E28" s="88"/>
-      <c r="F28" s="88"/>
-      <c r="G28" s="88"/>
-      <c r="H28" s="88"/>
-      <c r="I28" s="88"/>
-      <c r="J28" s="88"/>
-      <c r="K28" s="88"/>
-      <c r="L28" s="88"/>
-      <c r="M28" s="88"/>
+      <c r="D28" s="104"/>
+      <c r="E28" s="105"/>
+      <c r="F28" s="105"/>
+      <c r="G28" s="105"/>
+      <c r="H28" s="105"/>
+      <c r="I28" s="105"/>
+      <c r="J28" s="105"/>
+      <c r="K28" s="105"/>
+      <c r="L28" s="105"/>
+      <c r="M28" s="105"/>
     </row>
     <row r="29" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="32">
@@ -12201,16 +12201,16 @@
         <v>118</v>
       </c>
       <c r="C29" s="33"/>
-      <c r="D29" s="87"/>
-      <c r="E29" s="88"/>
-      <c r="F29" s="88"/>
-      <c r="G29" s="88"/>
-      <c r="H29" s="88"/>
-      <c r="I29" s="88"/>
-      <c r="J29" s="88"/>
-      <c r="K29" s="88"/>
-      <c r="L29" s="88"/>
-      <c r="M29" s="88"/>
+      <c r="D29" s="104"/>
+      <c r="E29" s="105"/>
+      <c r="F29" s="105"/>
+      <c r="G29" s="105"/>
+      <c r="H29" s="105"/>
+      <c r="I29" s="105"/>
+      <c r="J29" s="105"/>
+      <c r="K29" s="105"/>
+      <c r="L29" s="105"/>
+      <c r="M29" s="105"/>
     </row>
     <row r="30" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="32">
@@ -12220,16 +12220,16 @@
         <v>119</v>
       </c>
       <c r="C30" s="33"/>
-      <c r="D30" s="87"/>
-      <c r="E30" s="88"/>
-      <c r="F30" s="88"/>
-      <c r="G30" s="88"/>
-      <c r="H30" s="88"/>
-      <c r="I30" s="88"/>
-      <c r="J30" s="88"/>
-      <c r="K30" s="88"/>
-      <c r="L30" s="88"/>
-      <c r="M30" s="88"/>
+      <c r="D30" s="104"/>
+      <c r="E30" s="105"/>
+      <c r="F30" s="105"/>
+      <c r="G30" s="105"/>
+      <c r="H30" s="105"/>
+      <c r="I30" s="105"/>
+      <c r="J30" s="105"/>
+      <c r="K30" s="105"/>
+      <c r="L30" s="105"/>
+      <c r="M30" s="105"/>
     </row>
     <row r="31" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="32">
@@ -12239,16 +12239,16 @@
         <v>120</v>
       </c>
       <c r="C31" s="33"/>
-      <c r="D31" s="87"/>
-      <c r="E31" s="88"/>
-      <c r="F31" s="88"/>
-      <c r="G31" s="88"/>
-      <c r="H31" s="88"/>
-      <c r="I31" s="88"/>
-      <c r="J31" s="88"/>
-      <c r="K31" s="88"/>
-      <c r="L31" s="88"/>
-      <c r="M31" s="88"/>
+      <c r="D31" s="104"/>
+      <c r="E31" s="105"/>
+      <c r="F31" s="105"/>
+      <c r="G31" s="105"/>
+      <c r="H31" s="105"/>
+      <c r="I31" s="105"/>
+      <c r="J31" s="105"/>
+      <c r="K31" s="105"/>
+      <c r="L31" s="105"/>
+      <c r="M31" s="105"/>
     </row>
     <row r="32" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="32">
@@ -12258,16 +12258,16 @@
         <v>121</v>
       </c>
       <c r="C32" s="33"/>
-      <c r="D32" s="87"/>
-      <c r="E32" s="88"/>
-      <c r="F32" s="88"/>
-      <c r="G32" s="88"/>
-      <c r="H32" s="88"/>
-      <c r="I32" s="88"/>
-      <c r="J32" s="88"/>
-      <c r="K32" s="88"/>
-      <c r="L32" s="88"/>
-      <c r="M32" s="88"/>
+      <c r="D32" s="104"/>
+      <c r="E32" s="105"/>
+      <c r="F32" s="105"/>
+      <c r="G32" s="105"/>
+      <c r="H32" s="105"/>
+      <c r="I32" s="105"/>
+      <c r="J32" s="105"/>
+      <c r="K32" s="105"/>
+      <c r="L32" s="105"/>
+      <c r="M32" s="105"/>
     </row>
     <row r="33" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="32">
@@ -12277,16 +12277,16 @@
         <v>122</v>
       </c>
       <c r="C33" s="33"/>
-      <c r="D33" s="87"/>
-      <c r="E33" s="88"/>
-      <c r="F33" s="88"/>
-      <c r="G33" s="88"/>
-      <c r="H33" s="88"/>
-      <c r="I33" s="88"/>
-      <c r="J33" s="88"/>
-      <c r="K33" s="88"/>
-      <c r="L33" s="88"/>
-      <c r="M33" s="88"/>
+      <c r="D33" s="104"/>
+      <c r="E33" s="105"/>
+      <c r="F33" s="105"/>
+      <c r="G33" s="105"/>
+      <c r="H33" s="105"/>
+      <c r="I33" s="105"/>
+      <c r="J33" s="105"/>
+      <c r="K33" s="105"/>
+      <c r="L33" s="105"/>
+      <c r="M33" s="105"/>
     </row>
     <row r="34" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="32">
@@ -12296,16 +12296,16 @@
         <v>123</v>
       </c>
       <c r="C34" s="32"/>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="88"/>
-      <c r="G34" s="88"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="88"/>
-      <c r="J34" s="88"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="88"/>
-      <c r="M34" s="88"/>
+      <c r="D34" s="104"/>
+      <c r="E34" s="105"/>
+      <c r="F34" s="105"/>
+      <c r="G34" s="105"/>
+      <c r="H34" s="105"/>
+      <c r="I34" s="105"/>
+      <c r="J34" s="105"/>
+      <c r="K34" s="105"/>
+      <c r="L34" s="105"/>
+      <c r="M34" s="105"/>
     </row>
     <row r="35" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="32">
@@ -12315,16 +12315,16 @@
         <v>124</v>
       </c>
       <c r="C35" s="32"/>
-      <c r="D35" s="87"/>
-      <c r="E35" s="88"/>
-      <c r="F35" s="88"/>
-      <c r="G35" s="88"/>
-      <c r="H35" s="88"/>
-      <c r="I35" s="88"/>
-      <c r="J35" s="88"/>
-      <c r="K35" s="88"/>
-      <c r="L35" s="88"/>
-      <c r="M35" s="88"/>
+      <c r="D35" s="104"/>
+      <c r="E35" s="105"/>
+      <c r="F35" s="105"/>
+      <c r="G35" s="105"/>
+      <c r="H35" s="105"/>
+      <c r="I35" s="105"/>
+      <c r="J35" s="105"/>
+      <c r="K35" s="105"/>
+      <c r="L35" s="105"/>
+      <c r="M35" s="105"/>
     </row>
     <row r="36" spans="1:13" ht="18.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="32">
@@ -12334,16 +12334,16 @@
         <v>125</v>
       </c>
       <c r="C36" s="32"/>
-      <c r="D36" s="87"/>
-      <c r="E36" s="88"/>
-      <c r="F36" s="88"/>
-      <c r="G36" s="88"/>
-      <c r="H36" s="88"/>
-      <c r="I36" s="88"/>
-      <c r="J36" s="88"/>
-      <c r="K36" s="88"/>
-      <c r="L36" s="88"/>
-      <c r="M36" s="88"/>
+      <c r="D36" s="104"/>
+      <c r="E36" s="105"/>
+      <c r="F36" s="105"/>
+      <c r="G36" s="105"/>
+      <c r="H36" s="105"/>
+      <c r="I36" s="105"/>
+      <c r="J36" s="105"/>
+      <c r="K36" s="105"/>
+      <c r="L36" s="105"/>
+      <c r="M36" s="105"/>
     </row>
     <row r="37" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="32">
@@ -12353,16 +12353,16 @@
         <v>126</v>
       </c>
       <c r="C37" s="32"/>
-      <c r="D37" s="87"/>
-      <c r="E37" s="88"/>
-      <c r="F37" s="88"/>
-      <c r="G37" s="88"/>
-      <c r="H37" s="88"/>
-      <c r="I37" s="88"/>
-      <c r="J37" s="88"/>
-      <c r="K37" s="88"/>
-      <c r="L37" s="88"/>
-      <c r="M37" s="88"/>
+      <c r="D37" s="104"/>
+      <c r="E37" s="105"/>
+      <c r="F37" s="105"/>
+      <c r="G37" s="105"/>
+      <c r="H37" s="105"/>
+      <c r="I37" s="105"/>
+      <c r="J37" s="105"/>
+      <c r="K37" s="105"/>
+      <c r="L37" s="105"/>
+      <c r="M37" s="105"/>
     </row>
     <row r="38" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="32">
@@ -12372,16 +12372,16 @@
         <v>127</v>
       </c>
       <c r="C38" s="32"/>
-      <c r="D38" s="87"/>
-      <c r="E38" s="88"/>
-      <c r="F38" s="88"/>
-      <c r="G38" s="88"/>
-      <c r="H38" s="88"/>
-      <c r="I38" s="88"/>
-      <c r="J38" s="88"/>
-      <c r="K38" s="88"/>
-      <c r="L38" s="88"/>
-      <c r="M38" s="88"/>
+      <c r="D38" s="104"/>
+      <c r="E38" s="105"/>
+      <c r="F38" s="105"/>
+      <c r="G38" s="105"/>
+      <c r="H38" s="105"/>
+      <c r="I38" s="105"/>
+      <c r="J38" s="105"/>
+      <c r="K38" s="105"/>
+      <c r="L38" s="105"/>
+      <c r="M38" s="105"/>
     </row>
     <row r="39" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="32">
@@ -12391,16 +12391,16 @@
         <v>128</v>
       </c>
       <c r="C39" s="32"/>
-      <c r="D39" s="87"/>
-      <c r="E39" s="88"/>
-      <c r="F39" s="88"/>
-      <c r="G39" s="88"/>
-      <c r="H39" s="88"/>
-      <c r="I39" s="88"/>
-      <c r="J39" s="88"/>
-      <c r="K39" s="88"/>
-      <c r="L39" s="88"/>
-      <c r="M39" s="88"/>
+      <c r="D39" s="104"/>
+      <c r="E39" s="105"/>
+      <c r="F39" s="105"/>
+      <c r="G39" s="105"/>
+      <c r="H39" s="105"/>
+      <c r="I39" s="105"/>
+      <c r="J39" s="105"/>
+      <c r="K39" s="105"/>
+      <c r="L39" s="105"/>
+      <c r="M39" s="105"/>
     </row>
     <row r="40" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="32">
@@ -12410,16 +12410,16 @@
         <v>129</v>
       </c>
       <c r="C40" s="32"/>
-      <c r="D40" s="87"/>
-      <c r="E40" s="88"/>
-      <c r="F40" s="88"/>
-      <c r="G40" s="88"/>
-      <c r="H40" s="88"/>
-      <c r="I40" s="88"/>
-      <c r="J40" s="88"/>
-      <c r="K40" s="88"/>
-      <c r="L40" s="88"/>
-      <c r="M40" s="88"/>
+      <c r="D40" s="104"/>
+      <c r="E40" s="105"/>
+      <c r="F40" s="105"/>
+      <c r="G40" s="105"/>
+      <c r="H40" s="105"/>
+      <c r="I40" s="105"/>
+      <c r="J40" s="105"/>
+      <c r="K40" s="105"/>
+      <c r="L40" s="105"/>
+      <c r="M40" s="105"/>
     </row>
     <row r="41" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="32">
@@ -12429,16 +12429,16 @@
         <v>130</v>
       </c>
       <c r="C41" s="32"/>
-      <c r="D41" s="87"/>
-      <c r="E41" s="88"/>
-      <c r="F41" s="88"/>
-      <c r="G41" s="88"/>
-      <c r="H41" s="88"/>
-      <c r="I41" s="88"/>
-      <c r="J41" s="88"/>
-      <c r="K41" s="88"/>
-      <c r="L41" s="88"/>
-      <c r="M41" s="88"/>
+      <c r="D41" s="104"/>
+      <c r="E41" s="105"/>
+      <c r="F41" s="105"/>
+      <c r="G41" s="105"/>
+      <c r="H41" s="105"/>
+      <c r="I41" s="105"/>
+      <c r="J41" s="105"/>
+      <c r="K41" s="105"/>
+      <c r="L41" s="105"/>
+      <c r="M41" s="105"/>
     </row>
     <row r="42" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="32">
@@ -12448,16 +12448,16 @@
         <v>131</v>
       </c>
       <c r="C42" s="32"/>
-      <c r="D42" s="87"/>
-      <c r="E42" s="88"/>
-      <c r="F42" s="88"/>
-      <c r="G42" s="88"/>
-      <c r="H42" s="88"/>
-      <c r="I42" s="88"/>
-      <c r="J42" s="88"/>
-      <c r="K42" s="88"/>
-      <c r="L42" s="88"/>
-      <c r="M42" s="88"/>
+      <c r="D42" s="104"/>
+      <c r="E42" s="105"/>
+      <c r="F42" s="105"/>
+      <c r="G42" s="105"/>
+      <c r="H42" s="105"/>
+      <c r="I42" s="105"/>
+      <c r="J42" s="105"/>
+      <c r="K42" s="105"/>
+      <c r="L42" s="105"/>
+      <c r="M42" s="105"/>
     </row>
     <row r="43" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="32">
@@ -12467,529 +12467,529 @@
         <v>132</v>
       </c>
       <c r="C43" s="32"/>
-      <c r="D43" s="87"/>
-      <c r="E43" s="88"/>
-      <c r="F43" s="88"/>
-      <c r="G43" s="88"/>
-      <c r="H43" s="88"/>
-      <c r="I43" s="88"/>
-      <c r="J43" s="88"/>
-      <c r="K43" s="88"/>
-      <c r="L43" s="88"/>
-      <c r="M43" s="88"/>
+      <c r="D43" s="104"/>
+      <c r="E43" s="105"/>
+      <c r="F43" s="105"/>
+      <c r="G43" s="105"/>
+      <c r="H43" s="105"/>
+      <c r="I43" s="105"/>
+      <c r="J43" s="105"/>
+      <c r="K43" s="105"/>
+      <c r="L43" s="105"/>
+      <c r="M43" s="105"/>
     </row>
     <row r="44" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="32">
         <v>19</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
       <c r="C44" s="32"/>
-      <c r="D44" s="87"/>
-      <c r="E44" s="88"/>
-      <c r="F44" s="88"/>
-      <c r="G44" s="88"/>
-      <c r="H44" s="88"/>
-      <c r="I44" s="88"/>
-      <c r="J44" s="88"/>
-      <c r="K44" s="88"/>
-      <c r="L44" s="88"/>
-      <c r="M44" s="88"/>
+      <c r="D44" s="104"/>
+      <c r="E44" s="105"/>
+      <c r="F44" s="105"/>
+      <c r="G44" s="105"/>
+      <c r="H44" s="105"/>
+      <c r="I44" s="105"/>
+      <c r="J44" s="105"/>
+      <c r="K44" s="105"/>
+      <c r="L44" s="105"/>
+      <c r="M44" s="105"/>
     </row>
     <row r="45" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="32">
         <v>20</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C45" s="32"/>
-      <c r="D45" s="87"/>
-      <c r="E45" s="88"/>
-      <c r="F45" s="88"/>
-      <c r="G45" s="88"/>
-      <c r="H45" s="88"/>
-      <c r="I45" s="88"/>
-      <c r="J45" s="88"/>
-      <c r="K45" s="88"/>
-      <c r="L45" s="88"/>
-      <c r="M45" s="88"/>
+      <c r="D45" s="104"/>
+      <c r="E45" s="105"/>
+      <c r="F45" s="105"/>
+      <c r="G45" s="105"/>
+      <c r="H45" s="105"/>
+      <c r="I45" s="105"/>
+      <c r="J45" s="105"/>
+      <c r="K45" s="105"/>
+      <c r="L45" s="105"/>
+      <c r="M45" s="105"/>
     </row>
     <row r="46" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="32">
         <v>21</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C46" s="32"/>
-      <c r="D46" s="87"/>
-      <c r="E46" s="88"/>
-      <c r="F46" s="88"/>
-      <c r="G46" s="88"/>
-      <c r="H46" s="88"/>
-      <c r="I46" s="88"/>
-      <c r="J46" s="88"/>
-      <c r="K46" s="88"/>
-      <c r="L46" s="88"/>
-      <c r="M46" s="88"/>
+      <c r="D46" s="104"/>
+      <c r="E46" s="105"/>
+      <c r="F46" s="105"/>
+      <c r="G46" s="105"/>
+      <c r="H46" s="105"/>
+      <c r="I46" s="105"/>
+      <c r="J46" s="105"/>
+      <c r="K46" s="105"/>
+      <c r="L46" s="105"/>
+      <c r="M46" s="105"/>
     </row>
     <row r="47" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="32">
         <v>22</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C47" s="32"/>
-      <c r="D47" s="87"/>
-      <c r="E47" s="88"/>
-      <c r="F47" s="88"/>
-      <c r="G47" s="88"/>
-      <c r="H47" s="88"/>
-      <c r="I47" s="88"/>
-      <c r="J47" s="88"/>
-      <c r="K47" s="88"/>
-      <c r="L47" s="88"/>
-      <c r="M47" s="88"/>
+      <c r="D47" s="104"/>
+      <c r="E47" s="105"/>
+      <c r="F47" s="105"/>
+      <c r="G47" s="105"/>
+      <c r="H47" s="105"/>
+      <c r="I47" s="105"/>
+      <c r="J47" s="105"/>
+      <c r="K47" s="105"/>
+      <c r="L47" s="105"/>
+      <c r="M47" s="105"/>
     </row>
     <row r="48" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="32">
         <v>23</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C48" s="32"/>
-      <c r="D48" s="87"/>
-      <c r="E48" s="88"/>
-      <c r="F48" s="88"/>
-      <c r="G48" s="88"/>
-      <c r="H48" s="88"/>
-      <c r="I48" s="88"/>
-      <c r="J48" s="88"/>
-      <c r="K48" s="88"/>
-      <c r="L48" s="88"/>
-      <c r="M48" s="88"/>
+      <c r="D48" s="104"/>
+      <c r="E48" s="105"/>
+      <c r="F48" s="105"/>
+      <c r="G48" s="105"/>
+      <c r="H48" s="105"/>
+      <c r="I48" s="105"/>
+      <c r="J48" s="105"/>
+      <c r="K48" s="105"/>
+      <c r="L48" s="105"/>
+      <c r="M48" s="105"/>
     </row>
     <row r="49" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="32">
         <v>24</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C49" s="32"/>
-      <c r="D49" s="87"/>
-      <c r="E49" s="88"/>
-      <c r="F49" s="88"/>
-      <c r="G49" s="88"/>
-      <c r="H49" s="88"/>
-      <c r="I49" s="88"/>
-      <c r="J49" s="88"/>
-      <c r="K49" s="88"/>
-      <c r="L49" s="88"/>
-      <c r="M49" s="88"/>
+      <c r="D49" s="104"/>
+      <c r="E49" s="105"/>
+      <c r="F49" s="105"/>
+      <c r="G49" s="105"/>
+      <c r="H49" s="105"/>
+      <c r="I49" s="105"/>
+      <c r="J49" s="105"/>
+      <c r="K49" s="105"/>
+      <c r="L49" s="105"/>
+      <c r="M49" s="105"/>
     </row>
     <row r="50" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="32">
         <v>25</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C50" s="32"/>
-      <c r="D50" s="87"/>
-      <c r="E50" s="88"/>
-      <c r="F50" s="88"/>
-      <c r="G50" s="88"/>
-      <c r="H50" s="88"/>
-      <c r="I50" s="88"/>
-      <c r="J50" s="88"/>
-      <c r="K50" s="88"/>
-      <c r="L50" s="88"/>
-      <c r="M50" s="88"/>
+      <c r="D50" s="104"/>
+      <c r="E50" s="105"/>
+      <c r="F50" s="105"/>
+      <c r="G50" s="105"/>
+      <c r="H50" s="105"/>
+      <c r="I50" s="105"/>
+      <c r="J50" s="105"/>
+      <c r="K50" s="105"/>
+      <c r="L50" s="105"/>
+      <c r="M50" s="105"/>
     </row>
     <row r="51" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="32">
         <v>26</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C51" s="32"/>
-      <c r="D51" s="87"/>
-      <c r="E51" s="88"/>
-      <c r="F51" s="88"/>
-      <c r="G51" s="88"/>
-      <c r="H51" s="88"/>
-      <c r="I51" s="88"/>
-      <c r="J51" s="88"/>
-      <c r="K51" s="88"/>
-      <c r="L51" s="88"/>
-      <c r="M51" s="88"/>
+      <c r="D51" s="104"/>
+      <c r="E51" s="105"/>
+      <c r="F51" s="105"/>
+      <c r="G51" s="105"/>
+      <c r="H51" s="105"/>
+      <c r="I51" s="105"/>
+      <c r="J51" s="105"/>
+      <c r="K51" s="105"/>
+      <c r="L51" s="105"/>
+      <c r="M51" s="105"/>
     </row>
     <row r="52" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="32">
         <v>27</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C52" s="32"/>
-      <c r="D52" s="87"/>
-      <c r="E52" s="88"/>
-      <c r="F52" s="88"/>
-      <c r="G52" s="88"/>
-      <c r="H52" s="88"/>
-      <c r="I52" s="88"/>
-      <c r="J52" s="88"/>
-      <c r="K52" s="88"/>
-      <c r="L52" s="88"/>
-      <c r="M52" s="88"/>
+      <c r="D52" s="104"/>
+      <c r="E52" s="105"/>
+      <c r="F52" s="105"/>
+      <c r="G52" s="105"/>
+      <c r="H52" s="105"/>
+      <c r="I52" s="105"/>
+      <c r="J52" s="105"/>
+      <c r="K52" s="105"/>
+      <c r="L52" s="105"/>
+      <c r="M52" s="105"/>
     </row>
     <row r="53" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="32">
         <v>28</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C53" s="32"/>
-      <c r="D53" s="87"/>
-      <c r="E53" s="88"/>
-      <c r="F53" s="88"/>
-      <c r="G53" s="88"/>
-      <c r="H53" s="88"/>
-      <c r="I53" s="88"/>
-      <c r="J53" s="88"/>
-      <c r="K53" s="88"/>
-      <c r="L53" s="88"/>
-      <c r="M53" s="88"/>
+      <c r="D53" s="104"/>
+      <c r="E53" s="105"/>
+      <c r="F53" s="105"/>
+      <c r="G53" s="105"/>
+      <c r="H53" s="105"/>
+      <c r="I53" s="105"/>
+      <c r="J53" s="105"/>
+      <c r="K53" s="105"/>
+      <c r="L53" s="105"/>
+      <c r="M53" s="105"/>
     </row>
     <row r="54" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="32">
         <v>29</v>
       </c>
       <c r="B54" s="33" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C54" s="32"/>
-      <c r="D54" s="87"/>
-      <c r="E54" s="88"/>
-      <c r="F54" s="88"/>
-      <c r="G54" s="88"/>
-      <c r="H54" s="88"/>
-      <c r="I54" s="88"/>
-      <c r="J54" s="88"/>
-      <c r="K54" s="88"/>
-      <c r="L54" s="88"/>
-      <c r="M54" s="88"/>
+      <c r="D54" s="104"/>
+      <c r="E54" s="105"/>
+      <c r="F54" s="105"/>
+      <c r="G54" s="105"/>
+      <c r="H54" s="105"/>
+      <c r="I54" s="105"/>
+      <c r="J54" s="105"/>
+      <c r="K54" s="105"/>
+      <c r="L54" s="105"/>
+      <c r="M54" s="105"/>
     </row>
     <row r="55" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="32">
         <v>30</v>
       </c>
       <c r="B55" s="33" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C55" s="32"/>
-      <c r="D55" s="87"/>
-      <c r="E55" s="88"/>
-      <c r="F55" s="88"/>
-      <c r="G55" s="88"/>
-      <c r="H55" s="88"/>
-      <c r="I55" s="88"/>
-      <c r="J55" s="88"/>
-      <c r="K55" s="88"/>
-      <c r="L55" s="88"/>
-      <c r="M55" s="88"/>
+      <c r="D55" s="104"/>
+      <c r="E55" s="105"/>
+      <c r="F55" s="105"/>
+      <c r="G55" s="105"/>
+      <c r="H55" s="105"/>
+      <c r="I55" s="105"/>
+      <c r="J55" s="105"/>
+      <c r="K55" s="105"/>
+      <c r="L55" s="105"/>
+      <c r="M55" s="105"/>
     </row>
     <row r="56" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="32">
         <v>31</v>
       </c>
       <c r="B56" s="33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C56" s="32"/>
-      <c r="D56" s="87"/>
-      <c r="E56" s="88"/>
-      <c r="F56" s="88"/>
-      <c r="G56" s="88"/>
-      <c r="H56" s="88"/>
-      <c r="I56" s="88"/>
-      <c r="J56" s="88"/>
-      <c r="K56" s="88"/>
-      <c r="L56" s="88"/>
-      <c r="M56" s="88"/>
+      <c r="D56" s="104"/>
+      <c r="E56" s="105"/>
+      <c r="F56" s="105"/>
+      <c r="G56" s="105"/>
+      <c r="H56" s="105"/>
+      <c r="I56" s="105"/>
+      <c r="J56" s="105"/>
+      <c r="K56" s="105"/>
+      <c r="L56" s="105"/>
+      <c r="M56" s="105"/>
     </row>
     <row r="57" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="32">
         <v>32</v>
       </c>
       <c r="B57" s="33" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C57" s="32"/>
-      <c r="D57" s="87"/>
-      <c r="E57" s="88"/>
-      <c r="F57" s="88"/>
-      <c r="G57" s="88"/>
-      <c r="H57" s="88"/>
-      <c r="I57" s="88"/>
-      <c r="J57" s="88"/>
-      <c r="K57" s="88"/>
-      <c r="L57" s="88"/>
-      <c r="M57" s="88"/>
+      <c r="D57" s="104"/>
+      <c r="E57" s="105"/>
+      <c r="F57" s="105"/>
+      <c r="G57" s="105"/>
+      <c r="H57" s="105"/>
+      <c r="I57" s="105"/>
+      <c r="J57" s="105"/>
+      <c r="K57" s="105"/>
+      <c r="L57" s="105"/>
+      <c r="M57" s="105"/>
     </row>
     <row r="58" spans="1:13" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="32">
         <v>33</v>
       </c>
       <c r="B58" s="33" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C58" s="32"/>
-      <c r="D58" s="87"/>
-      <c r="E58" s="88"/>
-      <c r="F58" s="88"/>
-      <c r="G58" s="88"/>
-      <c r="H58" s="88"/>
-      <c r="I58" s="88"/>
-      <c r="J58" s="88"/>
-      <c r="K58" s="88"/>
-      <c r="L58" s="88"/>
-      <c r="M58" s="88"/>
+      <c r="D58" s="104"/>
+      <c r="E58" s="105"/>
+      <c r="F58" s="105"/>
+      <c r="G58" s="105"/>
+      <c r="H58" s="105"/>
+      <c r="I58" s="105"/>
+      <c r="J58" s="105"/>
+      <c r="K58" s="105"/>
+      <c r="L58" s="105"/>
+      <c r="M58" s="105"/>
     </row>
     <row r="59" spans="1:13" ht="21.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="32">
         <v>34</v>
       </c>
       <c r="B59" s="33" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C59" s="32"/>
-      <c r="D59" s="87"/>
-      <c r="E59" s="88"/>
-      <c r="F59" s="88"/>
-      <c r="G59" s="88"/>
-      <c r="H59" s="88"/>
-      <c r="I59" s="88"/>
-      <c r="J59" s="88"/>
-      <c r="K59" s="88"/>
-      <c r="L59" s="88"/>
-      <c r="M59" s="88"/>
+      <c r="D59" s="104"/>
+      <c r="E59" s="105"/>
+      <c r="F59" s="105"/>
+      <c r="G59" s="105"/>
+      <c r="H59" s="105"/>
+      <c r="I59" s="105"/>
+      <c r="J59" s="105"/>
+      <c r="K59" s="105"/>
+      <c r="L59" s="105"/>
+      <c r="M59" s="105"/>
     </row>
     <row r="60" spans="1:13" ht="21.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="32">
         <v>35</v>
       </c>
       <c r="B60" s="33" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C60" s="32"/>
-      <c r="D60" s="87"/>
-      <c r="E60" s="88"/>
-      <c r="F60" s="88"/>
-      <c r="G60" s="88"/>
-      <c r="H60" s="88"/>
-      <c r="I60" s="88"/>
-      <c r="J60" s="88"/>
-      <c r="K60" s="88"/>
-      <c r="L60" s="88"/>
-      <c r="M60" s="88"/>
+      <c r="D60" s="104"/>
+      <c r="E60" s="105"/>
+      <c r="F60" s="105"/>
+      <c r="G60" s="105"/>
+      <c r="H60" s="105"/>
+      <c r="I60" s="105"/>
+      <c r="J60" s="105"/>
+      <c r="K60" s="105"/>
+      <c r="L60" s="105"/>
+      <c r="M60" s="105"/>
     </row>
     <row r="61" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="32">
         <v>36</v>
       </c>
       <c r="B61" s="33" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C61" s="32"/>
-      <c r="D61" s="87"/>
-      <c r="E61" s="88"/>
-      <c r="F61" s="88"/>
-      <c r="G61" s="88"/>
-      <c r="H61" s="88"/>
-      <c r="I61" s="88"/>
-      <c r="J61" s="88"/>
-      <c r="K61" s="88"/>
-      <c r="L61" s="88"/>
-      <c r="M61" s="88"/>
+      <c r="D61" s="104"/>
+      <c r="E61" s="105"/>
+      <c r="F61" s="105"/>
+      <c r="G61" s="105"/>
+      <c r="H61" s="105"/>
+      <c r="I61" s="105"/>
+      <c r="J61" s="105"/>
+      <c r="K61" s="105"/>
+      <c r="L61" s="105"/>
+      <c r="M61" s="105"/>
     </row>
     <row r="62" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="32">
         <v>37</v>
       </c>
       <c r="B62" s="33" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C62" s="32"/>
-      <c r="D62" s="87"/>
-      <c r="E62" s="88"/>
-      <c r="F62" s="88"/>
-      <c r="G62" s="88"/>
-      <c r="H62" s="88"/>
-      <c r="I62" s="88"/>
-      <c r="J62" s="88"/>
-      <c r="K62" s="88"/>
-      <c r="L62" s="88"/>
-      <c r="M62" s="88"/>
+      <c r="D62" s="104"/>
+      <c r="E62" s="105"/>
+      <c r="F62" s="105"/>
+      <c r="G62" s="105"/>
+      <c r="H62" s="105"/>
+      <c r="I62" s="105"/>
+      <c r="J62" s="105"/>
+      <c r="K62" s="105"/>
+      <c r="L62" s="105"/>
+      <c r="M62" s="105"/>
     </row>
     <row r="63" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="32">
         <v>38</v>
       </c>
       <c r="B63" s="33" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C63" s="32"/>
-      <c r="D63" s="87"/>
-      <c r="E63" s="88"/>
-      <c r="F63" s="88"/>
-      <c r="G63" s="88"/>
-      <c r="H63" s="88"/>
-      <c r="I63" s="88"/>
-      <c r="J63" s="88"/>
-      <c r="K63" s="88"/>
-      <c r="L63" s="88"/>
-      <c r="M63" s="88"/>
+      <c r="D63" s="104"/>
+      <c r="E63" s="105"/>
+      <c r="F63" s="105"/>
+      <c r="G63" s="105"/>
+      <c r="H63" s="105"/>
+      <c r="I63" s="105"/>
+      <c r="J63" s="105"/>
+      <c r="K63" s="105"/>
+      <c r="L63" s="105"/>
+      <c r="M63" s="105"/>
     </row>
     <row r="64" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="32">
         <v>39</v>
       </c>
       <c r="B64" s="33" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C64" s="32"/>
-      <c r="D64" s="87"/>
-      <c r="E64" s="88"/>
-      <c r="F64" s="88"/>
-      <c r="G64" s="88"/>
-      <c r="H64" s="88"/>
-      <c r="I64" s="88"/>
-      <c r="J64" s="88"/>
-      <c r="K64" s="88"/>
-      <c r="L64" s="88"/>
-      <c r="M64" s="88"/>
+      <c r="D64" s="104"/>
+      <c r="E64" s="105"/>
+      <c r="F64" s="105"/>
+      <c r="G64" s="105"/>
+      <c r="H64" s="105"/>
+      <c r="I64" s="105"/>
+      <c r="J64" s="105"/>
+      <c r="K64" s="105"/>
+      <c r="L64" s="105"/>
+      <c r="M64" s="105"/>
     </row>
     <row r="65" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="32">
         <v>40</v>
       </c>
       <c r="B65" s="33" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C65" s="32"/>
-      <c r="D65" s="87"/>
-      <c r="E65" s="88"/>
-      <c r="F65" s="88"/>
-      <c r="G65" s="88"/>
-      <c r="H65" s="88"/>
-      <c r="I65" s="88"/>
-      <c r="J65" s="88"/>
-      <c r="K65" s="88"/>
-      <c r="L65" s="88"/>
-      <c r="M65" s="88"/>
+      <c r="D65" s="104"/>
+      <c r="E65" s="105"/>
+      <c r="F65" s="105"/>
+      <c r="G65" s="105"/>
+      <c r="H65" s="105"/>
+      <c r="I65" s="105"/>
+      <c r="J65" s="105"/>
+      <c r="K65" s="105"/>
+      <c r="L65" s="105"/>
+      <c r="M65" s="105"/>
     </row>
     <row r="66" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="32">
         <v>41</v>
       </c>
       <c r="B66" s="33" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C66" s="32"/>
-      <c r="D66" s="87"/>
-      <c r="E66" s="88"/>
-      <c r="F66" s="88"/>
-      <c r="G66" s="88"/>
-      <c r="H66" s="88"/>
-      <c r="I66" s="88"/>
-      <c r="J66" s="88"/>
-      <c r="K66" s="88"/>
-      <c r="L66" s="88"/>
-      <c r="M66" s="88"/>
+      <c r="D66" s="104"/>
+      <c r="E66" s="105"/>
+      <c r="F66" s="105"/>
+      <c r="G66" s="105"/>
+      <c r="H66" s="105"/>
+      <c r="I66" s="105"/>
+      <c r="J66" s="105"/>
+      <c r="K66" s="105"/>
+      <c r="L66" s="105"/>
+      <c r="M66" s="105"/>
     </row>
     <row r="67" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="32">
         <v>42</v>
       </c>
       <c r="B67" s="33" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C67" s="32"/>
-      <c r="D67" s="87"/>
-      <c r="E67" s="88"/>
-      <c r="F67" s="88"/>
-      <c r="G67" s="88"/>
-      <c r="H67" s="88"/>
-      <c r="I67" s="88"/>
-      <c r="J67" s="88"/>
-      <c r="K67" s="88"/>
-      <c r="L67" s="88"/>
-      <c r="M67" s="88"/>
+      <c r="D67" s="104"/>
+      <c r="E67" s="105"/>
+      <c r="F67" s="105"/>
+      <c r="G67" s="105"/>
+      <c r="H67" s="105"/>
+      <c r="I67" s="105"/>
+      <c r="J67" s="105"/>
+      <c r="K67" s="105"/>
+      <c r="L67" s="105"/>
+      <c r="M67" s="105"/>
     </row>
     <row r="68" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="32">
         <v>43</v>
       </c>
       <c r="B68" s="33" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C68" s="32"/>
-      <c r="D68" s="87"/>
-      <c r="E68" s="88"/>
-      <c r="F68" s="88"/>
-      <c r="G68" s="88"/>
-      <c r="H68" s="88"/>
-      <c r="I68" s="88"/>
-      <c r="J68" s="88"/>
-      <c r="K68" s="88"/>
-      <c r="L68" s="88"/>
-      <c r="M68" s="88"/>
+      <c r="D68" s="104"/>
+      <c r="E68" s="105"/>
+      <c r="F68" s="105"/>
+      <c r="G68" s="105"/>
+      <c r="H68" s="105"/>
+      <c r="I68" s="105"/>
+      <c r="J68" s="105"/>
+      <c r="K68" s="105"/>
+      <c r="L68" s="105"/>
+      <c r="M68" s="105"/>
     </row>
     <row r="69" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="32">
         <v>44</v>
       </c>
       <c r="B69" s="33" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C69" s="32"/>
-      <c r="D69" s="87"/>
-      <c r="E69" s="88"/>
-      <c r="F69" s="88"/>
-      <c r="G69" s="88"/>
-      <c r="H69" s="88"/>
-      <c r="I69" s="88"/>
-      <c r="J69" s="88"/>
-      <c r="K69" s="88"/>
-      <c r="L69" s="88"/>
-      <c r="M69" s="88"/>
+      <c r="D69" s="104"/>
+      <c r="E69" s="105"/>
+      <c r="F69" s="105"/>
+      <c r="G69" s="105"/>
+      <c r="H69" s="105"/>
+      <c r="I69" s="105"/>
+      <c r="J69" s="105"/>
+      <c r="K69" s="105"/>
+      <c r="L69" s="105"/>
+      <c r="M69" s="105"/>
     </row>
     <row r="70" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="32">
         <v>45</v>
       </c>
       <c r="B70" s="33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C70" s="32"/>
-      <c r="D70" s="87"/>
-      <c r="E70" s="88"/>
-      <c r="F70" s="88"/>
-      <c r="G70" s="88"/>
-      <c r="H70" s="88"/>
-      <c r="I70" s="88"/>
-      <c r="J70" s="88"/>
-      <c r="K70" s="88"/>
-      <c r="L70" s="88"/>
-      <c r="M70" s="88"/>
+      <c r="D70" s="104"/>
+      <c r="E70" s="105"/>
+      <c r="F70" s="105"/>
+      <c r="G70" s="105"/>
+      <c r="H70" s="105"/>
+      <c r="I70" s="105"/>
+      <c r="J70" s="105"/>
+      <c r="K70" s="105"/>
+      <c r="L70" s="105"/>
+      <c r="M70" s="105"/>
     </row>
     <row r="71" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="32">
@@ -12999,41 +12999,34 @@
         <v>160</v>
       </c>
       <c r="C71" s="32"/>
-      <c r="D71" s="87"/>
-      <c r="E71" s="88"/>
-      <c r="F71" s="88"/>
-      <c r="G71" s="88"/>
-      <c r="H71" s="88"/>
-      <c r="I71" s="88"/>
-      <c r="J71" s="88"/>
-      <c r="K71" s="88"/>
-      <c r="L71" s="88"/>
-      <c r="M71" s="88"/>
+      <c r="D71" s="104"/>
+      <c r="E71" s="105"/>
+      <c r="F71" s="105"/>
+      <c r="G71" s="105"/>
+      <c r="H71" s="105"/>
+      <c r="I71" s="105"/>
+      <c r="J71" s="105"/>
+      <c r="K71" s="105"/>
+      <c r="L71" s="105"/>
+      <c r="M71" s="105"/>
     </row>
     <row r="72" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="32"/>
       <c r="B72" s="33"/>
       <c r="C72" s="32"/>
-      <c r="D72" s="87"/>
-      <c r="E72" s="88"/>
-      <c r="F72" s="88"/>
-      <c r="G72" s="88"/>
-      <c r="H72" s="88"/>
-      <c r="I72" s="88"/>
-      <c r="J72" s="88"/>
-      <c r="K72" s="88"/>
-      <c r="L72" s="88"/>
-      <c r="M72" s="88"/>
+      <c r="D72" s="104"/>
+      <c r="E72" s="105"/>
+      <c r="F72" s="105"/>
+      <c r="G72" s="105"/>
+      <c r="H72" s="105"/>
+      <c r="I72" s="105"/>
+      <c r="J72" s="105"/>
+      <c r="K72" s="105"/>
+      <c r="L72" s="105"/>
+      <c r="M72" s="105"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="B6:M6"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A9:M9"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="B5:M5"/>
-    <mergeCell ref="B7:M7"/>
     <mergeCell ref="E21:M22"/>
     <mergeCell ref="A16:M16"/>
     <mergeCell ref="A17:M17"/>
@@ -13046,6 +13039,13 @@
     <mergeCell ref="A23:M23"/>
     <mergeCell ref="A24:M24"/>
     <mergeCell ref="D21:D22"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="B6:M6"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="B7:M7"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
@@ -17372,6 +17372,68 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
+      <UserInfo>
+        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
+        <AccountId>265</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
+        <AccountId>322</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
+        <AccountId>304</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
+        <AccountId>299</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
+        <AccountId>369</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
+        <AccountId>355</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
+        <AccountId>321</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
+        <AccountId>370</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005DA7AC6E4F4FAE42B9D9FCD9C82CAAE1" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="553e0bb76796fbad2df2b84fb95dc83d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87481c51-c14c-4071-bf64-faa2b5708bb6" xmlns:ns3="8029d101-3d2a-47c4-b15f-619642bf5e50" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d87cd7f238c73dc12c577d08dde48736" ns2:_="" ns3:_="">
     <xsd:import namespace="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
@@ -17620,69 +17682,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
+    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
-      <UserInfo>
-        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
-        <AccountId>265</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
-        <AccountId>322</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
-        <AccountId>304</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
-        <AccountId>299</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
-        <AccountId>369</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
-        <AccountId>355</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
-        <AccountId>321</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
-        <AccountId>370</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F7F06D0-41B3-4EAF-B418-88FC726117CC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17699,23 +17718,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
-    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fiix modificacion de scripts
</commit_message>
<xml_diff>
--- a/Guias Produccion/HU-55188.xlsx
+++ b/Guias Produccion/HU-55188.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Alliance\ScriptsEntidades\Guias Produccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089F567C-7287-4B83-905B-DB1E57CEAAFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1BA18FD-D63D-4E26-ADDB-4C94D494DC94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="165">
   <si>
     <t>Guia documentación</t>
   </si>
@@ -570,79 +570,94 @@
     <t>20-AlterDocumentoDespacho.sql</t>
   </si>
   <si>
-    <t>21-AddDictionaryParametrosLista.sql</t>
+    <t>21-AlterClienteCategoriaClientes.sql</t>
   </si>
   <si>
-    <t>22-AddDictionaryUsuarios.sql</t>
+    <t>22-AlterClienteTarifasLocales.sql</t>
   </si>
   <si>
-    <t>23-CreateIndexes_Entities.sql</t>
+    <t>23-AddDictionaryParametrosLista.sql</t>
   </si>
   <si>
-    <t>24-CreateIndexes_GuiasHouse.sql</t>
+    <t>24-AddDictionaryUsuarios.sql</t>
   </si>
   <si>
-    <t>25-CreateIndexes_GuiasHouseDetalles.sql</t>
+    <t>25-CreateIndexes_Entities.sql</t>
   </si>
   <si>
-    <t>26-CreateIndexes_OrdenesLocales.sql</t>
+    <t>26-CreateIndexes_GuiasHouse.sql</t>
   </si>
   <si>
-    <t>27-InsertContadoresTablaExcludedContacts.sql</t>
+    <t>27-CreateIndexes_GuiasHouseDetalles.sql</t>
   </si>
   <si>
-    <t>28-InsertContadoresTablaRolesActors.sql</t>
+    <t>28-CreateIndexes_OrdenesLocales.sql</t>
   </si>
   <si>
-    <t>29-InsertContadoresTablaEntityRelations.sql</t>
+    <t>29-InsertContadoresTablaExcludedContacts.sql</t>
   </si>
   <si>
-    <t>30-InsertContadoresTablaEntities.sql</t>
+    <t>30-InsertContadoresTablaRolesActors.sql</t>
   </si>
   <si>
-    <t>31-InsertContadoresTablaEntityTypes.sql</t>
+    <t>31-InsertContadoresTablaEntityRelations.sql</t>
   </si>
   <si>
-    <t>32-InsertMenuEntities.sql</t>
+    <t>32-InsertContadoresTablaEntities.sql</t>
   </si>
   <si>
-    <t>33-InsertMenuContactos.sql</t>
+    <t>33-InsertContadoresTablaEntityTypes.sql</t>
   </si>
   <si>
-    <t>34-InsertMenuBillTo.sql</t>
+    <t>34-InsertMenuEntities.sql</t>
   </si>
   <si>
-    <t>35-InsertParametrosLista.sql</t>
+    <t>35-InsertMenuContactos.sql</t>
   </si>
   <si>
-    <t>36-InsertMenuParametrosDocs.sql</t>
+    <t>36-InsertMenuBillTo.sql</t>
   </si>
   <si>
-    <t>37-InsertMenuCatalogosPermisosUsuariosBillTo.sql</t>
+    <t>37-InsertParametrosLista.sql</t>
   </si>
   <si>
-    <t>38-InsertMenuBillToConsigneesMenu.sql</t>
+    <t>38-InsertMenuParametrosDocs.sql</t>
   </si>
   <si>
-    <t>39-InsertMenuFinanciero.sql</t>
+    <t>39-InsertMenuCatalogosPermisosUsuariosBillTo.sql</t>
   </si>
   <si>
-    <t>40-InsertMenuConsignee.sql</t>
+    <t>40-InsertMenuBillToConsigneesMenu.sql</t>
   </si>
   <si>
-    <t>41-InsertTipoCodigo.sql</t>
+    <t>41-InsertMenuFinanciero.sql</t>
   </si>
   <si>
-    <t>42-InsertCatalogosUserRoles.sql</t>
+    <t>42-InsertMenuConsignee.sql</t>
   </si>
   <si>
-    <t>43-InsertCatalogosIdentificationsAndConsigneeAttributes.sql</t>
+    <t>43-InsertTipoCodigo.sql</t>
   </si>
   <si>
-    <t>44-InsertCliente.sql</t>
+    <t>44-InsertCatalogosUserRoles.sql</t>
   </si>
   <si>
-    <t>45-UpdateOpcionesRetraso.sql</t>
+    <t>45-InsertCatalogosIdentificationsAndConsigneeAttributes.sql</t>
+  </si>
+  <si>
+    <t>46-InsertCliente.sql</t>
+  </si>
+  <si>
+    <t>47-UpdateOpcionesRetraso.sql</t>
+  </si>
+  <si>
+    <t>48-DataValidationEntitiesAUX.sql</t>
+  </si>
+  <si>
+    <t>49-DataMigrationEntities.sql</t>
+  </si>
+  <si>
+    <t>50-HomologacionAgentesCliente.sql</t>
   </si>
 </sst>
 </file>
@@ -861,7 +876,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="68">
+  <borders count="73">
     <border>
       <left/>
       <right/>
@@ -1720,12 +1735,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="155">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1874,6 +1940,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="59" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="60" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1924,93 +2065,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="45" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="46" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="48" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="59" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="60" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2109,6 +2163,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2250,11 +2325,11 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp126.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="20" val="17"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="6"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp127.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="20" val="14"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="6"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp128.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2262,7 +2337,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp129.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="11" val="7"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="20" val="17"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp13.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2282,7 +2357,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp133.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="11" val="10"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="20" val="17"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp134.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2294,11 +2369,11 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp136.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="1" val="0"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="11" val="8"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp137.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="1" val="0"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="11" val="9"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp138.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2326,19 +2401,39 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp143.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="1" val="0"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp144.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="1" val="0"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp145.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
 </file>
 
-<file path=xl/ctrlProps/ctrlProp144.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
+<file path=xl/ctrlProps/ctrlProp146.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
 </file>
 
-<file path=xl/ctrlProps/ctrlProp145.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ctrlProps/ctrlProp147.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp148.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp149.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp15.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$18" noThreeD="1" sel="14" val="7"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp150.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp16.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10971,6 +11066,296 @@
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
                   <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000F6040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:noFill/>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>30480</xdr:colOff>
+          <xdr:row>70</xdr:row>
+          <xdr:rowOff>22860</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>1440180</xdr:colOff>
+          <xdr:row>70</xdr:row>
+          <xdr:rowOff>251460</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1271" name="Drop Down 247" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1271"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27DCAE7F-DA4F-E930-F2FA-7FB030F6CB5C}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:noFill/>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>30480</xdr:colOff>
+          <xdr:row>71</xdr:row>
+          <xdr:rowOff>22860</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>1440180</xdr:colOff>
+          <xdr:row>71</xdr:row>
+          <xdr:rowOff>251460</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1272" name="Drop Down 248" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1272"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{22019F6F-F4A4-A302-E89A-BD2F656B187A}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:noFill/>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>30480</xdr:colOff>
+          <xdr:row>72</xdr:row>
+          <xdr:rowOff>22860</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>1440180</xdr:colOff>
+          <xdr:row>72</xdr:row>
+          <xdr:rowOff>251460</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1273" name="Drop Down 249" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1273"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D0B409B-B897-EE6D-A6A1-2EDCF7DCF9F7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:noFill/>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>30480</xdr:colOff>
+          <xdr:row>73</xdr:row>
+          <xdr:rowOff>22860</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>1440180</xdr:colOff>
+          <xdr:row>73</xdr:row>
+          <xdr:rowOff>251460</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1274" name="Drop Down 250" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1274"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F734C03D-9E90-E8AD-5AA4-618DD6316207}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:noFill/>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>30480</xdr:colOff>
+          <xdr:row>74</xdr:row>
+          <xdr:rowOff>22860</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>1440180</xdr:colOff>
+          <xdr:row>74</xdr:row>
+          <xdr:rowOff>251460</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1275" name="Drop Down 251" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1275"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E80048C-0D2D-6C6B-A45B-027F9609DA30}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -11596,7 +11981,7 @@
   <sheetPr codeName="Hoja1">
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="A2:P72"/>
+  <dimension ref="A2:P75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.44140625" bestFit="1" customWidth="1"/>
@@ -11616,44 +12001,44 @@
   <sheetData>
     <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:16" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="80" t="s">
+      <c r="A3" s="105" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="81"/>
-      <c r="C3" s="81"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="81"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="81"/>
-      <c r="O3" s="76" t="s">
+      <c r="B3" s="106"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="106"/>
+      <c r="E3" s="106"/>
+      <c r="F3" s="106"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="106"/>
+      <c r="J3" s="106"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="106"/>
+      <c r="M3" s="106"/>
+      <c r="O3" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="P3" s="77"/>
+      <c r="P3" s="102"/>
     </row>
     <row r="4" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="85" t="s">
+      <c r="B4" s="110" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="86"/>
-      <c r="D4" s="86"/>
-      <c r="E4" s="86"/>
-      <c r="F4" s="86"/>
-      <c r="G4" s="86"/>
-      <c r="H4" s="86"/>
-      <c r="I4" s="86"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="87"/>
+      <c r="C4" s="111"/>
+      <c r="D4" s="111"/>
+      <c r="E4" s="111"/>
+      <c r="F4" s="111"/>
+      <c r="G4" s="111"/>
+      <c r="H4" s="111"/>
+      <c r="I4" s="111"/>
+      <c r="J4" s="112"/>
+      <c r="K4" s="112"/>
+      <c r="L4" s="112"/>
+      <c r="M4" s="112"/>
       <c r="O4" s="20" t="s">
         <v>2</v>
       </c>
@@ -11663,20 +12048,20 @@
       <c r="A5" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="88" t="s">
+      <c r="B5" s="113" t="s">
         <v>113</v>
       </c>
-      <c r="C5" s="88"/>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
-      <c r="K5" s="89"/>
-      <c r="L5" s="89"/>
-      <c r="M5" s="89"/>
+      <c r="C5" s="113"/>
+      <c r="D5" s="113"/>
+      <c r="E5" s="113"/>
+      <c r="F5" s="113"/>
+      <c r="G5" s="113"/>
+      <c r="H5" s="113"/>
+      <c r="I5" s="113"/>
+      <c r="J5" s="114"/>
+      <c r="K5" s="114"/>
+      <c r="L5" s="114"/>
+      <c r="M5" s="114"/>
       <c r="O5" s="14" t="s">
         <v>4</v>
       </c>
@@ -11686,20 +12071,20 @@
       <c r="A6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="78">
+      <c r="B6" s="103">
         <v>45974</v>
       </c>
-      <c r="C6" s="79"/>
-      <c r="D6" s="79"/>
-      <c r="E6" s="79"/>
-      <c r="F6" s="79"/>
-      <c r="G6" s="79"/>
-      <c r="H6" s="79"/>
-      <c r="I6" s="79"/>
-      <c r="J6" s="79"/>
-      <c r="K6" s="79"/>
-      <c r="L6" s="79"/>
-      <c r="M6" s="79"/>
+      <c r="C6" s="104"/>
+      <c r="D6" s="104"/>
+      <c r="E6" s="104"/>
+      <c r="F6" s="104"/>
+      <c r="G6" s="104"/>
+      <c r="H6" s="104"/>
+      <c r="I6" s="104"/>
+      <c r="J6" s="104"/>
+      <c r="K6" s="104"/>
+      <c r="L6" s="104"/>
+      <c r="M6" s="104"/>
       <c r="O6" s="13"/>
       <c r="P6" s="13"/>
     </row>
@@ -11707,18 +12092,18 @@
       <c r="A7" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="90"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="92"/>
-      <c r="K7" s="92"/>
-      <c r="L7" s="92"/>
-      <c r="M7" s="92"/>
+      <c r="B7" s="115"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
+      <c r="H7" s="116"/>
+      <c r="I7" s="116"/>
+      <c r="J7" s="117"/>
+      <c r="K7" s="117"/>
+      <c r="L7" s="117"/>
+      <c r="M7" s="117"/>
     </row>
     <row r="8" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11"/>
@@ -11736,21 +12121,21 @@
       <c r="M8" s="12"/>
     </row>
     <row r="9" spans="1:16" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="82" t="s">
+      <c r="A9" s="107" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="83"/>
-      <c r="C9" s="83"/>
-      <c r="D9" s="83"/>
-      <c r="E9" s="83"/>
-      <c r="F9" s="83"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="83"/>
-      <c r="I9" s="83"/>
-      <c r="J9" s="84"/>
-      <c r="K9" s="84"/>
-      <c r="L9" s="84"/>
-      <c r="M9" s="84"/>
+      <c r="B9" s="108"/>
+      <c r="C9" s="108"/>
+      <c r="D9" s="108"/>
+      <c r="E9" s="108"/>
+      <c r="F9" s="108"/>
+      <c r="G9" s="108"/>
+      <c r="H9" s="108"/>
+      <c r="I9" s="108"/>
+      <c r="J9" s="109"/>
+      <c r="K9" s="109"/>
+      <c r="L9" s="109"/>
+      <c r="M9" s="109"/>
     </row>
     <row r="10" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -11851,67 +12236,67 @@
       <c r="A14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="106"/>
-      <c r="C14" s="107"/>
-      <c r="D14" s="107"/>
-      <c r="E14" s="107"/>
-      <c r="F14" s="107"/>
-      <c r="G14" s="107"/>
-      <c r="H14" s="107"/>
-      <c r="I14" s="107"/>
-      <c r="J14" s="107"/>
-      <c r="K14" s="107"/>
-      <c r="L14" s="107"/>
-      <c r="M14" s="107"/>
+      <c r="B14" s="85"/>
+      <c r="C14" s="86"/>
+      <c r="D14" s="86"/>
+      <c r="E14" s="86"/>
+      <c r="F14" s="86"/>
+      <c r="G14" s="86"/>
+      <c r="H14" s="86"/>
+      <c r="I14" s="86"/>
+      <c r="J14" s="86"/>
+      <c r="K14" s="86"/>
+      <c r="L14" s="86"/>
+      <c r="M14" s="86"/>
     </row>
     <row r="15" spans="1:16" s="75" customFormat="1" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="106"/>
-      <c r="C15" s="107"/>
-      <c r="D15" s="107"/>
-      <c r="E15" s="107"/>
-      <c r="F15" s="107"/>
-      <c r="G15" s="107"/>
-      <c r="H15" s="107"/>
-      <c r="I15" s="107"/>
-      <c r="J15" s="107"/>
-      <c r="K15" s="107"/>
-      <c r="L15" s="107"/>
-      <c r="M15" s="107"/>
+      <c r="B15" s="85"/>
+      <c r="C15" s="86"/>
+      <c r="D15" s="86"/>
+      <c r="E15" s="86"/>
+      <c r="F15" s="86"/>
+      <c r="G15" s="86"/>
+      <c r="H15" s="86"/>
+      <c r="I15" s="86"/>
+      <c r="J15" s="86"/>
+      <c r="K15" s="86"/>
+      <c r="L15" s="86"/>
+      <c r="M15" s="86"/>
     </row>
     <row r="16" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="97"/>
-      <c r="B16" s="98"/>
-      <c r="C16" s="98"/>
-      <c r="D16" s="98"/>
-      <c r="E16" s="98"/>
-      <c r="F16" s="98"/>
-      <c r="G16" s="98"/>
-      <c r="H16" s="98"/>
-      <c r="I16" s="98"/>
-      <c r="J16" s="98"/>
-      <c r="K16" s="98"/>
-      <c r="L16" s="98"/>
-      <c r="M16" s="98"/>
+      <c r="A16" s="80"/>
+      <c r="B16" s="81"/>
+      <c r="C16" s="81"/>
+      <c r="D16" s="81"/>
+      <c r="E16" s="81"/>
+      <c r="F16" s="81"/>
+      <c r="G16" s="81"/>
+      <c r="H16" s="81"/>
+      <c r="I16" s="81"/>
+      <c r="J16" s="81"/>
+      <c r="K16" s="81"/>
+      <c r="L16" s="81"/>
+      <c r="M16" s="81"/>
     </row>
     <row r="17" spans="1:13" s="5" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="99" t="s">
+      <c r="A17" s="82" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="100"/>
-      <c r="C17" s="100"/>
-      <c r="D17" s="100"/>
-      <c r="E17" s="100"/>
-      <c r="F17" s="100"/>
-      <c r="G17" s="100"/>
-      <c r="H17" s="100"/>
-      <c r="I17" s="100"/>
-      <c r="J17" s="101"/>
-      <c r="K17" s="101"/>
-      <c r="L17" s="101"/>
-      <c r="M17" s="101"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="83"/>
+      <c r="E17" s="83"/>
+      <c r="F17" s="83"/>
+      <c r="G17" s="83"/>
+      <c r="H17" s="83"/>
+      <c r="I17" s="83"/>
+      <c r="J17" s="84"/>
+      <c r="K17" s="84"/>
+      <c r="L17" s="84"/>
+      <c r="M17" s="84"/>
     </row>
     <row r="18" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
@@ -11921,18 +12306,18 @@
       <c r="C18" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="108" t="s">
+      <c r="D18" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="110"/>
-      <c r="F18" s="110"/>
-      <c r="G18" s="110"/>
-      <c r="H18" s="110"/>
-      <c r="I18" s="110"/>
-      <c r="J18" s="111"/>
-      <c r="K18" s="111"/>
-      <c r="L18" s="111"/>
-      <c r="M18" s="111"/>
+      <c r="E18" s="89"/>
+      <c r="F18" s="89"/>
+      <c r="G18" s="89"/>
+      <c r="H18" s="89"/>
+      <c r="I18" s="89"/>
+      <c r="J18" s="90"/>
+      <c r="K18" s="90"/>
+      <c r="L18" s="90"/>
+      <c r="M18" s="90"/>
     </row>
     <row r="19" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
@@ -11942,16 +12327,16 @@
         <v>103</v>
       </c>
       <c r="C19" s="43"/>
-      <c r="D19" s="109"/>
-      <c r="E19" s="112"/>
-      <c r="F19" s="112"/>
-      <c r="G19" s="112"/>
-      <c r="H19" s="112"/>
-      <c r="I19" s="112"/>
-      <c r="J19" s="113"/>
-      <c r="K19" s="113"/>
-      <c r="L19" s="113"/>
-      <c r="M19" s="113"/>
+      <c r="D19" s="88"/>
+      <c r="E19" s="91"/>
+      <c r="F19" s="91"/>
+      <c r="G19" s="91"/>
+      <c r="H19" s="91"/>
+      <c r="I19" s="91"/>
+      <c r="J19" s="92"/>
+      <c r="K19" s="92"/>
+      <c r="L19" s="92"/>
+      <c r="M19" s="92"/>
     </row>
     <row r="20" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
@@ -11961,16 +12346,16 @@
         <v>103</v>
       </c>
       <c r="C20" s="43"/>
-      <c r="D20" s="109"/>
-      <c r="E20" s="112"/>
-      <c r="F20" s="112"/>
-      <c r="G20" s="112"/>
-      <c r="H20" s="112"/>
-      <c r="I20" s="112"/>
-      <c r="J20" s="113"/>
-      <c r="K20" s="113"/>
-      <c r="L20" s="113"/>
-      <c r="M20" s="113"/>
+      <c r="D20" s="88"/>
+      <c r="E20" s="91"/>
+      <c r="F20" s="91"/>
+      <c r="G20" s="91"/>
+      <c r="H20" s="91"/>
+      <c r="I20" s="91"/>
+      <c r="J20" s="92"/>
+      <c r="K20" s="92"/>
+      <c r="L20" s="92"/>
+      <c r="M20" s="92"/>
     </row>
     <row r="21" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -11980,20 +12365,20 @@
         <v>103</v>
       </c>
       <c r="C21" s="43"/>
-      <c r="D21" s="120" t="s">
+      <c r="D21" s="99" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="93" t="s">
+      <c r="E21" s="76" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="94"/>
-      <c r="G21" s="94"/>
-      <c r="H21" s="94"/>
-      <c r="I21" s="94"/>
-      <c r="J21" s="94"/>
-      <c r="K21" s="94"/>
-      <c r="L21" s="94"/>
-      <c r="M21" s="94"/>
+      <c r="F21" s="77"/>
+      <c r="G21" s="77"/>
+      <c r="H21" s="77"/>
+      <c r="I21" s="77"/>
+      <c r="J21" s="77"/>
+      <c r="K21" s="77"/>
+      <c r="L21" s="77"/>
+      <c r="M21" s="77"/>
     </row>
     <row r="22" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
@@ -12003,48 +12388,48 @@
       <c r="C22" s="43" t="s">
         <v>103</v>
       </c>
-      <c r="D22" s="121"/>
-      <c r="E22" s="95"/>
-      <c r="F22" s="96"/>
-      <c r="G22" s="96"/>
-      <c r="H22" s="96"/>
-      <c r="I22" s="96"/>
-      <c r="J22" s="96"/>
-      <c r="K22" s="96"/>
-      <c r="L22" s="96"/>
-      <c r="M22" s="96"/>
+      <c r="D22" s="100"/>
+      <c r="E22" s="78"/>
+      <c r="F22" s="79"/>
+      <c r="G22" s="79"/>
+      <c r="H22" s="79"/>
+      <c r="I22" s="79"/>
+      <c r="J22" s="79"/>
+      <c r="K22" s="79"/>
+      <c r="L22" s="79"/>
+      <c r="M22" s="79"/>
     </row>
     <row r="23" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="115"/>
-      <c r="B23" s="116"/>
-      <c r="C23" s="116"/>
-      <c r="D23" s="117"/>
-      <c r="E23" s="117"/>
-      <c r="F23" s="117"/>
-      <c r="G23" s="117"/>
-      <c r="H23" s="117"/>
-      <c r="I23" s="117"/>
-      <c r="J23" s="117"/>
-      <c r="K23" s="117"/>
-      <c r="L23" s="117"/>
-      <c r="M23" s="117"/>
+      <c r="A23" s="94"/>
+      <c r="B23" s="95"/>
+      <c r="C23" s="95"/>
+      <c r="D23" s="96"/>
+      <c r="E23" s="96"/>
+      <c r="F23" s="96"/>
+      <c r="G23" s="96"/>
+      <c r="H23" s="96"/>
+      <c r="I23" s="96"/>
+      <c r="J23" s="96"/>
+      <c r="K23" s="96"/>
+      <c r="L23" s="96"/>
+      <c r="M23" s="96"/>
     </row>
     <row r="24" spans="1:13" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="118" t="s">
+      <c r="A24" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="119"/>
-      <c r="C24" s="119"/>
-      <c r="D24" s="119"/>
-      <c r="E24" s="119"/>
-      <c r="F24" s="119"/>
-      <c r="G24" s="119"/>
-      <c r="H24" s="119"/>
-      <c r="I24" s="119"/>
-      <c r="J24" s="119"/>
-      <c r="K24" s="119"/>
-      <c r="L24" s="119"/>
-      <c r="M24" s="119"/>
+      <c r="B24" s="98"/>
+      <c r="C24" s="98"/>
+      <c r="D24" s="98"/>
+      <c r="E24" s="98"/>
+      <c r="F24" s="98"/>
+      <c r="G24" s="98"/>
+      <c r="H24" s="98"/>
+      <c r="I24" s="98"/>
+      <c r="J24" s="98"/>
+      <c r="K24" s="98"/>
+      <c r="L24" s="98"/>
+      <c r="M24" s="98"/>
     </row>
     <row r="25" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="15" t="s">
@@ -12056,18 +12441,18 @@
       <c r="C25" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="114" t="s">
+      <c r="D25" s="93" t="s">
         <v>37</v>
       </c>
-      <c r="E25" s="114"/>
-      <c r="F25" s="114"/>
-      <c r="G25" s="114"/>
-      <c r="H25" s="114"/>
-      <c r="I25" s="114"/>
-      <c r="J25" s="114"/>
-      <c r="K25" s="114"/>
-      <c r="L25" s="114"/>
-      <c r="M25" s="114"/>
+      <c r="E25" s="93"/>
+      <c r="F25" s="93"/>
+      <c r="G25" s="93"/>
+      <c r="H25" s="93"/>
+      <c r="I25" s="93"/>
+      <c r="J25" s="93"/>
+      <c r="K25" s="93"/>
+      <c r="L25" s="93"/>
+      <c r="M25" s="93"/>
     </row>
     <row r="26" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="32">
@@ -12077,18 +12462,18 @@
         <v>115</v>
       </c>
       <c r="C26" s="33"/>
-      <c r="D26" s="102" t="s">
+      <c r="D26" s="76" t="s">
         <v>111</v>
       </c>
-      <c r="E26" s="103"/>
-      <c r="F26" s="103"/>
-      <c r="G26" s="103"/>
-      <c r="H26" s="103"/>
-      <c r="I26" s="103"/>
-      <c r="J26" s="103"/>
-      <c r="K26" s="103"/>
-      <c r="L26" s="103"/>
-      <c r="M26" s="103"/>
+      <c r="E26" s="77"/>
+      <c r="F26" s="77"/>
+      <c r="G26" s="77"/>
+      <c r="H26" s="77"/>
+      <c r="I26" s="77"/>
+      <c r="J26" s="77"/>
+      <c r="K26" s="77"/>
+      <c r="L26" s="77"/>
+      <c r="M26" s="151"/>
     </row>
     <row r="27" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="32">
@@ -12098,16 +12483,16 @@
         <v>116</v>
       </c>
       <c r="C27" s="33"/>
-      <c r="D27" s="104"/>
-      <c r="E27" s="105"/>
-      <c r="F27" s="105"/>
-      <c r="G27" s="105"/>
-      <c r="H27" s="105"/>
-      <c r="I27" s="105"/>
-      <c r="J27" s="105"/>
-      <c r="K27" s="105"/>
-      <c r="L27" s="105"/>
-      <c r="M27" s="105"/>
+      <c r="D27" s="152"/>
+      <c r="E27" s="153"/>
+      <c r="F27" s="153"/>
+      <c r="G27" s="153"/>
+      <c r="H27" s="153"/>
+      <c r="I27" s="153"/>
+      <c r="J27" s="153"/>
+      <c r="K27" s="153"/>
+      <c r="L27" s="153"/>
+      <c r="M27" s="154"/>
     </row>
     <row r="28" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="32">
@@ -12117,16 +12502,16 @@
         <v>117</v>
       </c>
       <c r="C28" s="33"/>
-      <c r="D28" s="104"/>
-      <c r="E28" s="105"/>
-      <c r="F28" s="105"/>
-      <c r="G28" s="105"/>
-      <c r="H28" s="105"/>
-      <c r="I28" s="105"/>
-      <c r="J28" s="105"/>
-      <c r="K28" s="105"/>
-      <c r="L28" s="105"/>
-      <c r="M28" s="105"/>
+      <c r="D28" s="152"/>
+      <c r="E28" s="153"/>
+      <c r="F28" s="153"/>
+      <c r="G28" s="153"/>
+      <c r="H28" s="153"/>
+      <c r="I28" s="153"/>
+      <c r="J28" s="153"/>
+      <c r="K28" s="153"/>
+      <c r="L28" s="153"/>
+      <c r="M28" s="154"/>
     </row>
     <row r="29" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="32">
@@ -12136,16 +12521,16 @@
         <v>118</v>
       </c>
       <c r="C29" s="33"/>
-      <c r="D29" s="104"/>
-      <c r="E29" s="105"/>
-      <c r="F29" s="105"/>
-      <c r="G29" s="105"/>
-      <c r="H29" s="105"/>
-      <c r="I29" s="105"/>
-      <c r="J29" s="105"/>
-      <c r="K29" s="105"/>
-      <c r="L29" s="105"/>
-      <c r="M29" s="105"/>
+      <c r="D29" s="152"/>
+      <c r="E29" s="153"/>
+      <c r="F29" s="153"/>
+      <c r="G29" s="153"/>
+      <c r="H29" s="153"/>
+      <c r="I29" s="153"/>
+      <c r="J29" s="153"/>
+      <c r="K29" s="153"/>
+      <c r="L29" s="153"/>
+      <c r="M29" s="154"/>
     </row>
     <row r="30" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="32">
@@ -12155,16 +12540,16 @@
         <v>119</v>
       </c>
       <c r="C30" s="33"/>
-      <c r="D30" s="104"/>
-      <c r="E30" s="105"/>
-      <c r="F30" s="105"/>
-      <c r="G30" s="105"/>
-      <c r="H30" s="105"/>
-      <c r="I30" s="105"/>
-      <c r="J30" s="105"/>
-      <c r="K30" s="105"/>
-      <c r="L30" s="105"/>
-      <c r="M30" s="105"/>
+      <c r="D30" s="152"/>
+      <c r="E30" s="153"/>
+      <c r="F30" s="153"/>
+      <c r="G30" s="153"/>
+      <c r="H30" s="153"/>
+      <c r="I30" s="153"/>
+      <c r="J30" s="153"/>
+      <c r="K30" s="153"/>
+      <c r="L30" s="153"/>
+      <c r="M30" s="154"/>
     </row>
     <row r="31" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="32">
@@ -12174,16 +12559,16 @@
         <v>120</v>
       </c>
       <c r="C31" s="33"/>
-      <c r="D31" s="104"/>
-      <c r="E31" s="105"/>
-      <c r="F31" s="105"/>
-      <c r="G31" s="105"/>
-      <c r="H31" s="105"/>
-      <c r="I31" s="105"/>
-      <c r="J31" s="105"/>
-      <c r="K31" s="105"/>
-      <c r="L31" s="105"/>
-      <c r="M31" s="105"/>
+      <c r="D31" s="152"/>
+      <c r="E31" s="153"/>
+      <c r="F31" s="153"/>
+      <c r="G31" s="153"/>
+      <c r="H31" s="153"/>
+      <c r="I31" s="153"/>
+      <c r="J31" s="153"/>
+      <c r="K31" s="153"/>
+      <c r="L31" s="153"/>
+      <c r="M31" s="154"/>
     </row>
     <row r="32" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="32">
@@ -12193,16 +12578,16 @@
         <v>121</v>
       </c>
       <c r="C32" s="33"/>
-      <c r="D32" s="104"/>
-      <c r="E32" s="105"/>
-      <c r="F32" s="105"/>
-      <c r="G32" s="105"/>
-      <c r="H32" s="105"/>
-      <c r="I32" s="105"/>
-      <c r="J32" s="105"/>
-      <c r="K32" s="105"/>
-      <c r="L32" s="105"/>
-      <c r="M32" s="105"/>
+      <c r="D32" s="152"/>
+      <c r="E32" s="153"/>
+      <c r="F32" s="153"/>
+      <c r="G32" s="153"/>
+      <c r="H32" s="153"/>
+      <c r="I32" s="153"/>
+      <c r="J32" s="153"/>
+      <c r="K32" s="153"/>
+      <c r="L32" s="153"/>
+      <c r="M32" s="154"/>
     </row>
     <row r="33" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="32">
@@ -12212,16 +12597,16 @@
         <v>122</v>
       </c>
       <c r="C33" s="33"/>
-      <c r="D33" s="104"/>
-      <c r="E33" s="105"/>
-      <c r="F33" s="105"/>
-      <c r="G33" s="105"/>
-      <c r="H33" s="105"/>
-      <c r="I33" s="105"/>
-      <c r="J33" s="105"/>
-      <c r="K33" s="105"/>
-      <c r="L33" s="105"/>
-      <c r="M33" s="105"/>
+      <c r="D33" s="152"/>
+      <c r="E33" s="153"/>
+      <c r="F33" s="153"/>
+      <c r="G33" s="153"/>
+      <c r="H33" s="153"/>
+      <c r="I33" s="153"/>
+      <c r="J33" s="153"/>
+      <c r="K33" s="153"/>
+      <c r="L33" s="153"/>
+      <c r="M33" s="154"/>
     </row>
     <row r="34" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="32">
@@ -12230,17 +12615,17 @@
       <c r="B34" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="C34" s="32"/>
-      <c r="D34" s="104"/>
-      <c r="E34" s="105"/>
-      <c r="F34" s="105"/>
-      <c r="G34" s="105"/>
-      <c r="H34" s="105"/>
-      <c r="I34" s="105"/>
-      <c r="J34" s="105"/>
-      <c r="K34" s="105"/>
-      <c r="L34" s="105"/>
-      <c r="M34" s="105"/>
+      <c r="C34" s="33"/>
+      <c r="D34" s="152"/>
+      <c r="E34" s="153"/>
+      <c r="F34" s="153"/>
+      <c r="G34" s="153"/>
+      <c r="H34" s="153"/>
+      <c r="I34" s="153"/>
+      <c r="J34" s="153"/>
+      <c r="K34" s="153"/>
+      <c r="L34" s="153"/>
+      <c r="M34" s="154"/>
     </row>
     <row r="35" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="32">
@@ -12249,17 +12634,17 @@
       <c r="B35" s="33" t="s">
         <v>124</v>
       </c>
-      <c r="C35" s="32"/>
-      <c r="D35" s="104"/>
-      <c r="E35" s="105"/>
-      <c r="F35" s="105"/>
-      <c r="G35" s="105"/>
-      <c r="H35" s="105"/>
-      <c r="I35" s="105"/>
-      <c r="J35" s="105"/>
-      <c r="K35" s="105"/>
-      <c r="L35" s="105"/>
-      <c r="M35" s="105"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="152"/>
+      <c r="E35" s="153"/>
+      <c r="F35" s="153"/>
+      <c r="G35" s="153"/>
+      <c r="H35" s="153"/>
+      <c r="I35" s="153"/>
+      <c r="J35" s="153"/>
+      <c r="K35" s="153"/>
+      <c r="L35" s="153"/>
+      <c r="M35" s="154"/>
     </row>
     <row r="36" spans="1:13" ht="18.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="32">
@@ -12268,17 +12653,17 @@
       <c r="B36" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="C36" s="32"/>
-      <c r="D36" s="104"/>
-      <c r="E36" s="105"/>
-      <c r="F36" s="105"/>
-      <c r="G36" s="105"/>
-      <c r="H36" s="105"/>
-      <c r="I36" s="105"/>
-      <c r="J36" s="105"/>
-      <c r="K36" s="105"/>
-      <c r="L36" s="105"/>
-      <c r="M36" s="105"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="152"/>
+      <c r="E36" s="153"/>
+      <c r="F36" s="153"/>
+      <c r="G36" s="153"/>
+      <c r="H36" s="153"/>
+      <c r="I36" s="153"/>
+      <c r="J36" s="153"/>
+      <c r="K36" s="153"/>
+      <c r="L36" s="153"/>
+      <c r="M36" s="154"/>
     </row>
     <row r="37" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="32">
@@ -12287,17 +12672,17 @@
       <c r="B37" s="33" t="s">
         <v>126</v>
       </c>
-      <c r="C37" s="32"/>
-      <c r="D37" s="104"/>
-      <c r="E37" s="105"/>
-      <c r="F37" s="105"/>
-      <c r="G37" s="105"/>
-      <c r="H37" s="105"/>
-      <c r="I37" s="105"/>
-      <c r="J37" s="105"/>
-      <c r="K37" s="105"/>
-      <c r="L37" s="105"/>
-      <c r="M37" s="105"/>
+      <c r="C37" s="33"/>
+      <c r="D37" s="152"/>
+      <c r="E37" s="153"/>
+      <c r="F37" s="153"/>
+      <c r="G37" s="153"/>
+      <c r="H37" s="153"/>
+      <c r="I37" s="153"/>
+      <c r="J37" s="153"/>
+      <c r="K37" s="153"/>
+      <c r="L37" s="153"/>
+      <c r="M37" s="154"/>
     </row>
     <row r="38" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="32">
@@ -12306,17 +12691,17 @@
       <c r="B38" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="C38" s="32"/>
-      <c r="D38" s="104"/>
-      <c r="E38" s="105"/>
-      <c r="F38" s="105"/>
-      <c r="G38" s="105"/>
-      <c r="H38" s="105"/>
-      <c r="I38" s="105"/>
-      <c r="J38" s="105"/>
-      <c r="K38" s="105"/>
-      <c r="L38" s="105"/>
-      <c r="M38" s="105"/>
+      <c r="C38" s="33"/>
+      <c r="D38" s="152"/>
+      <c r="E38" s="153"/>
+      <c r="F38" s="153"/>
+      <c r="G38" s="153"/>
+      <c r="H38" s="153"/>
+      <c r="I38" s="153"/>
+      <c r="J38" s="153"/>
+      <c r="K38" s="153"/>
+      <c r="L38" s="153"/>
+      <c r="M38" s="154"/>
     </row>
     <row r="39" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="32">
@@ -12325,17 +12710,17 @@
       <c r="B39" s="33" t="s">
         <v>128</v>
       </c>
-      <c r="C39" s="32"/>
-      <c r="D39" s="104"/>
-      <c r="E39" s="105"/>
-      <c r="F39" s="105"/>
-      <c r="G39" s="105"/>
-      <c r="H39" s="105"/>
-      <c r="I39" s="105"/>
-      <c r="J39" s="105"/>
-      <c r="K39" s="105"/>
-      <c r="L39" s="105"/>
-      <c r="M39" s="105"/>
+      <c r="C39" s="33"/>
+      <c r="D39" s="152"/>
+      <c r="E39" s="153"/>
+      <c r="F39" s="153"/>
+      <c r="G39" s="153"/>
+      <c r="H39" s="153"/>
+      <c r="I39" s="153"/>
+      <c r="J39" s="153"/>
+      <c r="K39" s="153"/>
+      <c r="L39" s="153"/>
+      <c r="M39" s="154"/>
     </row>
     <row r="40" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="32">
@@ -12344,17 +12729,17 @@
       <c r="B40" s="33" t="s">
         <v>129</v>
       </c>
-      <c r="C40" s="32"/>
-      <c r="D40" s="104"/>
-      <c r="E40" s="105"/>
-      <c r="F40" s="105"/>
-      <c r="G40" s="105"/>
-      <c r="H40" s="105"/>
-      <c r="I40" s="105"/>
-      <c r="J40" s="105"/>
-      <c r="K40" s="105"/>
-      <c r="L40" s="105"/>
-      <c r="M40" s="105"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="152"/>
+      <c r="E40" s="153"/>
+      <c r="F40" s="153"/>
+      <c r="G40" s="153"/>
+      <c r="H40" s="153"/>
+      <c r="I40" s="153"/>
+      <c r="J40" s="153"/>
+      <c r="K40" s="153"/>
+      <c r="L40" s="153"/>
+      <c r="M40" s="154"/>
     </row>
     <row r="41" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="32">
@@ -12363,17 +12748,17 @@
       <c r="B41" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="C41" s="32"/>
-      <c r="D41" s="104"/>
-      <c r="E41" s="105"/>
-      <c r="F41" s="105"/>
-      <c r="G41" s="105"/>
-      <c r="H41" s="105"/>
-      <c r="I41" s="105"/>
-      <c r="J41" s="105"/>
-      <c r="K41" s="105"/>
-      <c r="L41" s="105"/>
-      <c r="M41" s="105"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="152"/>
+      <c r="E41" s="153"/>
+      <c r="F41" s="153"/>
+      <c r="G41" s="153"/>
+      <c r="H41" s="153"/>
+      <c r="I41" s="153"/>
+      <c r="J41" s="153"/>
+      <c r="K41" s="153"/>
+      <c r="L41" s="153"/>
+      <c r="M41" s="154"/>
     </row>
     <row r="42" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="32">
@@ -12382,17 +12767,17 @@
       <c r="B42" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="C42" s="32"/>
-      <c r="D42" s="104"/>
-      <c r="E42" s="105"/>
-      <c r="F42" s="105"/>
-      <c r="G42" s="105"/>
-      <c r="H42" s="105"/>
-      <c r="I42" s="105"/>
-      <c r="J42" s="105"/>
-      <c r="K42" s="105"/>
-      <c r="L42" s="105"/>
-      <c r="M42" s="105"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="152"/>
+      <c r="E42" s="153"/>
+      <c r="F42" s="153"/>
+      <c r="G42" s="153"/>
+      <c r="H42" s="153"/>
+      <c r="I42" s="153"/>
+      <c r="J42" s="153"/>
+      <c r="K42" s="153"/>
+      <c r="L42" s="153"/>
+      <c r="M42" s="154"/>
     </row>
     <row r="43" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="32">
@@ -12401,17 +12786,17 @@
       <c r="B43" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="C43" s="32"/>
-      <c r="D43" s="104"/>
-      <c r="E43" s="105"/>
-      <c r="F43" s="105"/>
-      <c r="G43" s="105"/>
-      <c r="H43" s="105"/>
-      <c r="I43" s="105"/>
-      <c r="J43" s="105"/>
-      <c r="K43" s="105"/>
-      <c r="L43" s="105"/>
-      <c r="M43" s="105"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="152"/>
+      <c r="E43" s="153"/>
+      <c r="F43" s="153"/>
+      <c r="G43" s="153"/>
+      <c r="H43" s="153"/>
+      <c r="I43" s="153"/>
+      <c r="J43" s="153"/>
+      <c r="K43" s="153"/>
+      <c r="L43" s="153"/>
+      <c r="M43" s="154"/>
     </row>
     <row r="44" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="32">
@@ -12420,17 +12805,17 @@
       <c r="B44" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="C44" s="32"/>
-      <c r="D44" s="104"/>
-      <c r="E44" s="105"/>
-      <c r="F44" s="105"/>
-      <c r="G44" s="105"/>
-      <c r="H44" s="105"/>
-      <c r="I44" s="105"/>
-      <c r="J44" s="105"/>
-      <c r="K44" s="105"/>
-      <c r="L44" s="105"/>
-      <c r="M44" s="105"/>
+      <c r="C44" s="33"/>
+      <c r="D44" s="152"/>
+      <c r="E44" s="153"/>
+      <c r="F44" s="153"/>
+      <c r="G44" s="153"/>
+      <c r="H44" s="153"/>
+      <c r="I44" s="153"/>
+      <c r="J44" s="153"/>
+      <c r="K44" s="153"/>
+      <c r="L44" s="153"/>
+      <c r="M44" s="154"/>
     </row>
     <row r="45" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="32">
@@ -12439,17 +12824,17 @@
       <c r="B45" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="C45" s="32"/>
-      <c r="D45" s="104"/>
-      <c r="E45" s="105"/>
-      <c r="F45" s="105"/>
-      <c r="G45" s="105"/>
-      <c r="H45" s="105"/>
-      <c r="I45" s="105"/>
-      <c r="J45" s="105"/>
-      <c r="K45" s="105"/>
-      <c r="L45" s="105"/>
-      <c r="M45" s="105"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="152"/>
+      <c r="E45" s="153"/>
+      <c r="F45" s="153"/>
+      <c r="G45" s="153"/>
+      <c r="H45" s="153"/>
+      <c r="I45" s="153"/>
+      <c r="J45" s="153"/>
+      <c r="K45" s="153"/>
+      <c r="L45" s="153"/>
+      <c r="M45" s="154"/>
     </row>
     <row r="46" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="32">
@@ -12458,17 +12843,17 @@
       <c r="B46" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="C46" s="32"/>
-      <c r="D46" s="104"/>
-      <c r="E46" s="105"/>
-      <c r="F46" s="105"/>
-      <c r="G46" s="105"/>
-      <c r="H46" s="105"/>
-      <c r="I46" s="105"/>
-      <c r="J46" s="105"/>
-      <c r="K46" s="105"/>
-      <c r="L46" s="105"/>
-      <c r="M46" s="105"/>
+      <c r="C46" s="33"/>
+      <c r="D46" s="152"/>
+      <c r="E46" s="153"/>
+      <c r="F46" s="153"/>
+      <c r="G46" s="153"/>
+      <c r="H46" s="153"/>
+      <c r="I46" s="153"/>
+      <c r="J46" s="153"/>
+      <c r="K46" s="153"/>
+      <c r="L46" s="153"/>
+      <c r="M46" s="154"/>
     </row>
     <row r="47" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="32">
@@ -12477,17 +12862,17 @@
       <c r="B47" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="C47" s="32"/>
-      <c r="D47" s="104"/>
-      <c r="E47" s="105"/>
-      <c r="F47" s="105"/>
-      <c r="G47" s="105"/>
-      <c r="H47" s="105"/>
-      <c r="I47" s="105"/>
-      <c r="J47" s="105"/>
-      <c r="K47" s="105"/>
-      <c r="L47" s="105"/>
-      <c r="M47" s="105"/>
+      <c r="C47" s="33"/>
+      <c r="D47" s="152"/>
+      <c r="E47" s="153"/>
+      <c r="F47" s="153"/>
+      <c r="G47" s="153"/>
+      <c r="H47" s="153"/>
+      <c r="I47" s="153"/>
+      <c r="J47" s="153"/>
+      <c r="K47" s="153"/>
+      <c r="L47" s="153"/>
+      <c r="M47" s="154"/>
     </row>
     <row r="48" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="32">
@@ -12496,17 +12881,17 @@
       <c r="B48" s="33" t="s">
         <v>137</v>
       </c>
-      <c r="C48" s="32"/>
-      <c r="D48" s="104"/>
-      <c r="E48" s="105"/>
-      <c r="F48" s="105"/>
-      <c r="G48" s="105"/>
-      <c r="H48" s="105"/>
-      <c r="I48" s="105"/>
-      <c r="J48" s="105"/>
-      <c r="K48" s="105"/>
-      <c r="L48" s="105"/>
-      <c r="M48" s="105"/>
+      <c r="C48" s="33"/>
+      <c r="D48" s="152"/>
+      <c r="E48" s="153"/>
+      <c r="F48" s="153"/>
+      <c r="G48" s="153"/>
+      <c r="H48" s="153"/>
+      <c r="I48" s="153"/>
+      <c r="J48" s="153"/>
+      <c r="K48" s="153"/>
+      <c r="L48" s="153"/>
+      <c r="M48" s="154"/>
     </row>
     <row r="49" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="32">
@@ -12515,17 +12900,17 @@
       <c r="B49" s="33" t="s">
         <v>138</v>
       </c>
-      <c r="C49" s="32"/>
-      <c r="D49" s="104"/>
-      <c r="E49" s="105"/>
-      <c r="F49" s="105"/>
-      <c r="G49" s="105"/>
-      <c r="H49" s="105"/>
-      <c r="I49" s="105"/>
-      <c r="J49" s="105"/>
-      <c r="K49" s="105"/>
-      <c r="L49" s="105"/>
-      <c r="M49" s="105"/>
+      <c r="C49" s="33"/>
+      <c r="D49" s="152"/>
+      <c r="E49" s="153"/>
+      <c r="F49" s="153"/>
+      <c r="G49" s="153"/>
+      <c r="H49" s="153"/>
+      <c r="I49" s="153"/>
+      <c r="J49" s="153"/>
+      <c r="K49" s="153"/>
+      <c r="L49" s="153"/>
+      <c r="M49" s="154"/>
     </row>
     <row r="50" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="32">
@@ -12534,17 +12919,17 @@
       <c r="B50" s="33" t="s">
         <v>139</v>
       </c>
-      <c r="C50" s="32"/>
-      <c r="D50" s="104"/>
-      <c r="E50" s="105"/>
-      <c r="F50" s="105"/>
-      <c r="G50" s="105"/>
-      <c r="H50" s="105"/>
-      <c r="I50" s="105"/>
-      <c r="J50" s="105"/>
-      <c r="K50" s="105"/>
-      <c r="L50" s="105"/>
-      <c r="M50" s="105"/>
+      <c r="C50" s="33"/>
+      <c r="D50" s="152"/>
+      <c r="E50" s="153"/>
+      <c r="F50" s="153"/>
+      <c r="G50" s="153"/>
+      <c r="H50" s="153"/>
+      <c r="I50" s="153"/>
+      <c r="J50" s="153"/>
+      <c r="K50" s="153"/>
+      <c r="L50" s="153"/>
+      <c r="M50" s="154"/>
     </row>
     <row r="51" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="32">
@@ -12553,17 +12938,17 @@
       <c r="B51" s="33" t="s">
         <v>140</v>
       </c>
-      <c r="C51" s="32"/>
-      <c r="D51" s="104"/>
-      <c r="E51" s="105"/>
-      <c r="F51" s="105"/>
-      <c r="G51" s="105"/>
-      <c r="H51" s="105"/>
-      <c r="I51" s="105"/>
-      <c r="J51" s="105"/>
-      <c r="K51" s="105"/>
-      <c r="L51" s="105"/>
-      <c r="M51" s="105"/>
+      <c r="C51" s="33"/>
+      <c r="D51" s="152"/>
+      <c r="E51" s="153"/>
+      <c r="F51" s="153"/>
+      <c r="G51" s="153"/>
+      <c r="H51" s="153"/>
+      <c r="I51" s="153"/>
+      <c r="J51" s="153"/>
+      <c r="K51" s="153"/>
+      <c r="L51" s="153"/>
+      <c r="M51" s="154"/>
     </row>
     <row r="52" spans="1:13" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="32">
@@ -12572,17 +12957,17 @@
       <c r="B52" s="33" t="s">
         <v>141</v>
       </c>
-      <c r="C52" s="32"/>
-      <c r="D52" s="104"/>
-      <c r="E52" s="105"/>
-      <c r="F52" s="105"/>
-      <c r="G52" s="105"/>
-      <c r="H52" s="105"/>
-      <c r="I52" s="105"/>
-      <c r="J52" s="105"/>
-      <c r="K52" s="105"/>
-      <c r="L52" s="105"/>
-      <c r="M52" s="105"/>
+      <c r="C52" s="33"/>
+      <c r="D52" s="152"/>
+      <c r="E52" s="153"/>
+      <c r="F52" s="153"/>
+      <c r="G52" s="153"/>
+      <c r="H52" s="153"/>
+      <c r="I52" s="153"/>
+      <c r="J52" s="153"/>
+      <c r="K52" s="153"/>
+      <c r="L52" s="153"/>
+      <c r="M52" s="154"/>
     </row>
     <row r="53" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="32">
@@ -12591,17 +12976,17 @@
       <c r="B53" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="C53" s="32"/>
-      <c r="D53" s="104"/>
-      <c r="E53" s="105"/>
-      <c r="F53" s="105"/>
-      <c r="G53" s="105"/>
-      <c r="H53" s="105"/>
-      <c r="I53" s="105"/>
-      <c r="J53" s="105"/>
-      <c r="K53" s="105"/>
-      <c r="L53" s="105"/>
-      <c r="M53" s="105"/>
+      <c r="C53" s="33"/>
+      <c r="D53" s="152"/>
+      <c r="E53" s="153"/>
+      <c r="F53" s="153"/>
+      <c r="G53" s="153"/>
+      <c r="H53" s="153"/>
+      <c r="I53" s="153"/>
+      <c r="J53" s="153"/>
+      <c r="K53" s="153"/>
+      <c r="L53" s="153"/>
+      <c r="M53" s="154"/>
     </row>
     <row r="54" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="32">
@@ -12610,17 +12995,17 @@
       <c r="B54" s="33" t="s">
         <v>143</v>
       </c>
-      <c r="C54" s="32"/>
-      <c r="D54" s="104"/>
-      <c r="E54" s="105"/>
-      <c r="F54" s="105"/>
-      <c r="G54" s="105"/>
-      <c r="H54" s="105"/>
-      <c r="I54" s="105"/>
-      <c r="J54" s="105"/>
-      <c r="K54" s="105"/>
-      <c r="L54" s="105"/>
-      <c r="M54" s="105"/>
+      <c r="C54" s="33"/>
+      <c r="D54" s="152"/>
+      <c r="E54" s="153"/>
+      <c r="F54" s="153"/>
+      <c r="G54" s="153"/>
+      <c r="H54" s="153"/>
+      <c r="I54" s="153"/>
+      <c r="J54" s="153"/>
+      <c r="K54" s="153"/>
+      <c r="L54" s="153"/>
+      <c r="M54" s="154"/>
     </row>
     <row r="55" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="32">
@@ -12629,17 +13014,17 @@
       <c r="B55" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="C55" s="32"/>
-      <c r="D55" s="104"/>
-      <c r="E55" s="105"/>
-      <c r="F55" s="105"/>
-      <c r="G55" s="105"/>
-      <c r="H55" s="105"/>
-      <c r="I55" s="105"/>
-      <c r="J55" s="105"/>
-      <c r="K55" s="105"/>
-      <c r="L55" s="105"/>
-      <c r="M55" s="105"/>
+      <c r="C55" s="33"/>
+      <c r="D55" s="152"/>
+      <c r="E55" s="153"/>
+      <c r="F55" s="153"/>
+      <c r="G55" s="153"/>
+      <c r="H55" s="153"/>
+      <c r="I55" s="153"/>
+      <c r="J55" s="153"/>
+      <c r="K55" s="153"/>
+      <c r="L55" s="153"/>
+      <c r="M55" s="154"/>
     </row>
     <row r="56" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="32">
@@ -12648,17 +13033,17 @@
       <c r="B56" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="C56" s="32"/>
-      <c r="D56" s="104"/>
-      <c r="E56" s="105"/>
-      <c r="F56" s="105"/>
-      <c r="G56" s="105"/>
-      <c r="H56" s="105"/>
-      <c r="I56" s="105"/>
-      <c r="J56" s="105"/>
-      <c r="K56" s="105"/>
-      <c r="L56" s="105"/>
-      <c r="M56" s="105"/>
+      <c r="C56" s="33"/>
+      <c r="D56" s="152"/>
+      <c r="E56" s="153"/>
+      <c r="F56" s="153"/>
+      <c r="G56" s="153"/>
+      <c r="H56" s="153"/>
+      <c r="I56" s="153"/>
+      <c r="J56" s="153"/>
+      <c r="K56" s="153"/>
+      <c r="L56" s="153"/>
+      <c r="M56" s="154"/>
     </row>
     <row r="57" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="32">
@@ -12667,17 +13052,17 @@
       <c r="B57" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="C57" s="32"/>
-      <c r="D57" s="104"/>
-      <c r="E57" s="105"/>
-      <c r="F57" s="105"/>
-      <c r="G57" s="105"/>
-      <c r="H57" s="105"/>
-      <c r="I57" s="105"/>
-      <c r="J57" s="105"/>
-      <c r="K57" s="105"/>
-      <c r="L57" s="105"/>
-      <c r="M57" s="105"/>
+      <c r="C57" s="33"/>
+      <c r="D57" s="152"/>
+      <c r="E57" s="153"/>
+      <c r="F57" s="153"/>
+      <c r="G57" s="153"/>
+      <c r="H57" s="153"/>
+      <c r="I57" s="153"/>
+      <c r="J57" s="153"/>
+      <c r="K57" s="153"/>
+      <c r="L57" s="153"/>
+      <c r="M57" s="154"/>
     </row>
     <row r="58" spans="1:13" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="32">
@@ -12686,17 +13071,17 @@
       <c r="B58" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="C58" s="32"/>
-      <c r="D58" s="104"/>
-      <c r="E58" s="105"/>
-      <c r="F58" s="105"/>
-      <c r="G58" s="105"/>
-      <c r="H58" s="105"/>
-      <c r="I58" s="105"/>
-      <c r="J58" s="105"/>
-      <c r="K58" s="105"/>
-      <c r="L58" s="105"/>
-      <c r="M58" s="105"/>
+      <c r="C58" s="33"/>
+      <c r="D58" s="152"/>
+      <c r="E58" s="153"/>
+      <c r="F58" s="153"/>
+      <c r="G58" s="153"/>
+      <c r="H58" s="153"/>
+      <c r="I58" s="153"/>
+      <c r="J58" s="153"/>
+      <c r="K58" s="153"/>
+      <c r="L58" s="153"/>
+      <c r="M58" s="154"/>
     </row>
     <row r="59" spans="1:13" ht="21.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="32">
@@ -12705,17 +13090,17 @@
       <c r="B59" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="C59" s="32"/>
-      <c r="D59" s="104"/>
-      <c r="E59" s="105"/>
-      <c r="F59" s="105"/>
-      <c r="G59" s="105"/>
-      <c r="H59" s="105"/>
-      <c r="I59" s="105"/>
-      <c r="J59" s="105"/>
-      <c r="K59" s="105"/>
-      <c r="L59" s="105"/>
-      <c r="M59" s="105"/>
+      <c r="C59" s="33"/>
+      <c r="D59" s="152"/>
+      <c r="E59" s="153"/>
+      <c r="F59" s="153"/>
+      <c r="G59" s="153"/>
+      <c r="H59" s="153"/>
+      <c r="I59" s="153"/>
+      <c r="J59" s="153"/>
+      <c r="K59" s="153"/>
+      <c r="L59" s="153"/>
+      <c r="M59" s="154"/>
     </row>
     <row r="60" spans="1:13" ht="21.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="32">
@@ -12724,17 +13109,17 @@
       <c r="B60" s="33" t="s">
         <v>149</v>
       </c>
-      <c r="C60" s="32"/>
-      <c r="D60" s="104"/>
-      <c r="E60" s="105"/>
-      <c r="F60" s="105"/>
-      <c r="G60" s="105"/>
-      <c r="H60" s="105"/>
-      <c r="I60" s="105"/>
-      <c r="J60" s="105"/>
-      <c r="K60" s="105"/>
-      <c r="L60" s="105"/>
-      <c r="M60" s="105"/>
+      <c r="C60" s="33"/>
+      <c r="D60" s="152"/>
+      <c r="E60" s="153"/>
+      <c r="F60" s="153"/>
+      <c r="G60" s="153"/>
+      <c r="H60" s="153"/>
+      <c r="I60" s="153"/>
+      <c r="J60" s="153"/>
+      <c r="K60" s="153"/>
+      <c r="L60" s="153"/>
+      <c r="M60" s="154"/>
     </row>
     <row r="61" spans="1:13" ht="20.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="32">
@@ -12743,17 +13128,17 @@
       <c r="B61" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="C61" s="32"/>
-      <c r="D61" s="104"/>
-      <c r="E61" s="105"/>
-      <c r="F61" s="105"/>
-      <c r="G61" s="105"/>
-      <c r="H61" s="105"/>
-      <c r="I61" s="105"/>
-      <c r="J61" s="105"/>
-      <c r="K61" s="105"/>
-      <c r="L61" s="105"/>
-      <c r="M61" s="105"/>
+      <c r="C61" s="33"/>
+      <c r="D61" s="152"/>
+      <c r="E61" s="153"/>
+      <c r="F61" s="153"/>
+      <c r="G61" s="153"/>
+      <c r="H61" s="153"/>
+      <c r="I61" s="153"/>
+      <c r="J61" s="153"/>
+      <c r="K61" s="153"/>
+      <c r="L61" s="153"/>
+      <c r="M61" s="154"/>
     </row>
     <row r="62" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="32">
@@ -12762,17 +13147,17 @@
       <c r="B62" s="33" t="s">
         <v>151</v>
       </c>
-      <c r="C62" s="32"/>
-      <c r="D62" s="104"/>
-      <c r="E62" s="105"/>
-      <c r="F62" s="105"/>
-      <c r="G62" s="105"/>
-      <c r="H62" s="105"/>
-      <c r="I62" s="105"/>
-      <c r="J62" s="105"/>
-      <c r="K62" s="105"/>
-      <c r="L62" s="105"/>
-      <c r="M62" s="105"/>
+      <c r="C62" s="33"/>
+      <c r="D62" s="152"/>
+      <c r="E62" s="153"/>
+      <c r="F62" s="153"/>
+      <c r="G62" s="153"/>
+      <c r="H62" s="153"/>
+      <c r="I62" s="153"/>
+      <c r="J62" s="153"/>
+      <c r="K62" s="153"/>
+      <c r="L62" s="153"/>
+      <c r="M62" s="154"/>
     </row>
     <row r="63" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="32">
@@ -12781,17 +13166,17 @@
       <c r="B63" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="C63" s="32"/>
-      <c r="D63" s="104"/>
-      <c r="E63" s="105"/>
-      <c r="F63" s="105"/>
-      <c r="G63" s="105"/>
-      <c r="H63" s="105"/>
-      <c r="I63" s="105"/>
-      <c r="J63" s="105"/>
-      <c r="K63" s="105"/>
-      <c r="L63" s="105"/>
-      <c r="M63" s="105"/>
+      <c r="C63" s="33"/>
+      <c r="D63" s="152"/>
+      <c r="E63" s="153"/>
+      <c r="F63" s="153"/>
+      <c r="G63" s="153"/>
+      <c r="H63" s="153"/>
+      <c r="I63" s="153"/>
+      <c r="J63" s="153"/>
+      <c r="K63" s="153"/>
+      <c r="L63" s="153"/>
+      <c r="M63" s="154"/>
     </row>
     <row r="64" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="32">
@@ -12800,17 +13185,17 @@
       <c r="B64" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="C64" s="32"/>
-      <c r="D64" s="104"/>
-      <c r="E64" s="105"/>
-      <c r="F64" s="105"/>
-      <c r="G64" s="105"/>
-      <c r="H64" s="105"/>
-      <c r="I64" s="105"/>
-      <c r="J64" s="105"/>
-      <c r="K64" s="105"/>
-      <c r="L64" s="105"/>
-      <c r="M64" s="105"/>
+      <c r="C64" s="33"/>
+      <c r="D64" s="152"/>
+      <c r="E64" s="153"/>
+      <c r="F64" s="153"/>
+      <c r="G64" s="153"/>
+      <c r="H64" s="153"/>
+      <c r="I64" s="153"/>
+      <c r="J64" s="153"/>
+      <c r="K64" s="153"/>
+      <c r="L64" s="153"/>
+      <c r="M64" s="154"/>
     </row>
     <row r="65" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="32">
@@ -12819,17 +13204,17 @@
       <c r="B65" s="33" t="s">
         <v>154</v>
       </c>
-      <c r="C65" s="32"/>
-      <c r="D65" s="104"/>
-      <c r="E65" s="105"/>
-      <c r="F65" s="105"/>
-      <c r="G65" s="105"/>
-      <c r="H65" s="105"/>
-      <c r="I65" s="105"/>
-      <c r="J65" s="105"/>
-      <c r="K65" s="105"/>
-      <c r="L65" s="105"/>
-      <c r="M65" s="105"/>
+      <c r="C65" s="33"/>
+      <c r="D65" s="152"/>
+      <c r="E65" s="153"/>
+      <c r="F65" s="153"/>
+      <c r="G65" s="153"/>
+      <c r="H65" s="153"/>
+      <c r="I65" s="153"/>
+      <c r="J65" s="153"/>
+      <c r="K65" s="153"/>
+      <c r="L65" s="153"/>
+      <c r="M65" s="154"/>
     </row>
     <row r="66" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="32">
@@ -12838,17 +13223,17 @@
       <c r="B66" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="C66" s="32"/>
-      <c r="D66" s="104"/>
-      <c r="E66" s="105"/>
-      <c r="F66" s="105"/>
-      <c r="G66" s="105"/>
-      <c r="H66" s="105"/>
-      <c r="I66" s="105"/>
-      <c r="J66" s="105"/>
-      <c r="K66" s="105"/>
-      <c r="L66" s="105"/>
-      <c r="M66" s="105"/>
+      <c r="C66" s="33"/>
+      <c r="D66" s="152"/>
+      <c r="E66" s="153"/>
+      <c r="F66" s="153"/>
+      <c r="G66" s="153"/>
+      <c r="H66" s="153"/>
+      <c r="I66" s="153"/>
+      <c r="J66" s="153"/>
+      <c r="K66" s="153"/>
+      <c r="L66" s="153"/>
+      <c r="M66" s="154"/>
     </row>
     <row r="67" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="32">
@@ -12857,17 +13242,17 @@
       <c r="B67" s="33" t="s">
         <v>156</v>
       </c>
-      <c r="C67" s="32"/>
-      <c r="D67" s="104"/>
-      <c r="E67" s="105"/>
-      <c r="F67" s="105"/>
-      <c r="G67" s="105"/>
-      <c r="H67" s="105"/>
-      <c r="I67" s="105"/>
-      <c r="J67" s="105"/>
-      <c r="K67" s="105"/>
-      <c r="L67" s="105"/>
-      <c r="M67" s="105"/>
+      <c r="C67" s="33"/>
+      <c r="D67" s="152"/>
+      <c r="E67" s="153"/>
+      <c r="F67" s="153"/>
+      <c r="G67" s="153"/>
+      <c r="H67" s="153"/>
+      <c r="I67" s="153"/>
+      <c r="J67" s="153"/>
+      <c r="K67" s="153"/>
+      <c r="L67" s="153"/>
+      <c r="M67" s="154"/>
     </row>
     <row r="68" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="32">
@@ -12876,17 +13261,17 @@
       <c r="B68" s="33" t="s">
         <v>157</v>
       </c>
-      <c r="C68" s="32"/>
-      <c r="D68" s="104"/>
-      <c r="E68" s="105"/>
-      <c r="F68" s="105"/>
-      <c r="G68" s="105"/>
-      <c r="H68" s="105"/>
-      <c r="I68" s="105"/>
-      <c r="J68" s="105"/>
-      <c r="K68" s="105"/>
-      <c r="L68" s="105"/>
-      <c r="M68" s="105"/>
+      <c r="C68" s="33"/>
+      <c r="D68" s="152"/>
+      <c r="E68" s="153"/>
+      <c r="F68" s="153"/>
+      <c r="G68" s="153"/>
+      <c r="H68" s="153"/>
+      <c r="I68" s="153"/>
+      <c r="J68" s="153"/>
+      <c r="K68" s="153"/>
+      <c r="L68" s="153"/>
+      <c r="M68" s="154"/>
     </row>
     <row r="69" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="32">
@@ -12895,17 +13280,17 @@
       <c r="B69" s="33" t="s">
         <v>158</v>
       </c>
-      <c r="C69" s="32"/>
-      <c r="D69" s="104"/>
-      <c r="E69" s="105"/>
-      <c r="F69" s="105"/>
-      <c r="G69" s="105"/>
-      <c r="H69" s="105"/>
-      <c r="I69" s="105"/>
-      <c r="J69" s="105"/>
-      <c r="K69" s="105"/>
-      <c r="L69" s="105"/>
-      <c r="M69" s="105"/>
+      <c r="C69" s="33"/>
+      <c r="D69" s="152"/>
+      <c r="E69" s="153"/>
+      <c r="F69" s="153"/>
+      <c r="G69" s="153"/>
+      <c r="H69" s="153"/>
+      <c r="I69" s="153"/>
+      <c r="J69" s="153"/>
+      <c r="K69" s="153"/>
+      <c r="L69" s="153"/>
+      <c r="M69" s="154"/>
     </row>
     <row r="70" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="32">
@@ -12914,54 +13299,125 @@
       <c r="B70" s="33" t="s">
         <v>159</v>
       </c>
-      <c r="C70" s="32"/>
-      <c r="D70" s="104"/>
-      <c r="E70" s="105"/>
-      <c r="F70" s="105"/>
-      <c r="G70" s="105"/>
-      <c r="H70" s="105"/>
-      <c r="I70" s="105"/>
-      <c r="J70" s="105"/>
-      <c r="K70" s="105"/>
-      <c r="L70" s="105"/>
-      <c r="M70" s="105"/>
+      <c r="C70" s="33"/>
+      <c r="D70" s="152"/>
+      <c r="E70" s="153"/>
+      <c r="F70" s="153"/>
+      <c r="G70" s="153"/>
+      <c r="H70" s="153"/>
+      <c r="I70" s="153"/>
+      <c r="J70" s="153"/>
+      <c r="K70" s="153"/>
+      <c r="L70" s="153"/>
+      <c r="M70" s="154"/>
     </row>
     <row r="71" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="32"/>
-      <c r="B71" s="33"/>
-      <c r="C71" s="32"/>
-      <c r="D71" s="104"/>
-      <c r="E71" s="105"/>
-      <c r="F71" s="105"/>
-      <c r="G71" s="105"/>
-      <c r="H71" s="105"/>
-      <c r="I71" s="105"/>
-      <c r="J71" s="105"/>
-      <c r="K71" s="105"/>
-      <c r="L71" s="105"/>
-      <c r="M71" s="105"/>
+      <c r="A71" s="32">
+        <v>46</v>
+      </c>
+      <c r="B71" s="33" t="s">
+        <v>160</v>
+      </c>
+      <c r="C71" s="33"/>
+      <c r="D71" s="152"/>
+      <c r="E71" s="153"/>
+      <c r="F71" s="153"/>
+      <c r="G71" s="153"/>
+      <c r="H71" s="153"/>
+      <c r="I71" s="153"/>
+      <c r="J71" s="153"/>
+      <c r="K71" s="153"/>
+      <c r="L71" s="153"/>
+      <c r="M71" s="154"/>
     </row>
     <row r="72" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="32"/>
-      <c r="B72" s="33"/>
-      <c r="C72" s="32"/>
-      <c r="D72" s="104"/>
-      <c r="E72" s="105"/>
-      <c r="F72" s="105"/>
-      <c r="G72" s="105"/>
-      <c r="H72" s="105"/>
-      <c r="I72" s="105"/>
-      <c r="J72" s="105"/>
-      <c r="K72" s="105"/>
-      <c r="L72" s="105"/>
-      <c r="M72" s="105"/>
+      <c r="A72" s="32">
+        <v>47</v>
+      </c>
+      <c r="B72" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="C72" s="33"/>
+      <c r="D72" s="152"/>
+      <c r="E72" s="153"/>
+      <c r="F72" s="153"/>
+      <c r="G72" s="153"/>
+      <c r="H72" s="153"/>
+      <c r="I72" s="153"/>
+      <c r="J72" s="153"/>
+      <c r="K72" s="153"/>
+      <c r="L72" s="153"/>
+      <c r="M72" s="154"/>
+    </row>
+    <row r="73" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="32">
+        <v>48</v>
+      </c>
+      <c r="B73" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="C73" s="33"/>
+      <c r="D73" s="152"/>
+      <c r="E73" s="153"/>
+      <c r="F73" s="153"/>
+      <c r="G73" s="153"/>
+      <c r="H73" s="153"/>
+      <c r="I73" s="153"/>
+      <c r="J73" s="153"/>
+      <c r="K73" s="153"/>
+      <c r="L73" s="153"/>
+      <c r="M73" s="154"/>
+    </row>
+    <row r="74" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="32">
+        <v>49</v>
+      </c>
+      <c r="B74" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="C74" s="33"/>
+      <c r="D74" s="152"/>
+      <c r="E74" s="153"/>
+      <c r="F74" s="153"/>
+      <c r="G74" s="153"/>
+      <c r="H74" s="153"/>
+      <c r="I74" s="153"/>
+      <c r="J74" s="153"/>
+      <c r="K74" s="153"/>
+      <c r="L74" s="153"/>
+      <c r="M74" s="154"/>
+    </row>
+    <row r="75" spans="1:13" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="32">
+        <v>50</v>
+      </c>
+      <c r="B75" s="33" t="s">
+        <v>164</v>
+      </c>
+      <c r="C75" s="33"/>
+      <c r="D75" s="155"/>
+      <c r="E75" s="156"/>
+      <c r="F75" s="156"/>
+      <c r="G75" s="156"/>
+      <c r="H75" s="156"/>
+      <c r="I75" s="156"/>
+      <c r="J75" s="156"/>
+      <c r="K75" s="156"/>
+      <c r="L75" s="156"/>
+      <c r="M75" s="157"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="B6:M6"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="B7:M7"/>
     <mergeCell ref="E21:M22"/>
     <mergeCell ref="A16:M16"/>
     <mergeCell ref="A17:M17"/>
-    <mergeCell ref="D26:M72"/>
     <mergeCell ref="B14:M14"/>
     <mergeCell ref="B15:M15"/>
     <mergeCell ref="D18:D20"/>
@@ -12970,13 +13426,7 @@
     <mergeCell ref="A23:M23"/>
     <mergeCell ref="A24:M24"/>
     <mergeCell ref="D21:D22"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="B6:M6"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A9:M9"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="B5:M5"/>
-    <mergeCell ref="B7:M7"/>
+    <mergeCell ref="D26:M75"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
@@ -16128,6 +16578,116 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>1440180</xdr:colOff>
                     <xdr:row>69</xdr:row>
+                    <xdr:rowOff>251460</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1271" r:id="rId148" name="Drop Down 247">
+              <controlPr defaultSize="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>30480</xdr:colOff>
+                    <xdr:row>70</xdr:row>
+                    <xdr:rowOff>22860</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>1440180</xdr:colOff>
+                    <xdr:row>70</xdr:row>
+                    <xdr:rowOff>251460</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1272" r:id="rId149" name="Drop Down 248">
+              <controlPr defaultSize="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>30480</xdr:colOff>
+                    <xdr:row>71</xdr:row>
+                    <xdr:rowOff>22860</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>1440180</xdr:colOff>
+                    <xdr:row>71</xdr:row>
+                    <xdr:rowOff>251460</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1273" r:id="rId150" name="Drop Down 249">
+              <controlPr defaultSize="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>30480</xdr:colOff>
+                    <xdr:row>72</xdr:row>
+                    <xdr:rowOff>22860</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>1440180</xdr:colOff>
+                    <xdr:row>72</xdr:row>
+                    <xdr:rowOff>251460</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1274" r:id="rId151" name="Drop Down 250">
+              <controlPr defaultSize="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>30480</xdr:colOff>
+                    <xdr:row>73</xdr:row>
+                    <xdr:rowOff>22860</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>1440180</xdr:colOff>
+                    <xdr:row>73</xdr:row>
+                    <xdr:rowOff>251460</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1275" r:id="rId152" name="Drop Down 251">
+              <controlPr defaultSize="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>30480</xdr:colOff>
+                    <xdr:row>74</xdr:row>
+                    <xdr:rowOff>22860</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>1440180</xdr:colOff>
+                    <xdr:row>74</xdr:row>
                     <xdr:rowOff>251460</xdr:rowOff>
                   </to>
                 </anchor>
@@ -16158,50 +16718,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="127" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="132"/>
-      <c r="C1" s="132"/>
-      <c r="D1" s="132"/>
-      <c r="E1" s="132"/>
-      <c r="F1" s="132"/>
-      <c r="G1" s="132"/>
-      <c r="H1" s="132"/>
-      <c r="I1" s="132"/>
-      <c r="J1" s="132"/>
-      <c r="K1" s="132"/>
-      <c r="L1" s="133"/>
+      <c r="B1" s="128"/>
+      <c r="C1" s="128"/>
+      <c r="D1" s="128"/>
+      <c r="E1" s="128"/>
+      <c r="F1" s="128"/>
+      <c r="G1" s="128"/>
+      <c r="H1" s="128"/>
+      <c r="I1" s="128"/>
+      <c r="J1" s="128"/>
+      <c r="K1" s="128"/>
+      <c r="L1" s="129"/>
     </row>
     <row r="2" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="134" t="s">
+      <c r="A2" s="130" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="135"/>
-      <c r="C2" s="135"/>
-      <c r="D2" s="135"/>
-      <c r="E2" s="135"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
-      <c r="I2" s="135"/>
-      <c r="J2" s="135"/>
-      <c r="K2" s="135"/>
-      <c r="L2" s="136"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="131"/>
+      <c r="D2" s="131"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="131"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="131"/>
+      <c r="I2" s="131"/>
+      <c r="J2" s="131"/>
+      <c r="K2" s="131"/>
+      <c r="L2" s="132"/>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="137"/>
-      <c r="B3" s="138"/>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="138"/>
-      <c r="F3" s="138"/>
-      <c r="G3" s="138"/>
-      <c r="H3" s="138"/>
-      <c r="I3" s="138"/>
-      <c r="J3" s="138"/>
-      <c r="K3" s="138"/>
-      <c r="L3" s="139"/>
+      <c r="A3" s="133"/>
+      <c r="B3" s="134"/>
+      <c r="C3" s="134"/>
+      <c r="D3" s="134"/>
+      <c r="E3" s="134"/>
+      <c r="F3" s="134"/>
+      <c r="G3" s="134"/>
+      <c r="H3" s="134"/>
+      <c r="I3" s="134"/>
+      <c r="J3" s="134"/>
+      <c r="K3" s="134"/>
+      <c r="L3" s="135"/>
     </row>
     <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -16291,65 +16851,65 @@
       <c r="A8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="142"/>
-      <c r="C8" s="143"/>
-      <c r="D8" s="143"/>
-      <c r="E8" s="143"/>
-      <c r="F8" s="143"/>
-      <c r="G8" s="143"/>
-      <c r="H8" s="143"/>
-      <c r="I8" s="143"/>
-      <c r="J8" s="143"/>
-      <c r="K8" s="143"/>
-      <c r="L8" s="144"/>
+      <c r="B8" s="138"/>
+      <c r="C8" s="139"/>
+      <c r="D8" s="139"/>
+      <c r="E8" s="139"/>
+      <c r="F8" s="139"/>
+      <c r="G8" s="139"/>
+      <c r="H8" s="139"/>
+      <c r="I8" s="139"/>
+      <c r="J8" s="139"/>
+      <c r="K8" s="139"/>
+      <c r="L8" s="140"/>
     </row>
     <row r="9" spans="1:12" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="145"/>
-      <c r="C9" s="143"/>
-      <c r="D9" s="143"/>
-      <c r="E9" s="143"/>
-      <c r="F9" s="143"/>
-      <c r="G9" s="143"/>
-      <c r="H9" s="143"/>
-      <c r="I9" s="143"/>
-      <c r="J9" s="143"/>
-      <c r="K9" s="143"/>
-      <c r="L9" s="144"/>
+      <c r="B9" s="141"/>
+      <c r="C9" s="139"/>
+      <c r="D9" s="139"/>
+      <c r="E9" s="139"/>
+      <c r="F9" s="139"/>
+      <c r="G9" s="139"/>
+      <c r="H9" s="139"/>
+      <c r="I9" s="139"/>
+      <c r="J9" s="139"/>
+      <c r="K9" s="139"/>
+      <c r="L9" s="140"/>
     </row>
     <row r="10" spans="1:12" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="140" t="s">
+      <c r="A10" s="136" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="141"/>
-      <c r="C10" s="141"/>
-      <c r="D10" s="141"/>
-      <c r="E10" s="141"/>
-      <c r="F10" s="141"/>
-      <c r="G10" s="141"/>
-      <c r="H10" s="141"/>
-      <c r="I10" s="141"/>
-      <c r="J10" s="141"/>
-      <c r="K10" s="141"/>
-      <c r="L10" s="141"/>
+      <c r="B10" s="137"/>
+      <c r="C10" s="137"/>
+      <c r="D10" s="137"/>
+      <c r="E10" s="137"/>
+      <c r="F10" s="137"/>
+      <c r="G10" s="137"/>
+      <c r="H10" s="137"/>
+      <c r="I10" s="137"/>
+      <c r="J10" s="137"/>
+      <c r="K10" s="137"/>
+      <c r="L10" s="137"/>
     </row>
     <row r="11" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="122" t="s">
+      <c r="A11" s="118" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="123"/>
-      <c r="C11" s="123"/>
-      <c r="D11" s="123"/>
-      <c r="E11" s="123"/>
-      <c r="F11" s="123"/>
-      <c r="G11" s="123"/>
-      <c r="H11" s="123"/>
-      <c r="I11" s="123"/>
-      <c r="J11" s="123"/>
-      <c r="K11" s="123"/>
-      <c r="L11" s="124"/>
+      <c r="B11" s="119"/>
+      <c r="C11" s="119"/>
+      <c r="D11" s="119"/>
+      <c r="E11" s="119"/>
+      <c r="F11" s="119"/>
+      <c r="G11" s="119"/>
+      <c r="H11" s="119"/>
+      <c r="I11" s="119"/>
+      <c r="J11" s="119"/>
+      <c r="K11" s="119"/>
+      <c r="L11" s="120"/>
     </row>
     <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
@@ -16361,101 +16921,101 @@
       <c r="C12" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="114" t="s">
+      <c r="D12" s="93" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="114"/>
-      <c r="F12" s="114"/>
-      <c r="G12" s="114"/>
-      <c r="H12" s="114"/>
-      <c r="I12" s="114"/>
-      <c r="J12" s="114"/>
-      <c r="K12" s="114"/>
-      <c r="L12" s="114"/>
+      <c r="E12" s="93"/>
+      <c r="F12" s="93"/>
+      <c r="G12" s="93"/>
+      <c r="H12" s="93"/>
+      <c r="I12" s="93"/>
+      <c r="J12" s="93"/>
+      <c r="K12" s="93"/>
+      <c r="L12" s="93"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="48"/>
       <c r="B13" s="49"/>
       <c r="C13" s="49"/>
-      <c r="D13" s="125"/>
-      <c r="E13" s="126"/>
-      <c r="F13" s="126"/>
-      <c r="G13" s="126"/>
-      <c r="H13" s="126"/>
-      <c r="I13" s="126"/>
-      <c r="J13" s="126"/>
-      <c r="K13" s="126"/>
-      <c r="L13" s="127"/>
+      <c r="D13" s="121"/>
+      <c r="E13" s="122"/>
+      <c r="F13" s="122"/>
+      <c r="G13" s="122"/>
+      <c r="H13" s="122"/>
+      <c r="I13" s="122"/>
+      <c r="J13" s="122"/>
+      <c r="K13" s="122"/>
+      <c r="L13" s="123"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="48"/>
       <c r="B14" s="49"/>
       <c r="C14" s="49"/>
-      <c r="D14" s="128"/>
-      <c r="E14" s="129"/>
-      <c r="F14" s="129"/>
-      <c r="G14" s="129"/>
-      <c r="H14" s="129"/>
-      <c r="I14" s="129"/>
-      <c r="J14" s="129"/>
-      <c r="K14" s="129"/>
-      <c r="L14" s="130"/>
+      <c r="D14" s="124"/>
+      <c r="E14" s="125"/>
+      <c r="F14" s="125"/>
+      <c r="G14" s="125"/>
+      <c r="H14" s="125"/>
+      <c r="I14" s="125"/>
+      <c r="J14" s="125"/>
+      <c r="K14" s="125"/>
+      <c r="L14" s="126"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="48"/>
       <c r="B15" s="49"/>
       <c r="C15" s="49"/>
-      <c r="D15" s="128"/>
-      <c r="E15" s="129"/>
-      <c r="F15" s="129"/>
-      <c r="G15" s="129"/>
-      <c r="H15" s="129"/>
-      <c r="I15" s="129"/>
-      <c r="J15" s="129"/>
-      <c r="K15" s="129"/>
-      <c r="L15" s="130"/>
+      <c r="D15" s="124"/>
+      <c r="E15" s="125"/>
+      <c r="F15" s="125"/>
+      <c r="G15" s="125"/>
+      <c r="H15" s="125"/>
+      <c r="I15" s="125"/>
+      <c r="J15" s="125"/>
+      <c r="K15" s="125"/>
+      <c r="L15" s="126"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="48"/>
       <c r="B16" s="49"/>
       <c r="C16" s="49"/>
-      <c r="D16" s="128"/>
-      <c r="E16" s="129"/>
-      <c r="F16" s="129"/>
-      <c r="G16" s="129"/>
-      <c r="H16" s="129"/>
-      <c r="I16" s="129"/>
-      <c r="J16" s="129"/>
-      <c r="K16" s="129"/>
-      <c r="L16" s="130"/>
+      <c r="D16" s="124"/>
+      <c r="E16" s="125"/>
+      <c r="F16" s="125"/>
+      <c r="G16" s="125"/>
+      <c r="H16" s="125"/>
+      <c r="I16" s="125"/>
+      <c r="J16" s="125"/>
+      <c r="K16" s="125"/>
+      <c r="L16" s="126"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="48"/>
       <c r="B17" s="49"/>
       <c r="C17" s="49"/>
-      <c r="D17" s="128"/>
-      <c r="E17" s="129"/>
-      <c r="F17" s="129"/>
-      <c r="G17" s="129"/>
-      <c r="H17" s="129"/>
-      <c r="I17" s="129"/>
-      <c r="J17" s="129"/>
-      <c r="K17" s="129"/>
-      <c r="L17" s="130"/>
+      <c r="D17" s="124"/>
+      <c r="E17" s="125"/>
+      <c r="F17" s="125"/>
+      <c r="G17" s="125"/>
+      <c r="H17" s="125"/>
+      <c r="I17" s="125"/>
+      <c r="J17" s="125"/>
+      <c r="K17" s="125"/>
+      <c r="L17" s="126"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="48"/>
       <c r="B18" s="49"/>
       <c r="C18" s="49"/>
-      <c r="D18" s="128"/>
-      <c r="E18" s="129"/>
-      <c r="F18" s="129"/>
-      <c r="G18" s="129"/>
-      <c r="H18" s="129"/>
-      <c r="I18" s="129"/>
-      <c r="J18" s="129"/>
-      <c r="K18" s="129"/>
-      <c r="L18" s="130"/>
+      <c r="D18" s="124"/>
+      <c r="E18" s="125"/>
+      <c r="F18" s="125"/>
+      <c r="G18" s="125"/>
+      <c r="H18" s="125"/>
+      <c r="I18" s="125"/>
+      <c r="J18" s="125"/>
+      <c r="K18" s="125"/>
+      <c r="L18" s="126"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -16544,10 +17104,10 @@
       <c r="B4" s="62"/>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="146" t="s">
+      <c r="A6" s="142" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="146"/>
+      <c r="B6" s="142"/>
     </row>
     <row r="8" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="65" t="s">
@@ -16706,53 +17266,53 @@
   <sheetData>
     <row r="1" spans="2:6" ht="5.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B2" s="148"/>
-      <c r="C2" s="148"/>
-      <c r="D2" s="149" t="s">
+      <c r="B2" s="144"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="145" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="150" t="s">
+      <c r="E2" s="146" t="s">
         <v>49</v>
       </c>
-      <c r="F2" s="150"/>
+      <c r="F2" s="146"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="148"/>
-      <c r="C3" s="148"/>
-      <c r="D3" s="149"/>
-      <c r="E3" s="150"/>
-      <c r="F3" s="150"/>
+      <c r="B3" s="144"/>
+      <c r="C3" s="144"/>
+      <c r="D3" s="145"/>
+      <c r="E3" s="146"/>
+      <c r="F3" s="146"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="148"/>
-      <c r="C4" s="148"/>
-      <c r="D4" s="149"/>
-      <c r="E4" s="150" t="s">
+      <c r="B4" s="144"/>
+      <c r="C4" s="144"/>
+      <c r="D4" s="145"/>
+      <c r="E4" s="146" t="s">
         <v>108</v>
       </c>
-      <c r="F4" s="150"/>
+      <c r="F4" s="146"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="151" t="s">
+      <c r="B5" s="147" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="151"/>
+      <c r="C5" s="147"/>
       <c r="D5" s="69" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="152" t="s">
+      <c r="E5" s="148" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="152"/>
+      <c r="F5" s="148"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="71" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="147"/>
-      <c r="D6" s="147"/>
-      <c r="E6" s="147"/>
-      <c r="F6" s="147"/>
+      <c r="C6" s="143"/>
+      <c r="D6" s="143"/>
+      <c r="E6" s="143"/>
+      <c r="F6" s="143"/>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="70" t="s">
@@ -17007,10 +17567,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="26" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="149" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="154"/>
+      <c r="B1" s="150"/>
     </row>
     <row r="2" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="27" t="s">
@@ -17281,15 +17841,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005DA7AC6E4F4FAE42B9D9FCD9C82CAAE1" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="553e0bb76796fbad2df2b84fb95dc83d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87481c51-c14c-4071-bf64-faa2b5708bb6" xmlns:ns3="8029d101-3d2a-47c4-b15f-619642bf5e50" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d87cd7f238c73dc12c577d08dde48736" ns2:_="" ns3:_="">
     <xsd:import namespace="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
@@ -17538,6 +18089,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -17592,14 +18152,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F7F06D0-41B3-4EAF-B418-88FC726117CC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17618,6 +18170,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
fix modificacion de zip
</commit_message>
<xml_diff>
--- a/Guias Produccion/HU-55188.xlsx
+++ b/Guias Produccion/HU-55188.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Alliance\ScriptsEntidades\Guias Produccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B5F96E-A5A5-49A8-BF07-F852966CE2B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C43AC9F-2460-49BE-BC90-3ED92A0BD607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="163">
   <si>
     <t>Guia documentación</t>
   </si>
@@ -652,30 +652,6 @@
   </si>
   <si>
     <t>48-UpdateOpcionesRetraso.sql</t>
-  </si>
-  <si>
-    <t>49-DataValidationEntitiesAUX.sql</t>
-  </si>
-  <si>
-    <t>50-DataMigrationEntities.sql</t>
-  </si>
-  <si>
-    <t>51-DataMappingGuiasHouse.sql</t>
-  </si>
-  <si>
-    <t>52-DataMappingGuias.sql</t>
-  </si>
-  <si>
-    <t>53-DataMappingGuiasHouseDetalles.sql</t>
-  </si>
-  <si>
-    <t>54-DataMappingAgentesCliente.sql</t>
-  </si>
-  <si>
-    <t>55-DataMappingContactos.sql</t>
-  </si>
-  <si>
-    <t>56-DataMappingOrdenesLocales.sql</t>
   </si>
 </sst>
 </file>
@@ -1969,56 +1945,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2083,35 +2038,62 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2210,12 +2192,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2449,47 +2425,15 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp147.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp148.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp149.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp15.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$18" noThreeD="1" sel="14" val="7"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp150.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp151.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="17"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp152.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp153.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp154.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp155.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp156.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp16.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11296,470 +11240,6 @@
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
                   <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000F9040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>30480</xdr:colOff>
-          <xdr:row>73</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1440180</xdr:colOff>
-          <xdr:row>74</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1274" name="Drop Down 250" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1274"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000FA040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>30480</xdr:colOff>
-          <xdr:row>74</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1440180</xdr:colOff>
-          <xdr:row>75</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1275" name="Drop Down 251" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1275"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000FB040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>30480</xdr:colOff>
-          <xdr:row>75</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1440180</xdr:colOff>
-          <xdr:row>76</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1276" name="Drop Down 252" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1276"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000FC040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>30480</xdr:colOff>
-          <xdr:row>76</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1440180</xdr:colOff>
-          <xdr:row>77</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1277" name="Drop Down 253" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1277"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000FD040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>30480</xdr:colOff>
-          <xdr:row>77</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1440180</xdr:colOff>
-          <xdr:row>78</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1278" name="Drop Down 254" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1278"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000FE040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>30480</xdr:colOff>
-          <xdr:row>78</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1440180</xdr:colOff>
-          <xdr:row>79</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1279" name="Drop Down 255" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1279"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000FF040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>30480</xdr:colOff>
-          <xdr:row>79</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1440180</xdr:colOff>
-          <xdr:row>80</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1280" name="Drop Down 256" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1280"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000000050000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>30480</xdr:colOff>
-          <xdr:row>80</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1440180</xdr:colOff>
-          <xdr:row>81</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1281" name="Drop Down 257" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1281"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E794172D-189D-BE14-3EC2-54662DAA20B9}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -12405,44 +11885,44 @@
   <sheetData>
     <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:16" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="80" t="s">
+      <c r="A3" s="113" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="81"/>
-      <c r="C3" s="81"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="81"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="81"/>
-      <c r="O3" s="76" t="s">
+      <c r="B3" s="114"/>
+      <c r="C3" s="114"/>
+      <c r="D3" s="114"/>
+      <c r="E3" s="114"/>
+      <c r="F3" s="114"/>
+      <c r="G3" s="114"/>
+      <c r="H3" s="114"/>
+      <c r="I3" s="114"/>
+      <c r="J3" s="114"/>
+      <c r="K3" s="114"/>
+      <c r="L3" s="114"/>
+      <c r="M3" s="114"/>
+      <c r="O3" s="109" t="s">
         <v>0</v>
       </c>
-      <c r="P3" s="77"/>
+      <c r="P3" s="110"/>
     </row>
     <row r="4" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="85" t="s">
+      <c r="B4" s="118" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="86"/>
-      <c r="D4" s="86"/>
-      <c r="E4" s="86"/>
-      <c r="F4" s="86"/>
-      <c r="G4" s="86"/>
-      <c r="H4" s="86"/>
-      <c r="I4" s="86"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="87"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="119"/>
+      <c r="J4" s="120"/>
+      <c r="K4" s="120"/>
+      <c r="L4" s="120"/>
+      <c r="M4" s="120"/>
       <c r="O4" s="20" t="s">
         <v>2</v>
       </c>
@@ -12452,20 +11932,20 @@
       <c r="A5" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="88" t="s">
+      <c r="B5" s="121" t="s">
         <v>113</v>
       </c>
-      <c r="C5" s="88"/>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
-      <c r="K5" s="89"/>
-      <c r="L5" s="89"/>
-      <c r="M5" s="89"/>
+      <c r="C5" s="121"/>
+      <c r="D5" s="121"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
+      <c r="H5" s="121"/>
+      <c r="I5" s="121"/>
+      <c r="J5" s="122"/>
+      <c r="K5" s="122"/>
+      <c r="L5" s="122"/>
+      <c r="M5" s="122"/>
       <c r="O5" s="14" t="s">
         <v>4</v>
       </c>
@@ -12475,20 +11955,20 @@
       <c r="A6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="78">
+      <c r="B6" s="111">
         <v>45974</v>
       </c>
-      <c r="C6" s="79"/>
-      <c r="D6" s="79"/>
-      <c r="E6" s="79"/>
-      <c r="F6" s="79"/>
-      <c r="G6" s="79"/>
-      <c r="H6" s="79"/>
-      <c r="I6" s="79"/>
-      <c r="J6" s="79"/>
-      <c r="K6" s="79"/>
-      <c r="L6" s="79"/>
-      <c r="M6" s="79"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="112"/>
+      <c r="E6" s="112"/>
+      <c r="F6" s="112"/>
+      <c r="G6" s="112"/>
+      <c r="H6" s="112"/>
+      <c r="I6" s="112"/>
+      <c r="J6" s="112"/>
+      <c r="K6" s="112"/>
+      <c r="L6" s="112"/>
+      <c r="M6" s="112"/>
       <c r="O6" s="13"/>
       <c r="P6" s="13"/>
     </row>
@@ -12496,18 +11976,18 @@
       <c r="A7" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="90"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="92"/>
-      <c r="K7" s="92"/>
-      <c r="L7" s="92"/>
-      <c r="M7" s="92"/>
+      <c r="B7" s="123"/>
+      <c r="C7" s="124"/>
+      <c r="D7" s="124"/>
+      <c r="E7" s="124"/>
+      <c r="F7" s="124"/>
+      <c r="G7" s="124"/>
+      <c r="H7" s="124"/>
+      <c r="I7" s="124"/>
+      <c r="J7" s="125"/>
+      <c r="K7" s="125"/>
+      <c r="L7" s="125"/>
+      <c r="M7" s="125"/>
     </row>
     <row r="8" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11"/>
@@ -12525,21 +12005,21 @@
       <c r="M8" s="12"/>
     </row>
     <row r="9" spans="1:16" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="82" t="s">
+      <c r="A9" s="115" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="83"/>
-      <c r="C9" s="83"/>
-      <c r="D9" s="83"/>
-      <c r="E9" s="83"/>
-      <c r="F9" s="83"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="83"/>
-      <c r="I9" s="83"/>
-      <c r="J9" s="84"/>
-      <c r="K9" s="84"/>
-      <c r="L9" s="84"/>
-      <c r="M9" s="84"/>
+      <c r="B9" s="116"/>
+      <c r="C9" s="116"/>
+      <c r="D9" s="116"/>
+      <c r="E9" s="116"/>
+      <c r="F9" s="116"/>
+      <c r="G9" s="116"/>
+      <c r="H9" s="116"/>
+      <c r="I9" s="116"/>
+      <c r="J9" s="117"/>
+      <c r="K9" s="117"/>
+      <c r="L9" s="117"/>
+      <c r="M9" s="117"/>
     </row>
     <row r="10" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -12640,67 +12120,67 @@
       <c r="A14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="98"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="99"/>
-      <c r="F14" s="99"/>
-      <c r="G14" s="99"/>
-      <c r="H14" s="99"/>
-      <c r="I14" s="99"/>
-      <c r="J14" s="99"/>
-      <c r="K14" s="99"/>
-      <c r="L14" s="99"/>
-      <c r="M14" s="99"/>
+      <c r="B14" s="91"/>
+      <c r="C14" s="92"/>
+      <c r="D14" s="92"/>
+      <c r="E14" s="92"/>
+      <c r="F14" s="92"/>
+      <c r="G14" s="92"/>
+      <c r="H14" s="92"/>
+      <c r="I14" s="92"/>
+      <c r="J14" s="92"/>
+      <c r="K14" s="92"/>
+      <c r="L14" s="92"/>
+      <c r="M14" s="92"/>
     </row>
     <row r="15" spans="1:16" s="75" customFormat="1" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="98"/>
-      <c r="C15" s="99"/>
-      <c r="D15" s="99"/>
-      <c r="E15" s="99"/>
-      <c r="F15" s="99"/>
-      <c r="G15" s="99"/>
-      <c r="H15" s="99"/>
-      <c r="I15" s="99"/>
-      <c r="J15" s="99"/>
-      <c r="K15" s="99"/>
-      <c r="L15" s="99"/>
-      <c r="M15" s="99"/>
+      <c r="B15" s="91"/>
+      <c r="C15" s="92"/>
+      <c r="D15" s="92"/>
+      <c r="E15" s="92"/>
+      <c r="F15" s="92"/>
+      <c r="G15" s="92"/>
+      <c r="H15" s="92"/>
+      <c r="I15" s="92"/>
+      <c r="J15" s="92"/>
+      <c r="K15" s="92"/>
+      <c r="L15" s="92"/>
+      <c r="M15" s="92"/>
     </row>
     <row r="16" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="93"/>
-      <c r="B16" s="94"/>
-      <c r="C16" s="94"/>
-      <c r="D16" s="94"/>
-      <c r="E16" s="94"/>
-      <c r="F16" s="94"/>
-      <c r="G16" s="94"/>
-      <c r="H16" s="94"/>
-      <c r="I16" s="94"/>
-      <c r="J16" s="94"/>
-      <c r="K16" s="94"/>
-      <c r="L16" s="94"/>
-      <c r="M16" s="94"/>
+      <c r="A16" s="86"/>
+      <c r="B16" s="87"/>
+      <c r="C16" s="87"/>
+      <c r="D16" s="87"/>
+      <c r="E16" s="87"/>
+      <c r="F16" s="87"/>
+      <c r="G16" s="87"/>
+      <c r="H16" s="87"/>
+      <c r="I16" s="87"/>
+      <c r="J16" s="87"/>
+      <c r="K16" s="87"/>
+      <c r="L16" s="87"/>
+      <c r="M16" s="87"/>
     </row>
     <row r="17" spans="1:13" s="5" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="95" t="s">
+      <c r="A17" s="88" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="96"/>
-      <c r="C17" s="96"/>
-      <c r="D17" s="96"/>
-      <c r="E17" s="96"/>
-      <c r="F17" s="96"/>
-      <c r="G17" s="96"/>
-      <c r="H17" s="96"/>
-      <c r="I17" s="96"/>
-      <c r="J17" s="97"/>
-      <c r="K17" s="97"/>
-      <c r="L17" s="97"/>
-      <c r="M17" s="97"/>
+      <c r="B17" s="89"/>
+      <c r="C17" s="89"/>
+      <c r="D17" s="89"/>
+      <c r="E17" s="89"/>
+      <c r="F17" s="89"/>
+      <c r="G17" s="89"/>
+      <c r="H17" s="89"/>
+      <c r="I17" s="89"/>
+      <c r="J17" s="90"/>
+      <c r="K17" s="90"/>
+      <c r="L17" s="90"/>
+      <c r="M17" s="90"/>
     </row>
     <row r="18" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
@@ -12710,18 +12190,18 @@
       <c r="C18" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="100" t="s">
+      <c r="D18" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="102"/>
-      <c r="F18" s="102"/>
-      <c r="G18" s="102"/>
-      <c r="H18" s="102"/>
-      <c r="I18" s="102"/>
-      <c r="J18" s="103"/>
-      <c r="K18" s="103"/>
-      <c r="L18" s="103"/>
-      <c r="M18" s="103"/>
+      <c r="E18" s="95"/>
+      <c r="F18" s="95"/>
+      <c r="G18" s="95"/>
+      <c r="H18" s="95"/>
+      <c r="I18" s="95"/>
+      <c r="J18" s="96"/>
+      <c r="K18" s="96"/>
+      <c r="L18" s="96"/>
+      <c r="M18" s="96"/>
     </row>
     <row r="19" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
@@ -12731,16 +12211,16 @@
         <v>103</v>
       </c>
       <c r="C19" s="43"/>
-      <c r="D19" s="101"/>
-      <c r="E19" s="104"/>
-      <c r="F19" s="104"/>
-      <c r="G19" s="104"/>
-      <c r="H19" s="104"/>
-      <c r="I19" s="104"/>
-      <c r="J19" s="105"/>
-      <c r="K19" s="105"/>
-      <c r="L19" s="105"/>
-      <c r="M19" s="105"/>
+      <c r="D19" s="94"/>
+      <c r="E19" s="97"/>
+      <c r="F19" s="97"/>
+      <c r="G19" s="97"/>
+      <c r="H19" s="97"/>
+      <c r="I19" s="97"/>
+      <c r="J19" s="98"/>
+      <c r="K19" s="98"/>
+      <c r="L19" s="98"/>
+      <c r="M19" s="98"/>
     </row>
     <row r="20" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
@@ -12750,16 +12230,16 @@
         <v>103</v>
       </c>
       <c r="C20" s="43"/>
-      <c r="D20" s="101"/>
-      <c r="E20" s="104"/>
-      <c r="F20" s="104"/>
-      <c r="G20" s="104"/>
-      <c r="H20" s="104"/>
-      <c r="I20" s="104"/>
-      <c r="J20" s="105"/>
-      <c r="K20" s="105"/>
-      <c r="L20" s="105"/>
-      <c r="M20" s="105"/>
+      <c r="D20" s="94"/>
+      <c r="E20" s="97"/>
+      <c r="F20" s="97"/>
+      <c r="G20" s="97"/>
+      <c r="H20" s="97"/>
+      <c r="I20" s="97"/>
+      <c r="J20" s="98"/>
+      <c r="K20" s="98"/>
+      <c r="L20" s="98"/>
+      <c r="M20" s="98"/>
     </row>
     <row r="21" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -12769,20 +12249,20 @@
         <v>103</v>
       </c>
       <c r="C21" s="43"/>
-      <c r="D21" s="112" t="s">
+      <c r="D21" s="105" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="114" t="s">
+      <c r="E21" s="77" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="115"/>
-      <c r="G21" s="115"/>
-      <c r="H21" s="115"/>
-      <c r="I21" s="115"/>
-      <c r="J21" s="115"/>
-      <c r="K21" s="115"/>
-      <c r="L21" s="115"/>
-      <c r="M21" s="115"/>
+      <c r="F21" s="78"/>
+      <c r="G21" s="78"/>
+      <c r="H21" s="78"/>
+      <c r="I21" s="78"/>
+      <c r="J21" s="78"/>
+      <c r="K21" s="78"/>
+      <c r="L21" s="78"/>
+      <c r="M21" s="78"/>
     </row>
     <row r="22" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
@@ -12792,48 +12272,48 @@
       <c r="C22" s="43" t="s">
         <v>103</v>
       </c>
-      <c r="D22" s="113"/>
-      <c r="E22" s="122"/>
-      <c r="F22" s="123"/>
-      <c r="G22" s="123"/>
-      <c r="H22" s="123"/>
-      <c r="I22" s="123"/>
-      <c r="J22" s="123"/>
-      <c r="K22" s="123"/>
-      <c r="L22" s="123"/>
-      <c r="M22" s="123"/>
+      <c r="D22" s="106"/>
+      <c r="E22" s="107"/>
+      <c r="F22" s="108"/>
+      <c r="G22" s="108"/>
+      <c r="H22" s="108"/>
+      <c r="I22" s="108"/>
+      <c r="J22" s="108"/>
+      <c r="K22" s="108"/>
+      <c r="L22" s="108"/>
+      <c r="M22" s="108"/>
     </row>
     <row r="23" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="107"/>
-      <c r="B23" s="108"/>
-      <c r="C23" s="108"/>
-      <c r="D23" s="109"/>
-      <c r="E23" s="109"/>
-      <c r="F23" s="109"/>
-      <c r="G23" s="109"/>
-      <c r="H23" s="109"/>
-      <c r="I23" s="109"/>
-      <c r="J23" s="109"/>
-      <c r="K23" s="109"/>
-      <c r="L23" s="109"/>
-      <c r="M23" s="109"/>
+      <c r="A23" s="100"/>
+      <c r="B23" s="101"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="102"/>
+      <c r="E23" s="102"/>
+      <c r="F23" s="102"/>
+      <c r="G23" s="102"/>
+      <c r="H23" s="102"/>
+      <c r="I23" s="102"/>
+      <c r="J23" s="102"/>
+      <c r="K23" s="102"/>
+      <c r="L23" s="102"/>
+      <c r="M23" s="102"/>
     </row>
     <row r="24" spans="1:13" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="110" t="s">
+      <c r="A24" s="103" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="111"/>
-      <c r="C24" s="111"/>
-      <c r="D24" s="111"/>
-      <c r="E24" s="111"/>
-      <c r="F24" s="111"/>
-      <c r="G24" s="111"/>
-      <c r="H24" s="111"/>
-      <c r="I24" s="111"/>
-      <c r="J24" s="111"/>
-      <c r="K24" s="111"/>
-      <c r="L24" s="111"/>
-      <c r="M24" s="111"/>
+      <c r="B24" s="104"/>
+      <c r="C24" s="104"/>
+      <c r="D24" s="104"/>
+      <c r="E24" s="104"/>
+      <c r="F24" s="104"/>
+      <c r="G24" s="104"/>
+      <c r="H24" s="104"/>
+      <c r="I24" s="104"/>
+      <c r="J24" s="104"/>
+      <c r="K24" s="104"/>
+      <c r="L24" s="104"/>
+      <c r="M24" s="104"/>
     </row>
     <row r="25" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="15" t="s">
@@ -12845,18 +12325,18 @@
       <c r="C25" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="106" t="s">
+      <c r="D25" s="99" t="s">
         <v>37</v>
       </c>
-      <c r="E25" s="106"/>
-      <c r="F25" s="106"/>
-      <c r="G25" s="106"/>
-      <c r="H25" s="106"/>
-      <c r="I25" s="106"/>
-      <c r="J25" s="106"/>
-      <c r="K25" s="106"/>
-      <c r="L25" s="106"/>
-      <c r="M25" s="106"/>
+      <c r="E25" s="99"/>
+      <c r="F25" s="99"/>
+      <c r="G25" s="99"/>
+      <c r="H25" s="99"/>
+      <c r="I25" s="99"/>
+      <c r="J25" s="99"/>
+      <c r="K25" s="99"/>
+      <c r="L25" s="99"/>
+      <c r="M25" s="99"/>
     </row>
     <row r="26" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="32">
@@ -12866,18 +12346,18 @@
         <v>115</v>
       </c>
       <c r="C26" s="33"/>
-      <c r="D26" s="114" t="s">
+      <c r="D26" s="77" t="s">
         <v>111</v>
       </c>
-      <c r="E26" s="115"/>
-      <c r="F26" s="115"/>
-      <c r="G26" s="115"/>
-      <c r="H26" s="115"/>
-      <c r="I26" s="115"/>
-      <c r="J26" s="115"/>
-      <c r="K26" s="115"/>
-      <c r="L26" s="115"/>
-      <c r="M26" s="116"/>
+      <c r="E26" s="78"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
+      <c r="I26" s="78"/>
+      <c r="J26" s="78"/>
+      <c r="K26" s="78"/>
+      <c r="L26" s="78"/>
+      <c r="M26" s="79"/>
     </row>
     <row r="27" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="32">
@@ -12887,16 +12367,16 @@
         <v>116</v>
       </c>
       <c r="C27" s="33"/>
-      <c r="D27" s="117"/>
-      <c r="E27" s="158"/>
-      <c r="F27" s="158"/>
-      <c r="G27" s="158"/>
-      <c r="H27" s="158"/>
-      <c r="I27" s="158"/>
-      <c r="J27" s="158"/>
-      <c r="K27" s="158"/>
-      <c r="L27" s="158"/>
-      <c r="M27" s="118"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="81"/>
+      <c r="F27" s="81"/>
+      <c r="G27" s="81"/>
+      <c r="H27" s="81"/>
+      <c r="I27" s="81"/>
+      <c r="J27" s="81"/>
+      <c r="K27" s="81"/>
+      <c r="L27" s="81"/>
+      <c r="M27" s="82"/>
     </row>
     <row r="28" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="32">
@@ -12906,16 +12386,16 @@
         <v>117</v>
       </c>
       <c r="C28" s="33"/>
-      <c r="D28" s="117"/>
-      <c r="E28" s="158"/>
-      <c r="F28" s="158"/>
-      <c r="G28" s="158"/>
-      <c r="H28" s="158"/>
-      <c r="I28" s="158"/>
-      <c r="J28" s="158"/>
-      <c r="K28" s="158"/>
-      <c r="L28" s="158"/>
-      <c r="M28" s="118"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="81"/>
+      <c r="F28" s="81"/>
+      <c r="G28" s="81"/>
+      <c r="H28" s="81"/>
+      <c r="I28" s="81"/>
+      <c r="J28" s="81"/>
+      <c r="K28" s="81"/>
+      <c r="L28" s="81"/>
+      <c r="M28" s="82"/>
     </row>
     <row r="29" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="32">
@@ -12925,16 +12405,16 @@
         <v>118</v>
       </c>
       <c r="C29" s="33"/>
-      <c r="D29" s="117"/>
-      <c r="E29" s="158"/>
-      <c r="F29" s="158"/>
-      <c r="G29" s="158"/>
-      <c r="H29" s="158"/>
-      <c r="I29" s="158"/>
-      <c r="J29" s="158"/>
-      <c r="K29" s="158"/>
-      <c r="L29" s="158"/>
-      <c r="M29" s="118"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="81"/>
+      <c r="F29" s="81"/>
+      <c r="G29" s="81"/>
+      <c r="H29" s="81"/>
+      <c r="I29" s="81"/>
+      <c r="J29" s="81"/>
+      <c r="K29" s="81"/>
+      <c r="L29" s="81"/>
+      <c r="M29" s="82"/>
     </row>
     <row r="30" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="32">
@@ -12944,16 +12424,16 @@
         <v>119</v>
       </c>
       <c r="C30" s="33"/>
-      <c r="D30" s="117"/>
-      <c r="E30" s="158"/>
-      <c r="F30" s="158"/>
-      <c r="G30" s="158"/>
-      <c r="H30" s="158"/>
-      <c r="I30" s="158"/>
-      <c r="J30" s="158"/>
-      <c r="K30" s="158"/>
-      <c r="L30" s="158"/>
-      <c r="M30" s="118"/>
+      <c r="D30" s="80"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="81"/>
+      <c r="H30" s="81"/>
+      <c r="I30" s="81"/>
+      <c r="J30" s="81"/>
+      <c r="K30" s="81"/>
+      <c r="L30" s="81"/>
+      <c r="M30" s="82"/>
     </row>
     <row r="31" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="32">
@@ -12963,16 +12443,16 @@
         <v>120</v>
       </c>
       <c r="C31" s="33"/>
-      <c r="D31" s="117"/>
-      <c r="E31" s="158"/>
-      <c r="F31" s="158"/>
-      <c r="G31" s="158"/>
-      <c r="H31" s="158"/>
-      <c r="I31" s="158"/>
-      <c r="J31" s="158"/>
-      <c r="K31" s="158"/>
-      <c r="L31" s="158"/>
-      <c r="M31" s="118"/>
+      <c r="D31" s="80"/>
+      <c r="E31" s="81"/>
+      <c r="F31" s="81"/>
+      <c r="G31" s="81"/>
+      <c r="H31" s="81"/>
+      <c r="I31" s="81"/>
+      <c r="J31" s="81"/>
+      <c r="K31" s="81"/>
+      <c r="L31" s="81"/>
+      <c r="M31" s="82"/>
     </row>
     <row r="32" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="32">
@@ -12982,16 +12462,16 @@
         <v>121</v>
       </c>
       <c r="C32" s="33"/>
-      <c r="D32" s="117"/>
-      <c r="E32" s="158"/>
-      <c r="F32" s="158"/>
-      <c r="G32" s="158"/>
-      <c r="H32" s="158"/>
-      <c r="I32" s="158"/>
-      <c r="J32" s="158"/>
-      <c r="K32" s="158"/>
-      <c r="L32" s="158"/>
-      <c r="M32" s="118"/>
+      <c r="D32" s="80"/>
+      <c r="E32" s="81"/>
+      <c r="F32" s="81"/>
+      <c r="G32" s="81"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="81"/>
+      <c r="J32" s="81"/>
+      <c r="K32" s="81"/>
+      <c r="L32" s="81"/>
+      <c r="M32" s="82"/>
     </row>
     <row r="33" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="32">
@@ -13001,16 +12481,16 @@
         <v>122</v>
       </c>
       <c r="C33" s="33"/>
-      <c r="D33" s="117"/>
-      <c r="E33" s="158"/>
-      <c r="F33" s="158"/>
-      <c r="G33" s="158"/>
-      <c r="H33" s="158"/>
-      <c r="I33" s="158"/>
-      <c r="J33" s="158"/>
-      <c r="K33" s="158"/>
-      <c r="L33" s="158"/>
-      <c r="M33" s="118"/>
+      <c r="D33" s="80"/>
+      <c r="E33" s="81"/>
+      <c r="F33" s="81"/>
+      <c r="G33" s="81"/>
+      <c r="H33" s="81"/>
+      <c r="I33" s="81"/>
+      <c r="J33" s="81"/>
+      <c r="K33" s="81"/>
+      <c r="L33" s="81"/>
+      <c r="M33" s="82"/>
     </row>
     <row r="34" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="32">
@@ -13020,16 +12500,16 @@
         <v>123</v>
       </c>
       <c r="C34" s="33"/>
-      <c r="D34" s="117"/>
-      <c r="E34" s="158"/>
-      <c r="F34" s="158"/>
-      <c r="G34" s="158"/>
-      <c r="H34" s="158"/>
-      <c r="I34" s="158"/>
-      <c r="J34" s="158"/>
-      <c r="K34" s="158"/>
-      <c r="L34" s="158"/>
-      <c r="M34" s="118"/>
+      <c r="D34" s="80"/>
+      <c r="E34" s="81"/>
+      <c r="F34" s="81"/>
+      <c r="G34" s="81"/>
+      <c r="H34" s="81"/>
+      <c r="I34" s="81"/>
+      <c r="J34" s="81"/>
+      <c r="K34" s="81"/>
+      <c r="L34" s="81"/>
+      <c r="M34" s="82"/>
     </row>
     <row r="35" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="32">
@@ -13039,16 +12519,16 @@
         <v>124</v>
       </c>
       <c r="C35" s="33"/>
-      <c r="D35" s="117"/>
-      <c r="E35" s="158"/>
-      <c r="F35" s="158"/>
-      <c r="G35" s="158"/>
-      <c r="H35" s="158"/>
-      <c r="I35" s="158"/>
-      <c r="J35" s="158"/>
-      <c r="K35" s="158"/>
-      <c r="L35" s="158"/>
-      <c r="M35" s="118"/>
+      <c r="D35" s="80"/>
+      <c r="E35" s="81"/>
+      <c r="F35" s="81"/>
+      <c r="G35" s="81"/>
+      <c r="H35" s="81"/>
+      <c r="I35" s="81"/>
+      <c r="J35" s="81"/>
+      <c r="K35" s="81"/>
+      <c r="L35" s="81"/>
+      <c r="M35" s="82"/>
     </row>
     <row r="36" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="32">
@@ -13058,16 +12538,16 @@
         <v>125</v>
       </c>
       <c r="C36" s="33"/>
-      <c r="D36" s="117"/>
-      <c r="E36" s="158"/>
-      <c r="F36" s="158"/>
-      <c r="G36" s="158"/>
-      <c r="H36" s="158"/>
-      <c r="I36" s="158"/>
-      <c r="J36" s="158"/>
-      <c r="K36" s="158"/>
-      <c r="L36" s="158"/>
-      <c r="M36" s="118"/>
+      <c r="D36" s="80"/>
+      <c r="E36" s="81"/>
+      <c r="F36" s="81"/>
+      <c r="G36" s="81"/>
+      <c r="H36" s="81"/>
+      <c r="I36" s="81"/>
+      <c r="J36" s="81"/>
+      <c r="K36" s="81"/>
+      <c r="L36" s="81"/>
+      <c r="M36" s="82"/>
     </row>
     <row r="37" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="32">
@@ -13077,16 +12557,16 @@
         <v>126</v>
       </c>
       <c r="C37" s="33"/>
-      <c r="D37" s="117"/>
-      <c r="E37" s="158"/>
-      <c r="F37" s="158"/>
-      <c r="G37" s="158"/>
-      <c r="H37" s="158"/>
-      <c r="I37" s="158"/>
-      <c r="J37" s="158"/>
-      <c r="K37" s="158"/>
-      <c r="L37" s="158"/>
-      <c r="M37" s="118"/>
+      <c r="D37" s="80"/>
+      <c r="E37" s="81"/>
+      <c r="F37" s="81"/>
+      <c r="G37" s="81"/>
+      <c r="H37" s="81"/>
+      <c r="I37" s="81"/>
+      <c r="J37" s="81"/>
+      <c r="K37" s="81"/>
+      <c r="L37" s="81"/>
+      <c r="M37" s="82"/>
     </row>
     <row r="38" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="32">
@@ -13096,16 +12576,16 @@
         <v>127</v>
       </c>
       <c r="C38" s="33"/>
-      <c r="D38" s="117"/>
-      <c r="E38" s="158"/>
-      <c r="F38" s="158"/>
-      <c r="G38" s="158"/>
-      <c r="H38" s="158"/>
-      <c r="I38" s="158"/>
-      <c r="J38" s="158"/>
-      <c r="K38" s="158"/>
-      <c r="L38" s="158"/>
-      <c r="M38" s="118"/>
+      <c r="D38" s="80"/>
+      <c r="E38" s="81"/>
+      <c r="F38" s="81"/>
+      <c r="G38" s="81"/>
+      <c r="H38" s="81"/>
+      <c r="I38" s="81"/>
+      <c r="J38" s="81"/>
+      <c r="K38" s="81"/>
+      <c r="L38" s="81"/>
+      <c r="M38" s="82"/>
     </row>
     <row r="39" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="32">
@@ -13115,16 +12595,16 @@
         <v>128</v>
       </c>
       <c r="C39" s="33"/>
-      <c r="D39" s="117"/>
-      <c r="E39" s="158"/>
-      <c r="F39" s="158"/>
-      <c r="G39" s="158"/>
-      <c r="H39" s="158"/>
-      <c r="I39" s="158"/>
-      <c r="J39" s="158"/>
-      <c r="K39" s="158"/>
-      <c r="L39" s="158"/>
-      <c r="M39" s="118"/>
+      <c r="D39" s="80"/>
+      <c r="E39" s="81"/>
+      <c r="F39" s="81"/>
+      <c r="G39" s="81"/>
+      <c r="H39" s="81"/>
+      <c r="I39" s="81"/>
+      <c r="J39" s="81"/>
+      <c r="K39" s="81"/>
+      <c r="L39" s="81"/>
+      <c r="M39" s="82"/>
     </row>
     <row r="40" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="32">
@@ -13134,16 +12614,16 @@
         <v>129</v>
       </c>
       <c r="C40" s="33"/>
-      <c r="D40" s="117"/>
-      <c r="E40" s="158"/>
-      <c r="F40" s="158"/>
-      <c r="G40" s="158"/>
-      <c r="H40" s="158"/>
-      <c r="I40" s="158"/>
-      <c r="J40" s="158"/>
-      <c r="K40" s="158"/>
-      <c r="L40" s="158"/>
-      <c r="M40" s="118"/>
+      <c r="D40" s="80"/>
+      <c r="E40" s="81"/>
+      <c r="F40" s="81"/>
+      <c r="G40" s="81"/>
+      <c r="H40" s="81"/>
+      <c r="I40" s="81"/>
+      <c r="J40" s="81"/>
+      <c r="K40" s="81"/>
+      <c r="L40" s="81"/>
+      <c r="M40" s="82"/>
     </row>
     <row r="41" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="32">
@@ -13153,16 +12633,16 @@
         <v>130</v>
       </c>
       <c r="C41" s="33"/>
-      <c r="D41" s="117"/>
-      <c r="E41" s="158"/>
-      <c r="F41" s="158"/>
-      <c r="G41" s="158"/>
-      <c r="H41" s="158"/>
-      <c r="I41" s="158"/>
-      <c r="J41" s="158"/>
-      <c r="K41" s="158"/>
-      <c r="L41" s="158"/>
-      <c r="M41" s="118"/>
+      <c r="D41" s="80"/>
+      <c r="E41" s="81"/>
+      <c r="F41" s="81"/>
+      <c r="G41" s="81"/>
+      <c r="H41" s="81"/>
+      <c r="I41" s="81"/>
+      <c r="J41" s="81"/>
+      <c r="K41" s="81"/>
+      <c r="L41" s="81"/>
+      <c r="M41" s="82"/>
     </row>
     <row r="42" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="32">
@@ -13172,16 +12652,16 @@
         <v>131</v>
       </c>
       <c r="C42" s="33"/>
-      <c r="D42" s="117"/>
-      <c r="E42" s="158"/>
-      <c r="F42" s="158"/>
-      <c r="G42" s="158"/>
-      <c r="H42" s="158"/>
-      <c r="I42" s="158"/>
-      <c r="J42" s="158"/>
-      <c r="K42" s="158"/>
-      <c r="L42" s="158"/>
-      <c r="M42" s="118"/>
+      <c r="D42" s="80"/>
+      <c r="E42" s="81"/>
+      <c r="F42" s="81"/>
+      <c r="G42" s="81"/>
+      <c r="H42" s="81"/>
+      <c r="I42" s="81"/>
+      <c r="J42" s="81"/>
+      <c r="K42" s="81"/>
+      <c r="L42" s="81"/>
+      <c r="M42" s="82"/>
     </row>
     <row r="43" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="32">
@@ -13191,16 +12671,16 @@
         <v>132</v>
       </c>
       <c r="C43" s="33"/>
-      <c r="D43" s="117"/>
-      <c r="E43" s="158"/>
-      <c r="F43" s="158"/>
-      <c r="G43" s="158"/>
-      <c r="H43" s="158"/>
-      <c r="I43" s="158"/>
-      <c r="J43" s="158"/>
-      <c r="K43" s="158"/>
-      <c r="L43" s="158"/>
-      <c r="M43" s="118"/>
+      <c r="D43" s="80"/>
+      <c r="E43" s="81"/>
+      <c r="F43" s="81"/>
+      <c r="G43" s="81"/>
+      <c r="H43" s="81"/>
+      <c r="I43" s="81"/>
+      <c r="J43" s="81"/>
+      <c r="K43" s="81"/>
+      <c r="L43" s="81"/>
+      <c r="M43" s="82"/>
     </row>
     <row r="44" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="32">
@@ -13210,16 +12690,16 @@
         <v>133</v>
       </c>
       <c r="C44" s="33"/>
-      <c r="D44" s="117"/>
-      <c r="E44" s="158"/>
-      <c r="F44" s="158"/>
-      <c r="G44" s="158"/>
-      <c r="H44" s="158"/>
-      <c r="I44" s="158"/>
-      <c r="J44" s="158"/>
-      <c r="K44" s="158"/>
-      <c r="L44" s="158"/>
-      <c r="M44" s="118"/>
+      <c r="D44" s="80"/>
+      <c r="E44" s="81"/>
+      <c r="F44" s="81"/>
+      <c r="G44" s="81"/>
+      <c r="H44" s="81"/>
+      <c r="I44" s="81"/>
+      <c r="J44" s="81"/>
+      <c r="K44" s="81"/>
+      <c r="L44" s="81"/>
+      <c r="M44" s="82"/>
     </row>
     <row r="45" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="32">
@@ -13229,16 +12709,16 @@
         <v>135</v>
       </c>
       <c r="C45" s="33"/>
-      <c r="D45" s="117"/>
-      <c r="E45" s="158"/>
-      <c r="F45" s="158"/>
-      <c r="G45" s="158"/>
-      <c r="H45" s="158"/>
-      <c r="I45" s="158"/>
-      <c r="J45" s="158"/>
-      <c r="K45" s="158"/>
-      <c r="L45" s="158"/>
-      <c r="M45" s="118"/>
+      <c r="D45" s="80"/>
+      <c r="E45" s="81"/>
+      <c r="F45" s="81"/>
+      <c r="G45" s="81"/>
+      <c r="H45" s="81"/>
+      <c r="I45" s="81"/>
+      <c r="J45" s="81"/>
+      <c r="K45" s="81"/>
+      <c r="L45" s="81"/>
+      <c r="M45" s="82"/>
     </row>
     <row r="46" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="32">
@@ -13248,16 +12728,16 @@
         <v>134</v>
       </c>
       <c r="C46" s="33"/>
-      <c r="D46" s="117"/>
-      <c r="E46" s="158"/>
-      <c r="F46" s="158"/>
-      <c r="G46" s="158"/>
-      <c r="H46" s="158"/>
-      <c r="I46" s="158"/>
-      <c r="J46" s="158"/>
-      <c r="K46" s="158"/>
-      <c r="L46" s="158"/>
-      <c r="M46" s="118"/>
+      <c r="D46" s="80"/>
+      <c r="E46" s="81"/>
+      <c r="F46" s="81"/>
+      <c r="G46" s="81"/>
+      <c r="H46" s="81"/>
+      <c r="I46" s="81"/>
+      <c r="J46" s="81"/>
+      <c r="K46" s="81"/>
+      <c r="L46" s="81"/>
+      <c r="M46" s="82"/>
     </row>
     <row r="47" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="32">
@@ -13267,16 +12747,16 @@
         <v>136</v>
       </c>
       <c r="C47" s="33"/>
-      <c r="D47" s="117"/>
-      <c r="E47" s="158"/>
-      <c r="F47" s="158"/>
-      <c r="G47" s="158"/>
-      <c r="H47" s="158"/>
-      <c r="I47" s="158"/>
-      <c r="J47" s="158"/>
-      <c r="K47" s="158"/>
-      <c r="L47" s="158"/>
-      <c r="M47" s="118"/>
+      <c r="D47" s="80"/>
+      <c r="E47" s="81"/>
+      <c r="F47" s="81"/>
+      <c r="G47" s="81"/>
+      <c r="H47" s="81"/>
+      <c r="I47" s="81"/>
+      <c r="J47" s="81"/>
+      <c r="K47" s="81"/>
+      <c r="L47" s="81"/>
+      <c r="M47" s="82"/>
     </row>
     <row r="48" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="32">
@@ -13286,16 +12766,16 @@
         <v>137</v>
       </c>
       <c r="C48" s="33"/>
-      <c r="D48" s="117"/>
-      <c r="E48" s="158"/>
-      <c r="F48" s="158"/>
-      <c r="G48" s="158"/>
-      <c r="H48" s="158"/>
-      <c r="I48" s="158"/>
-      <c r="J48" s="158"/>
-      <c r="K48" s="158"/>
-      <c r="L48" s="158"/>
-      <c r="M48" s="118"/>
+      <c r="D48" s="80"/>
+      <c r="E48" s="81"/>
+      <c r="F48" s="81"/>
+      <c r="G48" s="81"/>
+      <c r="H48" s="81"/>
+      <c r="I48" s="81"/>
+      <c r="J48" s="81"/>
+      <c r="K48" s="81"/>
+      <c r="L48" s="81"/>
+      <c r="M48" s="82"/>
     </row>
     <row r="49" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="32">
@@ -13305,16 +12785,16 @@
         <v>138</v>
       </c>
       <c r="C49" s="33"/>
-      <c r="D49" s="117"/>
-      <c r="E49" s="158"/>
-      <c r="F49" s="158"/>
-      <c r="G49" s="158"/>
-      <c r="H49" s="158"/>
-      <c r="I49" s="158"/>
-      <c r="J49" s="158"/>
-      <c r="K49" s="158"/>
-      <c r="L49" s="158"/>
-      <c r="M49" s="118"/>
+      <c r="D49" s="80"/>
+      <c r="E49" s="81"/>
+      <c r="F49" s="81"/>
+      <c r="G49" s="81"/>
+      <c r="H49" s="81"/>
+      <c r="I49" s="81"/>
+      <c r="J49" s="81"/>
+      <c r="K49" s="81"/>
+      <c r="L49" s="81"/>
+      <c r="M49" s="82"/>
     </row>
     <row r="50" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="32">
@@ -13324,16 +12804,16 @@
         <v>139</v>
       </c>
       <c r="C50" s="33"/>
-      <c r="D50" s="117"/>
-      <c r="E50" s="158"/>
-      <c r="F50" s="158"/>
-      <c r="G50" s="158"/>
-      <c r="H50" s="158"/>
-      <c r="I50" s="158"/>
-      <c r="J50" s="158"/>
-      <c r="K50" s="158"/>
-      <c r="L50" s="158"/>
-      <c r="M50" s="118"/>
+      <c r="D50" s="80"/>
+      <c r="E50" s="81"/>
+      <c r="F50" s="81"/>
+      <c r="G50" s="81"/>
+      <c r="H50" s="81"/>
+      <c r="I50" s="81"/>
+      <c r="J50" s="81"/>
+      <c r="K50" s="81"/>
+      <c r="L50" s="81"/>
+      <c r="M50" s="82"/>
     </row>
     <row r="51" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="32">
@@ -13343,16 +12823,16 @@
         <v>140</v>
       </c>
       <c r="C51" s="33"/>
-      <c r="D51" s="117"/>
-      <c r="E51" s="158"/>
-      <c r="F51" s="158"/>
-      <c r="G51" s="158"/>
-      <c r="H51" s="158"/>
-      <c r="I51" s="158"/>
-      <c r="J51" s="158"/>
-      <c r="K51" s="158"/>
-      <c r="L51" s="158"/>
-      <c r="M51" s="118"/>
+      <c r="D51" s="80"/>
+      <c r="E51" s="81"/>
+      <c r="F51" s="81"/>
+      <c r="G51" s="81"/>
+      <c r="H51" s="81"/>
+      <c r="I51" s="81"/>
+      <c r="J51" s="81"/>
+      <c r="K51" s="81"/>
+      <c r="L51" s="81"/>
+      <c r="M51" s="82"/>
     </row>
     <row r="52" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="32">
@@ -13362,16 +12842,16 @@
         <v>141</v>
       </c>
       <c r="C52" s="33"/>
-      <c r="D52" s="117"/>
-      <c r="E52" s="158"/>
-      <c r="F52" s="158"/>
-      <c r="G52" s="158"/>
-      <c r="H52" s="158"/>
-      <c r="I52" s="158"/>
-      <c r="J52" s="158"/>
-      <c r="K52" s="158"/>
-      <c r="L52" s="158"/>
-      <c r="M52" s="118"/>
+      <c r="D52" s="80"/>
+      <c r="E52" s="81"/>
+      <c r="F52" s="81"/>
+      <c r="G52" s="81"/>
+      <c r="H52" s="81"/>
+      <c r="I52" s="81"/>
+      <c r="J52" s="81"/>
+      <c r="K52" s="81"/>
+      <c r="L52" s="81"/>
+      <c r="M52" s="82"/>
     </row>
     <row r="53" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="32">
@@ -13381,16 +12861,16 @@
         <v>142</v>
       </c>
       <c r="C53" s="33"/>
-      <c r="D53" s="117"/>
-      <c r="E53" s="158"/>
-      <c r="F53" s="158"/>
-      <c r="G53" s="158"/>
-      <c r="H53" s="158"/>
-      <c r="I53" s="158"/>
-      <c r="J53" s="158"/>
-      <c r="K53" s="158"/>
-      <c r="L53" s="158"/>
-      <c r="M53" s="118"/>
+      <c r="D53" s="80"/>
+      <c r="E53" s="81"/>
+      <c r="F53" s="81"/>
+      <c r="G53" s="81"/>
+      <c r="H53" s="81"/>
+      <c r="I53" s="81"/>
+      <c r="J53" s="81"/>
+      <c r="K53" s="81"/>
+      <c r="L53" s="81"/>
+      <c r="M53" s="82"/>
     </row>
     <row r="54" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="32">
@@ -13400,16 +12880,16 @@
         <v>143</v>
       </c>
       <c r="C54" s="33"/>
-      <c r="D54" s="117"/>
-      <c r="E54" s="158"/>
-      <c r="F54" s="158"/>
-      <c r="G54" s="158"/>
-      <c r="H54" s="158"/>
-      <c r="I54" s="158"/>
-      <c r="J54" s="158"/>
-      <c r="K54" s="158"/>
-      <c r="L54" s="158"/>
-      <c r="M54" s="118"/>
+      <c r="D54" s="80"/>
+      <c r="E54" s="81"/>
+      <c r="F54" s="81"/>
+      <c r="G54" s="81"/>
+      <c r="H54" s="81"/>
+      <c r="I54" s="81"/>
+      <c r="J54" s="81"/>
+      <c r="K54" s="81"/>
+      <c r="L54" s="81"/>
+      <c r="M54" s="82"/>
     </row>
     <row r="55" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="32">
@@ -13419,16 +12899,16 @@
         <v>144</v>
       </c>
       <c r="C55" s="33"/>
-      <c r="D55" s="117"/>
-      <c r="E55" s="158"/>
-      <c r="F55" s="158"/>
-      <c r="G55" s="158"/>
-      <c r="H55" s="158"/>
-      <c r="I55" s="158"/>
-      <c r="J55" s="158"/>
-      <c r="K55" s="158"/>
-      <c r="L55" s="158"/>
-      <c r="M55" s="118"/>
+      <c r="D55" s="80"/>
+      <c r="E55" s="81"/>
+      <c r="F55" s="81"/>
+      <c r="G55" s="81"/>
+      <c r="H55" s="81"/>
+      <c r="I55" s="81"/>
+      <c r="J55" s="81"/>
+      <c r="K55" s="81"/>
+      <c r="L55" s="81"/>
+      <c r="M55" s="82"/>
     </row>
     <row r="56" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="32">
@@ -13438,16 +12918,16 @@
         <v>145</v>
       </c>
       <c r="C56" s="33"/>
-      <c r="D56" s="117"/>
-      <c r="E56" s="158"/>
-      <c r="F56" s="158"/>
-      <c r="G56" s="158"/>
-      <c r="H56" s="158"/>
-      <c r="I56" s="158"/>
-      <c r="J56" s="158"/>
-      <c r="K56" s="158"/>
-      <c r="L56" s="158"/>
-      <c r="M56" s="118"/>
+      <c r="D56" s="80"/>
+      <c r="E56" s="81"/>
+      <c r="F56" s="81"/>
+      <c r="G56" s="81"/>
+      <c r="H56" s="81"/>
+      <c r="I56" s="81"/>
+      <c r="J56" s="81"/>
+      <c r="K56" s="81"/>
+      <c r="L56" s="81"/>
+      <c r="M56" s="82"/>
     </row>
     <row r="57" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="32">
@@ -13457,16 +12937,16 @@
         <v>146</v>
       </c>
       <c r="C57" s="33"/>
-      <c r="D57" s="117"/>
-      <c r="E57" s="158"/>
-      <c r="F57" s="158"/>
-      <c r="G57" s="158"/>
-      <c r="H57" s="158"/>
-      <c r="I57" s="158"/>
-      <c r="J57" s="158"/>
-      <c r="K57" s="158"/>
-      <c r="L57" s="158"/>
-      <c r="M57" s="118"/>
+      <c r="D57" s="80"/>
+      <c r="E57" s="81"/>
+      <c r="F57" s="81"/>
+      <c r="G57" s="81"/>
+      <c r="H57" s="81"/>
+      <c r="I57" s="81"/>
+      <c r="J57" s="81"/>
+      <c r="K57" s="81"/>
+      <c r="L57" s="81"/>
+      <c r="M57" s="82"/>
     </row>
     <row r="58" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="32">
@@ -13476,16 +12956,16 @@
         <v>147</v>
       </c>
       <c r="C58" s="33"/>
-      <c r="D58" s="117"/>
-      <c r="E58" s="158"/>
-      <c r="F58" s="158"/>
-      <c r="G58" s="158"/>
-      <c r="H58" s="158"/>
-      <c r="I58" s="158"/>
-      <c r="J58" s="158"/>
-      <c r="K58" s="158"/>
-      <c r="L58" s="158"/>
-      <c r="M58" s="118"/>
+      <c r="D58" s="80"/>
+      <c r="E58" s="81"/>
+      <c r="F58" s="81"/>
+      <c r="G58" s="81"/>
+      <c r="H58" s="81"/>
+      <c r="I58" s="81"/>
+      <c r="J58" s="81"/>
+      <c r="K58" s="81"/>
+      <c r="L58" s="81"/>
+      <c r="M58" s="82"/>
     </row>
     <row r="59" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="32">
@@ -13495,16 +12975,16 @@
         <v>148</v>
       </c>
       <c r="C59" s="33"/>
-      <c r="D59" s="117"/>
-      <c r="E59" s="158"/>
-      <c r="F59" s="158"/>
-      <c r="G59" s="158"/>
-      <c r="H59" s="158"/>
-      <c r="I59" s="158"/>
-      <c r="J59" s="158"/>
-      <c r="K59" s="158"/>
-      <c r="L59" s="158"/>
-      <c r="M59" s="118"/>
+      <c r="D59" s="80"/>
+      <c r="E59" s="81"/>
+      <c r="F59" s="81"/>
+      <c r="G59" s="81"/>
+      <c r="H59" s="81"/>
+      <c r="I59" s="81"/>
+      <c r="J59" s="81"/>
+      <c r="K59" s="81"/>
+      <c r="L59" s="81"/>
+      <c r="M59" s="82"/>
     </row>
     <row r="60" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="32">
@@ -13514,16 +12994,16 @@
         <v>149</v>
       </c>
       <c r="C60" s="33"/>
-      <c r="D60" s="117"/>
-      <c r="E60" s="158"/>
-      <c r="F60" s="158"/>
-      <c r="G60" s="158"/>
-      <c r="H60" s="158"/>
-      <c r="I60" s="158"/>
-      <c r="J60" s="158"/>
-      <c r="K60" s="158"/>
-      <c r="L60" s="158"/>
-      <c r="M60" s="118"/>
+      <c r="D60" s="80"/>
+      <c r="E60" s="81"/>
+      <c r="F60" s="81"/>
+      <c r="G60" s="81"/>
+      <c r="H60" s="81"/>
+      <c r="I60" s="81"/>
+      <c r="J60" s="81"/>
+      <c r="K60" s="81"/>
+      <c r="L60" s="81"/>
+      <c r="M60" s="82"/>
     </row>
     <row r="61" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="32">
@@ -13533,16 +13013,16 @@
         <v>150</v>
       </c>
       <c r="C61" s="33"/>
-      <c r="D61" s="117"/>
-      <c r="E61" s="158"/>
-      <c r="F61" s="158"/>
-      <c r="G61" s="158"/>
-      <c r="H61" s="158"/>
-      <c r="I61" s="158"/>
-      <c r="J61" s="158"/>
-      <c r="K61" s="158"/>
-      <c r="L61" s="158"/>
-      <c r="M61" s="118"/>
+      <c r="D61" s="80"/>
+      <c r="E61" s="81"/>
+      <c r="F61" s="81"/>
+      <c r="G61" s="81"/>
+      <c r="H61" s="81"/>
+      <c r="I61" s="81"/>
+      <c r="J61" s="81"/>
+      <c r="K61" s="81"/>
+      <c r="L61" s="81"/>
+      <c r="M61" s="82"/>
     </row>
     <row r="62" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="32">
@@ -13552,16 +13032,16 @@
         <v>151</v>
       </c>
       <c r="C62" s="33"/>
-      <c r="D62" s="117"/>
-      <c r="E62" s="158"/>
-      <c r="F62" s="158"/>
-      <c r="G62" s="158"/>
-      <c r="H62" s="158"/>
-      <c r="I62" s="158"/>
-      <c r="J62" s="158"/>
-      <c r="K62" s="158"/>
-      <c r="L62" s="158"/>
-      <c r="M62" s="118"/>
+      <c r="D62" s="80"/>
+      <c r="E62" s="81"/>
+      <c r="F62" s="81"/>
+      <c r="G62" s="81"/>
+      <c r="H62" s="81"/>
+      <c r="I62" s="81"/>
+      <c r="J62" s="81"/>
+      <c r="K62" s="81"/>
+      <c r="L62" s="81"/>
+      <c r="M62" s="82"/>
     </row>
     <row r="63" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="32">
@@ -13571,16 +13051,16 @@
         <v>152</v>
       </c>
       <c r="C63" s="33"/>
-      <c r="D63" s="117"/>
-      <c r="E63" s="158"/>
-      <c r="F63" s="158"/>
-      <c r="G63" s="158"/>
-      <c r="H63" s="158"/>
-      <c r="I63" s="158"/>
-      <c r="J63" s="158"/>
-      <c r="K63" s="158"/>
-      <c r="L63" s="158"/>
-      <c r="M63" s="118"/>
+      <c r="D63" s="80"/>
+      <c r="E63" s="81"/>
+      <c r="F63" s="81"/>
+      <c r="G63" s="81"/>
+      <c r="H63" s="81"/>
+      <c r="I63" s="81"/>
+      <c r="J63" s="81"/>
+      <c r="K63" s="81"/>
+      <c r="L63" s="81"/>
+      <c r="M63" s="82"/>
     </row>
     <row r="64" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="32">
@@ -13590,16 +13070,16 @@
         <v>153</v>
       </c>
       <c r="C64" s="33"/>
-      <c r="D64" s="117"/>
-      <c r="E64" s="158"/>
-      <c r="F64" s="158"/>
-      <c r="G64" s="158"/>
-      <c r="H64" s="158"/>
-      <c r="I64" s="158"/>
-      <c r="J64" s="158"/>
-      <c r="K64" s="158"/>
-      <c r="L64" s="158"/>
-      <c r="M64" s="118"/>
+      <c r="D64" s="80"/>
+      <c r="E64" s="81"/>
+      <c r="F64" s="81"/>
+      <c r="G64" s="81"/>
+      <c r="H64" s="81"/>
+      <c r="I64" s="81"/>
+      <c r="J64" s="81"/>
+      <c r="K64" s="81"/>
+      <c r="L64" s="81"/>
+      <c r="M64" s="82"/>
     </row>
     <row r="65" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="32">
@@ -13609,16 +13089,16 @@
         <v>154</v>
       </c>
       <c r="C65" s="33"/>
-      <c r="D65" s="117"/>
-      <c r="E65" s="158"/>
-      <c r="F65" s="158"/>
-      <c r="G65" s="158"/>
-      <c r="H65" s="158"/>
-      <c r="I65" s="158"/>
-      <c r="J65" s="158"/>
-      <c r="K65" s="158"/>
-      <c r="L65" s="158"/>
-      <c r="M65" s="118"/>
+      <c r="D65" s="80"/>
+      <c r="E65" s="81"/>
+      <c r="F65" s="81"/>
+      <c r="G65" s="81"/>
+      <c r="H65" s="81"/>
+      <c r="I65" s="81"/>
+      <c r="J65" s="81"/>
+      <c r="K65" s="81"/>
+      <c r="L65" s="81"/>
+      <c r="M65" s="82"/>
     </row>
     <row r="66" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="32">
@@ -13628,16 +13108,16 @@
         <v>155</v>
       </c>
       <c r="C66" s="33"/>
-      <c r="D66" s="117"/>
-      <c r="E66" s="158"/>
-      <c r="F66" s="158"/>
-      <c r="G66" s="158"/>
-      <c r="H66" s="158"/>
-      <c r="I66" s="158"/>
-      <c r="J66" s="158"/>
-      <c r="K66" s="158"/>
-      <c r="L66" s="158"/>
-      <c r="M66" s="118"/>
+      <c r="D66" s="80"/>
+      <c r="E66" s="81"/>
+      <c r="F66" s="81"/>
+      <c r="G66" s="81"/>
+      <c r="H66" s="81"/>
+      <c r="I66" s="81"/>
+      <c r="J66" s="81"/>
+      <c r="K66" s="81"/>
+      <c r="L66" s="81"/>
+      <c r="M66" s="82"/>
     </row>
     <row r="67" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="32">
@@ -13647,16 +13127,16 @@
         <v>156</v>
       </c>
       <c r="C67" s="33"/>
-      <c r="D67" s="117"/>
-      <c r="E67" s="158"/>
-      <c r="F67" s="158"/>
-      <c r="G67" s="158"/>
-      <c r="H67" s="158"/>
-      <c r="I67" s="158"/>
-      <c r="J67" s="158"/>
-      <c r="K67" s="158"/>
-      <c r="L67" s="158"/>
-      <c r="M67" s="118"/>
+      <c r="D67" s="80"/>
+      <c r="E67" s="81"/>
+      <c r="F67" s="81"/>
+      <c r="G67" s="81"/>
+      <c r="H67" s="81"/>
+      <c r="I67" s="81"/>
+      <c r="J67" s="81"/>
+      <c r="K67" s="81"/>
+      <c r="L67" s="81"/>
+      <c r="M67" s="82"/>
     </row>
     <row r="68" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="32">
@@ -13666,16 +13146,16 @@
         <v>157</v>
       </c>
       <c r="C68" s="33"/>
-      <c r="D68" s="117"/>
-      <c r="E68" s="158"/>
-      <c r="F68" s="158"/>
-      <c r="G68" s="158"/>
-      <c r="H68" s="158"/>
-      <c r="I68" s="158"/>
-      <c r="J68" s="158"/>
-      <c r="K68" s="158"/>
-      <c r="L68" s="158"/>
-      <c r="M68" s="118"/>
+      <c r="D68" s="80"/>
+      <c r="E68" s="81"/>
+      <c r="F68" s="81"/>
+      <c r="G68" s="81"/>
+      <c r="H68" s="81"/>
+      <c r="I68" s="81"/>
+      <c r="J68" s="81"/>
+      <c r="K68" s="81"/>
+      <c r="L68" s="81"/>
+      <c r="M68" s="82"/>
     </row>
     <row r="69" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="32">
@@ -13685,16 +13165,16 @@
         <v>158</v>
       </c>
       <c r="C69" s="33"/>
-      <c r="D69" s="117"/>
-      <c r="E69" s="158"/>
-      <c r="F69" s="158"/>
-      <c r="G69" s="158"/>
-      <c r="H69" s="158"/>
-      <c r="I69" s="158"/>
-      <c r="J69" s="158"/>
-      <c r="K69" s="158"/>
-      <c r="L69" s="158"/>
-      <c r="M69" s="118"/>
+      <c r="D69" s="80"/>
+      <c r="E69" s="81"/>
+      <c r="F69" s="81"/>
+      <c r="G69" s="81"/>
+      <c r="H69" s="81"/>
+      <c r="I69" s="81"/>
+      <c r="J69" s="81"/>
+      <c r="K69" s="81"/>
+      <c r="L69" s="81"/>
+      <c r="M69" s="82"/>
     </row>
     <row r="70" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="32">
@@ -13704,16 +13184,16 @@
         <v>159</v>
       </c>
       <c r="C70" s="33"/>
-      <c r="D70" s="117"/>
-      <c r="E70" s="158"/>
-      <c r="F70" s="158"/>
-      <c r="G70" s="158"/>
-      <c r="H70" s="158"/>
-      <c r="I70" s="158"/>
-      <c r="J70" s="158"/>
-      <c r="K70" s="158"/>
-      <c r="L70" s="158"/>
-      <c r="M70" s="118"/>
+      <c r="D70" s="80"/>
+      <c r="E70" s="81"/>
+      <c r="F70" s="81"/>
+      <c r="G70" s="81"/>
+      <c r="H70" s="81"/>
+      <c r="I70" s="81"/>
+      <c r="J70" s="81"/>
+      <c r="K70" s="81"/>
+      <c r="L70" s="81"/>
+      <c r="M70" s="82"/>
     </row>
     <row r="71" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="32">
@@ -13723,16 +13203,16 @@
         <v>160</v>
       </c>
       <c r="C71" s="33"/>
-      <c r="D71" s="117"/>
-      <c r="E71" s="158"/>
-      <c r="F71" s="158"/>
-      <c r="G71" s="158"/>
-      <c r="H71" s="158"/>
-      <c r="I71" s="158"/>
-      <c r="J71" s="158"/>
-      <c r="K71" s="158"/>
-      <c r="L71" s="158"/>
-      <c r="M71" s="118"/>
+      <c r="D71" s="80"/>
+      <c r="E71" s="81"/>
+      <c r="F71" s="81"/>
+      <c r="G71" s="81"/>
+      <c r="H71" s="81"/>
+      <c r="I71" s="81"/>
+      <c r="J71" s="81"/>
+      <c r="K71" s="81"/>
+      <c r="L71" s="81"/>
+      <c r="M71" s="82"/>
     </row>
     <row r="72" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="32">
@@ -13742,16 +13222,16 @@
         <v>161</v>
       </c>
       <c r="C72" s="33"/>
-      <c r="D72" s="117"/>
-      <c r="E72" s="158"/>
-      <c r="F72" s="158"/>
-      <c r="G72" s="158"/>
-      <c r="H72" s="158"/>
-      <c r="I72" s="158"/>
-      <c r="J72" s="158"/>
-      <c r="K72" s="158"/>
-      <c r="L72" s="158"/>
-      <c r="M72" s="118"/>
+      <c r="D72" s="80"/>
+      <c r="E72" s="81"/>
+      <c r="F72" s="81"/>
+      <c r="G72" s="81"/>
+      <c r="H72" s="81"/>
+      <c r="I72" s="81"/>
+      <c r="J72" s="81"/>
+      <c r="K72" s="81"/>
+      <c r="L72" s="81"/>
+      <c r="M72" s="82"/>
     </row>
     <row r="73" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="32">
@@ -13761,176 +13241,146 @@
         <v>162</v>
       </c>
       <c r="C73" s="33"/>
-      <c r="D73" s="117"/>
-      <c r="E73" s="158"/>
-      <c r="F73" s="158"/>
-      <c r="G73" s="158"/>
-      <c r="H73" s="158"/>
-      <c r="I73" s="158"/>
-      <c r="J73" s="158"/>
-      <c r="K73" s="158"/>
-      <c r="L73" s="158"/>
-      <c r="M73" s="118"/>
+      <c r="D73" s="80"/>
+      <c r="E73" s="81"/>
+      <c r="F73" s="81"/>
+      <c r="G73" s="81"/>
+      <c r="H73" s="81"/>
+      <c r="I73" s="81"/>
+      <c r="J73" s="81"/>
+      <c r="K73" s="81"/>
+      <c r="L73" s="81"/>
+      <c r="M73" s="82"/>
     </row>
     <row r="74" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="32">
-        <v>49</v>
-      </c>
-      <c r="B74" s="33" t="s">
-        <v>163</v>
-      </c>
+      <c r="A74" s="32"/>
+      <c r="B74" s="33"/>
       <c r="C74" s="33"/>
-      <c r="D74" s="117"/>
-      <c r="E74" s="158"/>
-      <c r="F74" s="158"/>
-      <c r="G74" s="158"/>
-      <c r="H74" s="158"/>
-      <c r="I74" s="158"/>
-      <c r="J74" s="158"/>
-      <c r="K74" s="158"/>
-      <c r="L74" s="158"/>
-      <c r="M74" s="118"/>
+      <c r="D74" s="80"/>
+      <c r="E74" s="81"/>
+      <c r="F74" s="81"/>
+      <c r="G74" s="81"/>
+      <c r="H74" s="81"/>
+      <c r="I74" s="81"/>
+      <c r="J74" s="81"/>
+      <c r="K74" s="81"/>
+      <c r="L74" s="81"/>
+      <c r="M74" s="82"/>
     </row>
     <row r="75" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="32">
-        <v>50</v>
-      </c>
-      <c r="B75" s="33" t="s">
-        <v>164</v>
-      </c>
+      <c r="A75" s="32"/>
+      <c r="B75" s="33"/>
       <c r="C75" s="33"/>
-      <c r="D75" s="117"/>
-      <c r="E75" s="158"/>
-      <c r="F75" s="158"/>
-      <c r="G75" s="158"/>
-      <c r="H75" s="158"/>
-      <c r="I75" s="158"/>
-      <c r="J75" s="158"/>
-      <c r="K75" s="158"/>
-      <c r="L75" s="158"/>
-      <c r="M75" s="118"/>
+      <c r="D75" s="80"/>
+      <c r="E75" s="81"/>
+      <c r="F75" s="81"/>
+      <c r="G75" s="81"/>
+      <c r="H75" s="81"/>
+      <c r="I75" s="81"/>
+      <c r="J75" s="81"/>
+      <c r="K75" s="81"/>
+      <c r="L75" s="81"/>
+      <c r="M75" s="82"/>
     </row>
     <row r="76" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="32">
-        <v>51</v>
-      </c>
-      <c r="B76" s="33" t="s">
-        <v>165</v>
-      </c>
+      <c r="A76" s="32"/>
+      <c r="B76" s="33"/>
       <c r="C76" s="33"/>
-      <c r="D76" s="117"/>
-      <c r="E76" s="158"/>
-      <c r="F76" s="158"/>
-      <c r="G76" s="158"/>
-      <c r="H76" s="158"/>
-      <c r="I76" s="158"/>
-      <c r="J76" s="158"/>
-      <c r="K76" s="158"/>
-      <c r="L76" s="158"/>
-      <c r="M76" s="118"/>
+      <c r="D76" s="80"/>
+      <c r="E76" s="81"/>
+      <c r="F76" s="81"/>
+      <c r="G76" s="81"/>
+      <c r="H76" s="81"/>
+      <c r="I76" s="81"/>
+      <c r="J76" s="81"/>
+      <c r="K76" s="81"/>
+      <c r="L76" s="81"/>
+      <c r="M76" s="82"/>
     </row>
     <row r="77" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="32">
-        <v>52</v>
-      </c>
-      <c r="B77" s="33" t="s">
-        <v>166</v>
-      </c>
+      <c r="A77" s="32"/>
+      <c r="B77" s="33"/>
       <c r="C77" s="33"/>
-      <c r="D77" s="117"/>
-      <c r="E77" s="158"/>
-      <c r="F77" s="158"/>
-      <c r="G77" s="158"/>
-      <c r="H77" s="158"/>
-      <c r="I77" s="158"/>
-      <c r="J77" s="158"/>
-      <c r="K77" s="158"/>
-      <c r="L77" s="158"/>
-      <c r="M77" s="118"/>
+      <c r="D77" s="80"/>
+      <c r="E77" s="81"/>
+      <c r="F77" s="81"/>
+      <c r="G77" s="81"/>
+      <c r="H77" s="81"/>
+      <c r="I77" s="81"/>
+      <c r="J77" s="81"/>
+      <c r="K77" s="81"/>
+      <c r="L77" s="81"/>
+      <c r="M77" s="82"/>
     </row>
     <row r="78" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="32">
-        <v>53</v>
-      </c>
-      <c r="B78" s="33" t="s">
-        <v>167</v>
-      </c>
+      <c r="A78" s="32"/>
+      <c r="B78" s="33"/>
       <c r="C78" s="33"/>
-      <c r="D78" s="117"/>
-      <c r="E78" s="158"/>
-      <c r="F78" s="158"/>
-      <c r="G78" s="158"/>
-      <c r="H78" s="158"/>
-      <c r="I78" s="158"/>
-      <c r="J78" s="158"/>
-      <c r="K78" s="158"/>
-      <c r="L78" s="158"/>
-      <c r="M78" s="118"/>
+      <c r="D78" s="80"/>
+      <c r="E78" s="81"/>
+      <c r="F78" s="81"/>
+      <c r="G78" s="81"/>
+      <c r="H78" s="81"/>
+      <c r="I78" s="81"/>
+      <c r="J78" s="81"/>
+      <c r="K78" s="81"/>
+      <c r="L78" s="81"/>
+      <c r="M78" s="82"/>
     </row>
     <row r="79" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="32">
-        <v>54</v>
-      </c>
-      <c r="B79" s="33" t="s">
-        <v>168</v>
-      </c>
+      <c r="A79" s="32"/>
+      <c r="B79" s="33"/>
       <c r="C79" s="33"/>
-      <c r="D79" s="117"/>
-      <c r="E79" s="158"/>
-      <c r="F79" s="158"/>
-      <c r="G79" s="158"/>
-      <c r="H79" s="158"/>
-      <c r="I79" s="158"/>
-      <c r="J79" s="158"/>
-      <c r="K79" s="158"/>
-      <c r="L79" s="158"/>
-      <c r="M79" s="118"/>
+      <c r="D79" s="80"/>
+      <c r="E79" s="81"/>
+      <c r="F79" s="81"/>
+      <c r="G79" s="81"/>
+      <c r="H79" s="81"/>
+      <c r="I79" s="81"/>
+      <c r="J79" s="81"/>
+      <c r="K79" s="81"/>
+      <c r="L79" s="81"/>
+      <c r="M79" s="82"/>
     </row>
     <row r="80" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="32">
-        <v>55</v>
-      </c>
-      <c r="B80" s="33" t="s">
-        <v>169</v>
-      </c>
+      <c r="A80" s="32"/>
+      <c r="B80" s="33"/>
       <c r="C80" s="33"/>
-      <c r="D80" s="117"/>
-      <c r="E80" s="158"/>
-      <c r="F80" s="158"/>
-      <c r="G80" s="158"/>
-      <c r="H80" s="158"/>
-      <c r="I80" s="158"/>
-      <c r="J80" s="158"/>
-      <c r="K80" s="158"/>
-      <c r="L80" s="158"/>
-      <c r="M80" s="118"/>
+      <c r="D80" s="80"/>
+      <c r="E80" s="81"/>
+      <c r="F80" s="81"/>
+      <c r="G80" s="81"/>
+      <c r="H80" s="81"/>
+      <c r="I80" s="81"/>
+      <c r="J80" s="81"/>
+      <c r="K80" s="81"/>
+      <c r="L80" s="81"/>
+      <c r="M80" s="82"/>
     </row>
     <row r="81" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="157">
-        <v>56</v>
-      </c>
-      <c r="B81" s="33" t="s">
-        <v>170</v>
-      </c>
+      <c r="A81" s="76"/>
+      <c r="B81" s="33"/>
       <c r="C81" s="33"/>
-      <c r="D81" s="119"/>
-      <c r="E81" s="120"/>
-      <c r="F81" s="120"/>
-      <c r="G81" s="120"/>
-      <c r="H81" s="120"/>
-      <c r="I81" s="120"/>
-      <c r="J81" s="120"/>
-      <c r="K81" s="120"/>
-      <c r="L81" s="120"/>
-      <c r="M81" s="121"/>
+      <c r="D81" s="83"/>
+      <c r="E81" s="84"/>
+      <c r="F81" s="84"/>
+      <c r="G81" s="84"/>
+      <c r="H81" s="84"/>
+      <c r="I81" s="84"/>
+      <c r="J81" s="84"/>
+      <c r="K81" s="84"/>
+      <c r="L81" s="84"/>
+      <c r="M81" s="85"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="D25:M25"/>
-    <mergeCell ref="A23:M23"/>
-    <mergeCell ref="A24:M24"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:M22"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="B6:M6"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="B7:M7"/>
     <mergeCell ref="D26:M81"/>
     <mergeCell ref="A16:M16"/>
     <mergeCell ref="A17:M17"/>
@@ -13938,13 +13388,11 @@
     <mergeCell ref="B15:M15"/>
     <mergeCell ref="D18:D20"/>
     <mergeCell ref="E18:M20"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="B6:M6"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A9:M9"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="B5:M5"/>
-    <mergeCell ref="B7:M7"/>
+    <mergeCell ref="D25:M25"/>
+    <mergeCell ref="A23:M23"/>
+    <mergeCell ref="A24:M24"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:M22"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
@@ -17162,182 +16610,6 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>1440180</xdr:colOff>
                     <xdr:row>73</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1274" r:id="rId151" name="Drop Down 250">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>30480</xdr:colOff>
-                    <xdr:row>73</xdr:row>
-                    <xdr:rowOff>22860</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1440180</xdr:colOff>
-                    <xdr:row>74</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1275" r:id="rId152" name="Drop Down 251">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>30480</xdr:colOff>
-                    <xdr:row>74</xdr:row>
-                    <xdr:rowOff>22860</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1440180</xdr:colOff>
-                    <xdr:row>75</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1276" r:id="rId153" name="Drop Down 252">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>30480</xdr:colOff>
-                    <xdr:row>75</xdr:row>
-                    <xdr:rowOff>22860</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1440180</xdr:colOff>
-                    <xdr:row>76</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1277" r:id="rId154" name="Drop Down 253">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>30480</xdr:colOff>
-                    <xdr:row>76</xdr:row>
-                    <xdr:rowOff>22860</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1440180</xdr:colOff>
-                    <xdr:row>77</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1278" r:id="rId155" name="Drop Down 254">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>30480</xdr:colOff>
-                    <xdr:row>77</xdr:row>
-                    <xdr:rowOff>22860</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1440180</xdr:colOff>
-                    <xdr:row>78</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1279" r:id="rId156" name="Drop Down 255">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>30480</xdr:colOff>
-                    <xdr:row>78</xdr:row>
-                    <xdr:rowOff>22860</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1440180</xdr:colOff>
-                    <xdr:row>79</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1280" r:id="rId157" name="Drop Down 256">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>30480</xdr:colOff>
-                    <xdr:row>79</xdr:row>
-                    <xdr:rowOff>22860</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1440180</xdr:colOff>
-                    <xdr:row>80</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1281" r:id="rId158" name="Drop Down 257">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>30480</xdr:colOff>
-                    <xdr:row>80</xdr:row>
-                    <xdr:rowOff>22860</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1440180</xdr:colOff>
-                    <xdr:row>81</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
                 </anchor>
@@ -17368,50 +16640,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="135" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="134"/>
-      <c r="C1" s="134"/>
-      <c r="D1" s="134"/>
-      <c r="E1" s="134"/>
-      <c r="F1" s="134"/>
-      <c r="G1" s="134"/>
-      <c r="H1" s="134"/>
-      <c r="I1" s="134"/>
-      <c r="J1" s="134"/>
-      <c r="K1" s="134"/>
-      <c r="L1" s="135"/>
+      <c r="B1" s="136"/>
+      <c r="C1" s="136"/>
+      <c r="D1" s="136"/>
+      <c r="E1" s="136"/>
+      <c r="F1" s="136"/>
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="136"/>
+      <c r="J1" s="136"/>
+      <c r="K1" s="136"/>
+      <c r="L1" s="137"/>
     </row>
     <row r="2" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="136" t="s">
+      <c r="A2" s="138" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="137"/>
-      <c r="C2" s="137"/>
-      <c r="D2" s="137"/>
-      <c r="E2" s="137"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="137"/>
-      <c r="H2" s="137"/>
-      <c r="I2" s="137"/>
-      <c r="J2" s="137"/>
-      <c r="K2" s="137"/>
-      <c r="L2" s="138"/>
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="139"/>
+      <c r="I2" s="139"/>
+      <c r="J2" s="139"/>
+      <c r="K2" s="139"/>
+      <c r="L2" s="140"/>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="139"/>
-      <c r="B3" s="140"/>
-      <c r="C3" s="140"/>
-      <c r="D3" s="140"/>
-      <c r="E3" s="140"/>
-      <c r="F3" s="140"/>
-      <c r="G3" s="140"/>
-      <c r="H3" s="140"/>
-      <c r="I3" s="140"/>
-      <c r="J3" s="140"/>
-      <c r="K3" s="140"/>
-      <c r="L3" s="141"/>
+      <c r="A3" s="141"/>
+      <c r="B3" s="142"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="143"/>
     </row>
     <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -17501,65 +16773,65 @@
       <c r="A8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="144"/>
-      <c r="C8" s="145"/>
-      <c r="D8" s="145"/>
-      <c r="E8" s="145"/>
-      <c r="F8" s="145"/>
-      <c r="G8" s="145"/>
-      <c r="H8" s="145"/>
-      <c r="I8" s="145"/>
-      <c r="J8" s="145"/>
-      <c r="K8" s="145"/>
-      <c r="L8" s="146"/>
+      <c r="B8" s="146"/>
+      <c r="C8" s="147"/>
+      <c r="D8" s="147"/>
+      <c r="E8" s="147"/>
+      <c r="F8" s="147"/>
+      <c r="G8" s="147"/>
+      <c r="H8" s="147"/>
+      <c r="I8" s="147"/>
+      <c r="J8" s="147"/>
+      <c r="K8" s="147"/>
+      <c r="L8" s="148"/>
     </row>
     <row r="9" spans="1:12" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="147"/>
-      <c r="C9" s="145"/>
-      <c r="D9" s="145"/>
-      <c r="E9" s="145"/>
-      <c r="F9" s="145"/>
-      <c r="G9" s="145"/>
-      <c r="H9" s="145"/>
-      <c r="I9" s="145"/>
-      <c r="J9" s="145"/>
-      <c r="K9" s="145"/>
-      <c r="L9" s="146"/>
+      <c r="B9" s="149"/>
+      <c r="C9" s="147"/>
+      <c r="D9" s="147"/>
+      <c r="E9" s="147"/>
+      <c r="F9" s="147"/>
+      <c r="G9" s="147"/>
+      <c r="H9" s="147"/>
+      <c r="I9" s="147"/>
+      <c r="J9" s="147"/>
+      <c r="K9" s="147"/>
+      <c r="L9" s="148"/>
     </row>
     <row r="10" spans="1:12" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="142" t="s">
+      <c r="A10" s="144" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="143"/>
-      <c r="C10" s="143"/>
-      <c r="D10" s="143"/>
-      <c r="E10" s="143"/>
-      <c r="F10" s="143"/>
-      <c r="G10" s="143"/>
-      <c r="H10" s="143"/>
-      <c r="I10" s="143"/>
-      <c r="J10" s="143"/>
-      <c r="K10" s="143"/>
-      <c r="L10" s="143"/>
+      <c r="B10" s="145"/>
+      <c r="C10" s="145"/>
+      <c r="D10" s="145"/>
+      <c r="E10" s="145"/>
+      <c r="F10" s="145"/>
+      <c r="G10" s="145"/>
+      <c r="H10" s="145"/>
+      <c r="I10" s="145"/>
+      <c r="J10" s="145"/>
+      <c r="K10" s="145"/>
+      <c r="L10" s="145"/>
     </row>
     <row r="11" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="124" t="s">
+      <c r="A11" s="126" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="125"/>
-      <c r="C11" s="125"/>
-      <c r="D11" s="125"/>
-      <c r="E11" s="125"/>
-      <c r="F11" s="125"/>
-      <c r="G11" s="125"/>
-      <c r="H11" s="125"/>
-      <c r="I11" s="125"/>
-      <c r="J11" s="125"/>
-      <c r="K11" s="125"/>
-      <c r="L11" s="126"/>
+      <c r="B11" s="127"/>
+      <c r="C11" s="127"/>
+      <c r="D11" s="127"/>
+      <c r="E11" s="127"/>
+      <c r="F11" s="127"/>
+      <c r="G11" s="127"/>
+      <c r="H11" s="127"/>
+      <c r="I11" s="127"/>
+      <c r="J11" s="127"/>
+      <c r="K11" s="127"/>
+      <c r="L11" s="128"/>
     </row>
     <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
@@ -17571,101 +16843,101 @@
       <c r="C12" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="106" t="s">
+      <c r="D12" s="99" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="106"/>
-      <c r="F12" s="106"/>
-      <c r="G12" s="106"/>
-      <c r="H12" s="106"/>
-      <c r="I12" s="106"/>
-      <c r="J12" s="106"/>
-      <c r="K12" s="106"/>
-      <c r="L12" s="106"/>
+      <c r="E12" s="99"/>
+      <c r="F12" s="99"/>
+      <c r="G12" s="99"/>
+      <c r="H12" s="99"/>
+      <c r="I12" s="99"/>
+      <c r="J12" s="99"/>
+      <c r="K12" s="99"/>
+      <c r="L12" s="99"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="48"/>
       <c r="B13" s="49"/>
       <c r="C13" s="49"/>
-      <c r="D13" s="127"/>
-      <c r="E13" s="128"/>
-      <c r="F13" s="128"/>
-      <c r="G13" s="128"/>
-      <c r="H13" s="128"/>
-      <c r="I13" s="128"/>
-      <c r="J13" s="128"/>
-      <c r="K13" s="128"/>
-      <c r="L13" s="129"/>
+      <c r="D13" s="129"/>
+      <c r="E13" s="130"/>
+      <c r="F13" s="130"/>
+      <c r="G13" s="130"/>
+      <c r="H13" s="130"/>
+      <c r="I13" s="130"/>
+      <c r="J13" s="130"/>
+      <c r="K13" s="130"/>
+      <c r="L13" s="131"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="48"/>
       <c r="B14" s="49"/>
       <c r="C14" s="49"/>
-      <c r="D14" s="130"/>
-      <c r="E14" s="131"/>
-      <c r="F14" s="131"/>
-      <c r="G14" s="131"/>
-      <c r="H14" s="131"/>
-      <c r="I14" s="131"/>
-      <c r="J14" s="131"/>
-      <c r="K14" s="131"/>
-      <c r="L14" s="132"/>
+      <c r="D14" s="132"/>
+      <c r="E14" s="133"/>
+      <c r="F14" s="133"/>
+      <c r="G14" s="133"/>
+      <c r="H14" s="133"/>
+      <c r="I14" s="133"/>
+      <c r="J14" s="133"/>
+      <c r="K14" s="133"/>
+      <c r="L14" s="134"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="48"/>
       <c r="B15" s="49"/>
       <c r="C15" s="49"/>
-      <c r="D15" s="130"/>
-      <c r="E15" s="131"/>
-      <c r="F15" s="131"/>
-      <c r="G15" s="131"/>
-      <c r="H15" s="131"/>
-      <c r="I15" s="131"/>
-      <c r="J15" s="131"/>
-      <c r="K15" s="131"/>
-      <c r="L15" s="132"/>
+      <c r="D15" s="132"/>
+      <c r="E15" s="133"/>
+      <c r="F15" s="133"/>
+      <c r="G15" s="133"/>
+      <c r="H15" s="133"/>
+      <c r="I15" s="133"/>
+      <c r="J15" s="133"/>
+      <c r="K15" s="133"/>
+      <c r="L15" s="134"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="48"/>
       <c r="B16" s="49"/>
       <c r="C16" s="49"/>
-      <c r="D16" s="130"/>
-      <c r="E16" s="131"/>
-      <c r="F16" s="131"/>
-      <c r="G16" s="131"/>
-      <c r="H16" s="131"/>
-      <c r="I16" s="131"/>
-      <c r="J16" s="131"/>
-      <c r="K16" s="131"/>
-      <c r="L16" s="132"/>
+      <c r="D16" s="132"/>
+      <c r="E16" s="133"/>
+      <c r="F16" s="133"/>
+      <c r="G16" s="133"/>
+      <c r="H16" s="133"/>
+      <c r="I16" s="133"/>
+      <c r="J16" s="133"/>
+      <c r="K16" s="133"/>
+      <c r="L16" s="134"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="48"/>
       <c r="B17" s="49"/>
       <c r="C17" s="49"/>
-      <c r="D17" s="130"/>
-      <c r="E17" s="131"/>
-      <c r="F17" s="131"/>
-      <c r="G17" s="131"/>
-      <c r="H17" s="131"/>
-      <c r="I17" s="131"/>
-      <c r="J17" s="131"/>
-      <c r="K17" s="131"/>
-      <c r="L17" s="132"/>
+      <c r="D17" s="132"/>
+      <c r="E17" s="133"/>
+      <c r="F17" s="133"/>
+      <c r="G17" s="133"/>
+      <c r="H17" s="133"/>
+      <c r="I17" s="133"/>
+      <c r="J17" s="133"/>
+      <c r="K17" s="133"/>
+      <c r="L17" s="134"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="48"/>
       <c r="B18" s="49"/>
       <c r="C18" s="49"/>
-      <c r="D18" s="130"/>
-      <c r="E18" s="131"/>
-      <c r="F18" s="131"/>
-      <c r="G18" s="131"/>
-      <c r="H18" s="131"/>
-      <c r="I18" s="131"/>
-      <c r="J18" s="131"/>
-      <c r="K18" s="131"/>
-      <c r="L18" s="132"/>
+      <c r="D18" s="132"/>
+      <c r="E18" s="133"/>
+      <c r="F18" s="133"/>
+      <c r="G18" s="133"/>
+      <c r="H18" s="133"/>
+      <c r="I18" s="133"/>
+      <c r="J18" s="133"/>
+      <c r="K18" s="133"/>
+      <c r="L18" s="134"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -17754,10 +17026,10 @@
       <c r="B4" s="62"/>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="148" t="s">
+      <c r="A6" s="150" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="148"/>
+      <c r="B6" s="150"/>
     </row>
     <row r="8" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="65" t="s">
@@ -17916,53 +17188,53 @@
   <sheetData>
     <row r="1" spans="2:6" ht="5.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B2" s="150"/>
-      <c r="C2" s="150"/>
-      <c r="D2" s="151" t="s">
+      <c r="B2" s="152"/>
+      <c r="C2" s="152"/>
+      <c r="D2" s="153" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="152" t="s">
+      <c r="E2" s="154" t="s">
         <v>49</v>
       </c>
-      <c r="F2" s="152"/>
+      <c r="F2" s="154"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="150"/>
-      <c r="C3" s="150"/>
-      <c r="D3" s="151"/>
-      <c r="E3" s="152"/>
-      <c r="F3" s="152"/>
+      <c r="B3" s="152"/>
+      <c r="C3" s="152"/>
+      <c r="D3" s="153"/>
+      <c r="E3" s="154"/>
+      <c r="F3" s="154"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="150"/>
-      <c r="C4" s="150"/>
-      <c r="D4" s="151"/>
-      <c r="E4" s="152" t="s">
+      <c r="B4" s="152"/>
+      <c r="C4" s="152"/>
+      <c r="D4" s="153"/>
+      <c r="E4" s="154" t="s">
         <v>108</v>
       </c>
-      <c r="F4" s="152"/>
+      <c r="F4" s="154"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="153" t="s">
+      <c r="B5" s="155" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="153"/>
+      <c r="C5" s="155"/>
       <c r="D5" s="69" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="154" t="s">
+      <c r="E5" s="156" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="154"/>
+      <c r="F5" s="156"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="71" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="149"/>
-      <c r="D6" s="149"/>
-      <c r="E6" s="149"/>
-      <c r="F6" s="149"/>
+      <c r="C6" s="151"/>
+      <c r="D6" s="151"/>
+      <c r="E6" s="151"/>
+      <c r="F6" s="151"/>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="70" t="s">
@@ -18217,10 +17489,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="26" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="155" t="s">
+      <c r="A1" s="157" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="156"/>
+      <c r="B1" s="158"/>
     </row>
     <row r="2" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="27" t="s">
@@ -18491,12 +17763,56 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
+      <UserInfo>
+        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
+        <AccountId>265</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
+        <AccountId>322</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
+        <AccountId>304</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
+        <AccountId>299</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
+        <AccountId>369</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
+        <AccountId>355</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
+        <AccountId>321</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
+        <AccountId>370</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18749,62 +18065,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
-      <UserInfo>
-        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
-        <AccountId>265</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
-        <AccountId>322</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
-        <AccountId>304</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
-        <AccountId>299</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
-        <AccountId>369</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
-        <AccountId>355</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
-        <AccountId>321</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
-        <AccountId>370</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
+    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -18829,12 +18104,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
-    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix modificacion de sp
</commit_message>
<xml_diff>
--- a/Guias Produccion/HU-55188.xlsx
+++ b/Guias Produccion/HU-55188.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Alliance\ScriptsEntidades\Guias Produccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8367990A-B46E-4B68-8486-143D9D19443A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{317B416B-0D47-47D1-8081-2D2A87BC03A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="164">
   <si>
     <t>Guia documentación</t>
   </si>
@@ -652,6 +652,9 @@
   </si>
   <si>
     <t>48-UpdateOpcionesRetraso.sql</t>
+  </si>
+  <si>
+    <t>49-UpdateIdiomas.sql</t>
   </si>
 </sst>
 </file>
@@ -1796,7 +1799,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2194,6 +2197,9 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="45" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -2425,10 +2431,14 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp147.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp148.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
-<file path=xl/ctrlProps/ctrlProp148.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ctrlProps/ctrlProp149.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
@@ -11240,6 +11250,64 @@
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
                   <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000F9040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:noFill/>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>30480</xdr:colOff>
+          <xdr:row>73</xdr:row>
+          <xdr:rowOff>22860</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>1440180</xdr:colOff>
+          <xdr:row>74</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1274" name="Drop Down 250" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1274"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000FA040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -12346,7 +12414,7 @@
         <v>115</v>
       </c>
       <c r="C26" s="33"/>
-      <c r="D26" s="77" t="s">
+      <c r="D26" s="159" t="s">
         <v>111</v>
       </c>
       <c r="E26" s="78"/>
@@ -13253,8 +13321,12 @@
       <c r="M73" s="82"/>
     </row>
     <row r="74" spans="1:13" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="32"/>
-      <c r="B74" s="33"/>
+      <c r="A74" s="32">
+        <v>49</v>
+      </c>
+      <c r="B74" s="33" t="s">
+        <v>163</v>
+      </c>
       <c r="C74" s="33"/>
       <c r="D74" s="80"/>
       <c r="E74" s="81"/>
@@ -16610,6 +16682,28 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>1440180</xdr:colOff>
                     <xdr:row>73</xdr:row>
+                    <xdr:rowOff>0</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1274" r:id="rId151" name="Drop Down 250">
+              <controlPr defaultSize="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>30480</xdr:colOff>
+                    <xdr:row>73</xdr:row>
+                    <xdr:rowOff>22860</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>1440180</xdr:colOff>
+                    <xdr:row>74</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
                 </anchor>

</xml_diff>